<commit_message>
feat(reporting): implement KPI governance platform
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -59,7 +59,7 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>18 Jul 2026, 20:30</t>
+    <t>18 Jul 2026, 20:43</t>
   </si>
   <si>
     <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Order Sales  ·  Revenue Trends</t>
@@ -71,7 +71,7 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 20:30</t>
+    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 20:43</t>
   </si>
   <si>
     <t>FINANCIAL PERFORMANCE</t>

</xml_diff>

<commit_message>
feat(reporting): govern KPIs and soft-sunset legacy reporting APIs
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -59,7 +59,7 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>18 Jul 2026, 20:43</t>
+    <t>18 Jul 2026, 20:54</t>
   </si>
   <si>
     <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Order Sales  ·  Revenue Trends</t>
@@ -71,7 +71,7 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 20:43</t>
+    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 20:54</t>
   </si>
   <si>
     <t>FINANCIAL PERFORMANCE</t>

</xml_diff>

<commit_message>
feat(reporting): standardize reporting product semantics
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -8,14 +8,14 @@
     <sheet sheetId="2" name="Executive Summary" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Financial Summary" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Order Sales" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Revenue Trends" state="visible" r:id="rId8"/>
+    <sheet sheetId="5" name="Check Revenue Trends" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="105">
   <si>
     <t>MINEUQR</t>
   </si>
@@ -59,10 +59,10 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>18 Jul 2026, 20:54</t>
-  </si>
-  <si>
-    <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Order Sales  ·  Revenue Trends</t>
+    <t>18 Jul 2026, 21:23</t>
+  </si>
+  <si>
+    <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Order Sales  ·  Check Revenue Trends</t>
   </si>
   <si>
     <t>Confidential — Internal Use  ·  Prepared by MineuQR</t>
@@ -71,13 +71,13 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 20:54</t>
-  </si>
-  <si>
-    <t>FINANCIAL PERFORMANCE</t>
-  </si>
-  <si>
-    <t>Revenue</t>
+    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 21:23</t>
+  </si>
+  <si>
+    <t>CHECK REVENUE PERFORMANCE</t>
+  </si>
+  <si>
+    <t>Check Revenue</t>
   </si>
   <si>
     <t>Tax Collected</t>
@@ -158,12 +158,18 @@
     <t>REPORTING BASIS</t>
   </si>
   <si>
+    <t>Check Revenue = sum of paid Check totals (not Order Sales).</t>
+  </si>
+  <si>
+    <t>Order Sales</t>
+  </si>
+  <si>
+    <t>Order Sales = completed (served) order totals (not Check Revenue).</t>
+  </si>
+  <si>
     <t>SAR (ر.س)</t>
   </si>
   <si>
-    <t>Order Sales</t>
-  </si>
-  <si>
     <t>Monthly Report  ·  Daily Order Sales — July 2026</t>
   </si>
   <si>
@@ -275,13 +281,13 @@
     <t>1,646.00 ر.س</t>
   </si>
   <si>
-    <t>Revenue Trends</t>
-  </si>
-  <si>
-    <t>Monthly Report  ·  Daily Revenue — July 2026</t>
-  </si>
-  <si>
-    <t>REVENUE TREND</t>
+    <t>Check Revenue Trends</t>
+  </si>
+  <si>
+    <t>Monthly Report  ·  Daily Check Revenue — July 2026</t>
+  </si>
+  <si>
+    <t>CHECK REVENUE TREND</t>
   </si>
   <si>
     <t>800.00 ر.س</t>
@@ -1816,7 +1822,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="10.2" customWidth="1"/>
@@ -2184,7 +2190,7 @@
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="22" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B23" s="22"/>
       <c r="C23" s="22"/>
@@ -2204,7 +2210,7 @@
     </row>
     <row r="24" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="24" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="B24" s="24"/>
       <c r="C24" s="24"/>
@@ -2214,7 +2220,7 @@
       <c r="G24" s="24"/>
       <c r="H24" s="24"/>
       <c r="I24" s="25" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="J24" s="25"/>
       <c r="K24" s="25"/>
@@ -2224,7 +2230,7 @@
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="22" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B25" s="22"/>
       <c r="C25" s="22"/>
@@ -2234,7 +2240,7 @@
       <c r="G25" s="22"/>
       <c r="H25" s="22"/>
       <c r="I25" s="23" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="J25" s="23"/>
       <c r="K25" s="23"/>
@@ -2242,8 +2248,48 @@
       <c r="M25" s="23"/>
       <c r="N25" s="23"/>
     </row>
+    <row r="26" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="J26" s="25"/>
+      <c r="K26" s="25"/>
+      <c r="L26" s="25"/>
+      <c r="M26" s="25"/>
+      <c r="N26" s="25"/>
+    </row>
+    <row r="27" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="I27" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="J27" s="23"/>
+      <c r="K27" s="23"/>
+      <c r="L27" s="23"/>
+      <c r="M27" s="23"/>
+      <c r="N27" s="23"/>
+    </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="38">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A5:N5"/>
@@ -2278,6 +2324,10 @@
     <mergeCell ref="I24:N24"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="I25:N25"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="I26:N26"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="I27:N27"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.25" footer="0.3"/>
@@ -2319,7 +2369,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2353,7 +2403,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -2661,12 +2711,12 @@
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="26" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="26"/>
       <c r="D24" s="27" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E24" s="27"/>
       <c r="F24" s="27"/>
@@ -2685,22 +2735,22 @@
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="28" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B25" s="28"/>
       <c r="C25" s="28"/>
       <c r="D25" s="28" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E25" s="28"/>
       <c r="F25" s="28"/>
       <c r="G25" s="28" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H25" s="28"/>
       <c r="I25" s="28"/>
       <c r="J25" s="29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="K25" s="29"/>
       <c r="L25" s="29"/>
@@ -2709,22 +2759,22 @@
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="30" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B26" s="30"/>
       <c r="C26" s="30"/>
       <c r="D26" s="30" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E26" s="30"/>
       <c r="F26" s="30"/>
       <c r="G26" s="30" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H26" s="30"/>
       <c r="I26" s="30"/>
       <c r="J26" s="31" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="K26" s="31"/>
       <c r="L26" s="31"/>
@@ -2733,22 +2783,22 @@
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="28" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B27" s="28"/>
       <c r="C27" s="28"/>
       <c r="D27" s="28" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E27" s="28"/>
       <c r="F27" s="28"/>
       <c r="G27" s="28" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H27" s="28"/>
       <c r="I27" s="28"/>
       <c r="J27" s="29" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="K27" s="29"/>
       <c r="L27" s="29"/>
@@ -2757,22 +2807,22 @@
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="30" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B28" s="30"/>
       <c r="C28" s="30"/>
       <c r="D28" s="30" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E28" s="30"/>
       <c r="F28" s="30"/>
       <c r="G28" s="30" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H28" s="30"/>
       <c r="I28" s="30"/>
       <c r="J28" s="31" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="K28" s="31"/>
       <c r="L28" s="31"/>
@@ -2781,22 +2831,22 @@
     </row>
     <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="28" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B29" s="28"/>
       <c r="C29" s="28"/>
       <c r="D29" s="28" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E29" s="28"/>
       <c r="F29" s="28"/>
       <c r="G29" s="28" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H29" s="28"/>
       <c r="I29" s="28"/>
       <c r="J29" s="29" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K29" s="29"/>
       <c r="L29" s="29"/>
@@ -2805,22 +2855,22 @@
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="30" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B30" s="30"/>
       <c r="C30" s="30"/>
       <c r="D30" s="30" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E30" s="30"/>
       <c r="F30" s="30"/>
       <c r="G30" s="30" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H30" s="30"/>
       <c r="I30" s="30"/>
       <c r="J30" s="31" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="K30" s="31"/>
       <c r="L30" s="31"/>
@@ -2829,22 +2879,22 @@
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="28" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B31" s="28"/>
       <c r="C31" s="28"/>
       <c r="D31" s="28" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E31" s="28"/>
       <c r="F31" s="28"/>
       <c r="G31" s="28" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H31" s="28"/>
       <c r="I31" s="28"/>
       <c r="J31" s="29" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K31" s="29"/>
       <c r="L31" s="29"/>
@@ -2853,22 +2903,22 @@
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="30" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B32" s="30"/>
       <c r="C32" s="30"/>
       <c r="D32" s="30" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E32" s="30"/>
       <c r="F32" s="30"/>
       <c r="G32" s="30" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H32" s="30"/>
       <c r="I32" s="30"/>
       <c r="J32" s="31" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K32" s="31"/>
       <c r="L32" s="31"/>
@@ -2877,22 +2927,22 @@
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="28" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B33" s="28"/>
       <c r="C33" s="28"/>
       <c r="D33" s="28" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E33" s="28"/>
       <c r="F33" s="28"/>
       <c r="G33" s="28" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H33" s="28"/>
       <c r="I33" s="28"/>
       <c r="J33" s="29" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K33" s="29"/>
       <c r="L33" s="29"/>
@@ -2901,22 +2951,22 @@
     </row>
     <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="30" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B34" s="30"/>
       <c r="C34" s="30"/>
       <c r="D34" s="30" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E34" s="30"/>
       <c r="F34" s="30"/>
       <c r="G34" s="30" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H34" s="30"/>
       <c r="I34" s="30"/>
       <c r="J34" s="31" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K34" s="31"/>
       <c r="L34" s="31"/>
@@ -2925,22 +2975,22 @@
     </row>
     <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B35" s="28"/>
       <c r="C35" s="28"/>
       <c r="D35" s="28" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E35" s="28"/>
       <c r="F35" s="28"/>
       <c r="G35" s="28" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H35" s="28"/>
       <c r="I35" s="28"/>
       <c r="J35" s="29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="K35" s="29"/>
       <c r="L35" s="29"/>
@@ -2949,22 +2999,22 @@
     </row>
     <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B36" s="30"/>
       <c r="C36" s="30"/>
       <c r="D36" s="30" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E36" s="30"/>
       <c r="F36" s="30"/>
       <c r="G36" s="30" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H36" s="30"/>
       <c r="I36" s="30"/>
       <c r="J36" s="31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="K36" s="31"/>
       <c r="L36" s="31"/>
@@ -2973,22 +3023,22 @@
     </row>
     <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="28" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B37" s="28"/>
       <c r="C37" s="28"/>
       <c r="D37" s="28" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E37" s="28"/>
       <c r="F37" s="28"/>
       <c r="G37" s="28" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H37" s="28"/>
       <c r="I37" s="28"/>
       <c r="J37" s="29" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="K37" s="29"/>
       <c r="L37" s="29"/>
@@ -2997,22 +3047,22 @@
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="30" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B38" s="30"/>
       <c r="C38" s="30"/>
       <c r="D38" s="30" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E38" s="30"/>
       <c r="F38" s="30"/>
       <c r="G38" s="30" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H38" s="30"/>
       <c r="I38" s="30"/>
       <c r="J38" s="31" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="K38" s="31"/>
       <c r="L38" s="31"/>
@@ -3137,7 +3187,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -3155,7 +3205,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3189,7 +3239,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -3513,7 +3563,7 @@
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="26" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="26"/>
@@ -3535,13 +3585,13 @@
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="28" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B26" s="28"/>
       <c r="C26" s="28"/>
       <c r="D26" s="28"/>
       <c r="E26" s="29" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F26" s="29"/>
       <c r="G26" s="29"/>
@@ -3557,20 +3607,20 @@
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="30" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B27" s="30"/>
       <c r="C27" s="30"/>
       <c r="D27" s="30"/>
       <c r="E27" s="31" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F27" s="31"/>
       <c r="G27" s="31"/>
       <c r="H27" s="31"/>
       <c r="I27" s="31"/>
       <c r="J27" s="30" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K27" s="30"/>
       <c r="L27" s="30"/>
@@ -3579,20 +3629,20 @@
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="28" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B28" s="28"/>
       <c r="C28" s="28"/>
       <c r="D28" s="28"/>
       <c r="E28" s="29" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F28" s="29"/>
       <c r="G28" s="29"/>
       <c r="H28" s="29"/>
       <c r="I28" s="29"/>
       <c r="J28" s="28" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K28" s="28"/>
       <c r="L28" s="28"/>
@@ -3601,20 +3651,20 @@
     </row>
     <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="30" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B29" s="30"/>
       <c r="C29" s="30"/>
       <c r="D29" s="30"/>
       <c r="E29" s="31" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F29" s="31"/>
       <c r="G29" s="31"/>
       <c r="H29" s="31"/>
       <c r="I29" s="31"/>
       <c r="J29" s="30" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="K29" s="30"/>
       <c r="L29" s="30"/>
@@ -3623,20 +3673,20 @@
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="28" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B30" s="28"/>
       <c r="C30" s="28"/>
       <c r="D30" s="28"/>
       <c r="E30" s="29" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F30" s="29"/>
       <c r="G30" s="29"/>
       <c r="H30" s="29"/>
       <c r="I30" s="29"/>
       <c r="J30" s="28" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K30" s="28"/>
       <c r="L30" s="28"/>
@@ -3645,13 +3695,13 @@
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="30" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B31" s="30"/>
       <c r="C31" s="30"/>
       <c r="D31" s="30"/>
       <c r="E31" s="31" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F31" s="31"/>
       <c r="G31" s="31"/>
@@ -3667,20 +3717,20 @@
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="28" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B32" s="28"/>
       <c r="C32" s="28"/>
       <c r="D32" s="28"/>
       <c r="E32" s="29" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F32" s="29"/>
       <c r="G32" s="29"/>
       <c r="H32" s="29"/>
       <c r="I32" s="29"/>
       <c r="J32" s="28" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K32" s="28"/>
       <c r="L32" s="28"/>
@@ -3689,20 +3739,20 @@
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="30" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B33" s="30"/>
       <c r="C33" s="30"/>
       <c r="D33" s="30"/>
       <c r="E33" s="31" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F33" s="31"/>
       <c r="G33" s="31"/>
       <c r="H33" s="31"/>
       <c r="I33" s="31"/>
       <c r="J33" s="30" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K33" s="30"/>
       <c r="L33" s="30"/>
@@ -3711,20 +3761,20 @@
     </row>
     <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="28" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B34" s="28"/>
       <c r="C34" s="28"/>
       <c r="D34" s="28"/>
       <c r="E34" s="29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F34" s="29"/>
       <c r="G34" s="29"/>
       <c r="H34" s="29"/>
       <c r="I34" s="29"/>
       <c r="J34" s="28" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="K34" s="28"/>
       <c r="L34" s="28"/>
@@ -3733,20 +3783,20 @@
     </row>
     <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="30" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B35" s="30"/>
       <c r="C35" s="30"/>
       <c r="D35" s="30"/>
       <c r="E35" s="31" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F35" s="31"/>
       <c r="G35" s="31"/>
       <c r="H35" s="31"/>
       <c r="I35" s="31"/>
       <c r="J35" s="30" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K35" s="30"/>
       <c r="L35" s="30"/>
@@ -3755,13 +3805,13 @@
     </row>
     <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B36" s="28"/>
       <c r="C36" s="28"/>
       <c r="D36" s="28"/>
       <c r="E36" s="29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F36" s="29"/>
       <c r="G36" s="29"/>
@@ -3777,20 +3827,20 @@
     </row>
     <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B37" s="30"/>
       <c r="C37" s="30"/>
       <c r="D37" s="30"/>
       <c r="E37" s="31" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F37" s="31"/>
       <c r="G37" s="31"/>
       <c r="H37" s="31"/>
       <c r="I37" s="31"/>
       <c r="J37" s="30" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K37" s="30"/>
       <c r="L37" s="30"/>
@@ -3799,20 +3849,20 @@
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="28" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B38" s="28"/>
       <c r="C38" s="28"/>
       <c r="D38" s="28"/>
       <c r="E38" s="29" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F38" s="29"/>
       <c r="G38" s="29"/>
       <c r="H38" s="29"/>
       <c r="I38" s="29"/>
       <c r="J38" s="28" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K38" s="28"/>
       <c r="L38" s="28"/>
@@ -3821,20 +3871,20 @@
     </row>
     <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="30" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B39" s="30"/>
       <c r="C39" s="30"/>
       <c r="D39" s="30"/>
       <c r="E39" s="31" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F39" s="31"/>
       <c r="G39" s="31"/>
       <c r="H39" s="31"/>
       <c r="I39" s="31"/>
       <c r="J39" s="30" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="K39" s="30"/>
       <c r="L39" s="30"/>

</xml_diff>

<commit_message>
feat(reporting): rationalize executive summary presentation
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="106">
   <si>
     <t>MINEUQR</t>
   </si>
@@ -35,7 +35,7 @@
     <t>July 2026</t>
   </si>
   <si>
-    <t>Executive Financial Document</t>
+    <t>Business performance overview</t>
   </si>
   <si>
     <t>Currency</t>
@@ -59,7 +59,7 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>18 Jul 2026, 21:23</t>
+    <t>18 Jul 2026, 21:58</t>
   </si>
   <si>
     <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Order Sales  ·  Check Revenue Trends</t>
@@ -71,100 +71,106 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 21:23</t>
-  </si>
-  <si>
-    <t>CHECK REVENUE PERFORMANCE</t>
+    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 21:58</t>
+  </si>
+  <si>
+    <t>AT A GLANCE</t>
+  </si>
+  <si>
+    <t>How the restaurant performed this period — details follow in later sections.</t>
   </si>
   <si>
     <t>Check Revenue</t>
   </si>
   <si>
+    <t>Order Sales</t>
+  </si>
+  <si>
+    <t>Paid Checks</t>
+  </si>
+  <si>
+    <t>14,612.50 ر.س</t>
+  </si>
+  <si>
+    <t>19,222.00 ر.س</t>
+  </si>
+  <si>
+    <t>68</t>
+  </si>
+  <si>
+    <t>Orders</t>
+  </si>
+  <si>
+    <t>Average Check</t>
+  </si>
+  <si>
+    <t>Average Order</t>
+  </si>
+  <si>
+    <t>103</t>
+  </si>
+  <si>
+    <t>214.89 ر.س</t>
+  </si>
+  <si>
+    <t>215.98 ر.س</t>
+  </si>
+  <si>
+    <t>Financial Summary</t>
+  </si>
+  <si>
+    <t>Monthly Report  ·  July 2026</t>
+  </si>
+  <si>
+    <t>CHECK REVENUE DETAIL</t>
+  </si>
+  <si>
+    <t>TAX</t>
+  </si>
+  <si>
     <t>Tax Collected</t>
   </si>
   <si>
-    <t>Paid Checks</t>
-  </si>
-  <si>
-    <t>14,612.50 ر.س</t>
-  </si>
-  <si>
     <t>2,191.91 ر.س</t>
   </si>
   <si>
-    <t>68</t>
-  </si>
-  <si>
-    <t>Average Check</t>
-  </si>
-  <si>
-    <t>Order Sales (Period)</t>
-  </si>
-  <si>
-    <t>Average Order (Period)</t>
-  </si>
-  <si>
-    <t>214.89 ر.س</t>
-  </si>
-  <si>
-    <t>19,222.00 ر.س</t>
-  </si>
-  <si>
-    <t>215.98 ر.س</t>
-  </si>
-  <si>
-    <t>Orders (Period)</t>
+    <t>ORDER SALES DETAIL</t>
+  </si>
+  <si>
+    <t>Completed Orders</t>
+  </si>
+  <si>
+    <t>89</t>
+  </si>
+  <si>
+    <t>ADJUSTMENTS</t>
   </si>
   <si>
     <t>Complimentary Checks</t>
   </si>
   <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Complimentary Amount</t>
+  </si>
+  <si>
+    <t>120.00 ر.س</t>
+  </si>
+  <si>
     <t>Voided Checks</t>
   </si>
   <si>
-    <t>103</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
-    <t>Financial Summary</t>
-  </si>
-  <si>
-    <t>Monthly Report  ·  July 2026</t>
-  </si>
-  <si>
-    <t>ORDER SALES</t>
-  </si>
-  <si>
-    <t>Completed Orders</t>
-  </si>
-  <si>
-    <t>89</t>
-  </si>
-  <si>
-    <t>ADJUSTMENTS</t>
-  </si>
-  <si>
-    <t>Complimentary Amount</t>
-  </si>
-  <si>
-    <t>120.00 ر.س</t>
-  </si>
-  <si>
     <t>REPORTING BASIS</t>
   </si>
   <si>
     <t>Check Revenue = sum of paid Check totals (not Order Sales).</t>
   </si>
   <si>
-    <t>Order Sales</t>
-  </si>
-  <si>
-    <t>Order Sales = completed (served) order totals (not Check Revenue).</t>
+    <t>Order Sales = completed (served) order totals from Order Read (not Check Revenue).</t>
   </si>
   <si>
     <t>SAR (ر.س)</t>
@@ -179,9 +185,6 @@
     <t>Period</t>
   </si>
   <si>
-    <t>Orders</t>
-  </si>
-  <si>
     <t>1 Jul</t>
   </si>
   <si>
@@ -287,7 +290,7 @@
     <t>Monthly Report  ·  Daily Check Revenue — July 2026</t>
   </si>
   <si>
-    <t>CHECK REVENUE TREND</t>
+    <t>CHECK REVENUE TRENDS</t>
   </si>
   <si>
     <t>800.00 ر.س</t>
@@ -543,7 +546,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -592,6 +595,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="13" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1521,7 +1527,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="10.2" customWidth="1"/>
@@ -1613,200 +1619,156 @@
       <c r="M5" s="19"/>
       <c r="N5" s="19"/>
     </row>
-    <row r="7" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="20" t="s">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="F7" s="20" t="s">
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
+      <c r="M6" s="20"/>
+      <c r="N6" s="20"/>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="21" t="s">
         <v>21</v>
-      </c>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20"/>
-      <c r="I7" s="20"/>
-      <c r="K7" s="20" t="s">
-        <v>22</v>
-      </c>
-      <c r="L7" s="20"/>
-      <c r="M7" s="20"/>
-      <c r="N7" s="20"/>
-    </row>
-    <row r="8" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
-        <v>23</v>
       </c>
       <c r="B8" s="21"/>
       <c r="C8" s="21"/>
       <c r="D8" s="21"/>
       <c r="F8" s="21" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G8" s="21"/>
       <c r="H8" s="21"/>
       <c r="I8" s="21"/>
       <c r="K8" s="21" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="L8" s="21"/>
       <c r="M8" s="21"/>
       <c r="N8" s="21"/>
     </row>
-    <row r="9" ht="5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="20" t="s">
+    <row r="9" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="F9" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+      <c r="K9" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="F11" s="20" t="s">
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+    </row>
+    <row r="10" ht="5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="21" t="s">
         <v>27</v>
-      </c>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-      <c r="K11" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="L11" s="20"/>
-      <c r="M11" s="20"/>
-      <c r="N11" s="20"/>
-    </row>
-    <row r="12" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
-        <v>29</v>
       </c>
       <c r="B12" s="21"/>
       <c r="C12" s="21"/>
       <c r="D12" s="21"/>
       <c r="F12" s="21" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G12" s="21"/>
       <c r="H12" s="21"/>
       <c r="I12" s="21"/>
       <c r="K12" s="21" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="L12" s="21"/>
       <c r="M12" s="21"/>
       <c r="N12" s="21"/>
     </row>
-    <row r="13" ht="5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-    </row>
-    <row r="15" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="20" t="s">
+    <row r="13" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="F13" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="22"/>
+      <c r="K13" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="F15" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="K15" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="L15" s="20"/>
-      <c r="M15" s="20"/>
-      <c r="N15" s="20"/>
-    </row>
-    <row r="16" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="F16" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="21"/>
-      <c r="K16" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="L16" s="21"/>
-      <c r="M16" s="21"/>
-      <c r="N16" s="21"/>
-    </row>
-    <row r="17" ht="5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="22"/>
+    </row>
+    <row r="14" ht="5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="N14" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="22">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A5:N5"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="K7:N7"/>
+    <mergeCell ref="A6:N6"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="F8:I8"/>
     <mergeCell ref="K8:N8"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="F9:I9"/>
     <mergeCell ref="K9:N9"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="F11:I11"/>
-    <mergeCell ref="K11:N11"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="K10:N10"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="F12:I12"/>
     <mergeCell ref="K12:N12"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="F13:I13"/>
     <mergeCell ref="K13:N13"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="K15:N15"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="K16:N16"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="K17:N17"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="K14:N14"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.25" footer="0.3"/>
@@ -1822,7 +1784,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="10.2" customWidth="1"/>
@@ -1830,7 +1792,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -1848,7 +1810,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1898,7 +1860,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -1915,381 +1877,399 @@
       <c r="N5" s="19"/>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="22"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="23" t="s">
+      <c r="A6" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="24"/>
+      <c r="M6" s="24"/>
+      <c r="N6" s="24"/>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
-      <c r="N6" s="23"/>
-    </row>
-    <row r="7" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="24" t="s">
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
+      <c r="N7" s="26"/>
+    </row>
+    <row r="8" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="J8" s="24"/>
+      <c r="K8" s="24"/>
+      <c r="L8" s="24"/>
+      <c r="M8" s="24"/>
+      <c r="N8" s="24"/>
+    </row>
+    <row r="10" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+    </row>
+    <row r="11" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="J11" s="24"/>
+      <c r="K11" s="24"/>
+      <c r="L11" s="24"/>
+      <c r="M11" s="24"/>
+      <c r="N11" s="24"/>
+    </row>
+    <row r="13" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="19"/>
+      <c r="N13" s="19"/>
+    </row>
+    <row r="14" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
+      <c r="L14" s="24"/>
+      <c r="M14" s="24"/>
+      <c r="N14" s="24"/>
+    </row>
+    <row r="15" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="J15" s="26"/>
+      <c r="K15" s="26"/>
+      <c r="L15" s="26"/>
+      <c r="M15" s="26"/>
+      <c r="N15" s="26"/>
+    </row>
+    <row r="16" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
+      <c r="L16" s="24"/>
+      <c r="M16" s="24"/>
+      <c r="N16" s="24"/>
+    </row>
+    <row r="17" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="J17" s="26"/>
+      <c r="K17" s="26"/>
+      <c r="L17" s="26"/>
+      <c r="M17" s="26"/>
+      <c r="N17" s="26"/>
+    </row>
+    <row r="19" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="19"/>
+      <c r="N19" s="19"/>
+    </row>
+    <row r="20" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
+      <c r="L20" s="24"/>
+      <c r="M20" s="24"/>
+      <c r="N20" s="24"/>
+    </row>
+    <row r="21" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="25"/>
+      <c r="I21" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="J21" s="26"/>
+      <c r="K21" s="26"/>
+      <c r="L21" s="26"/>
+      <c r="M21" s="26"/>
+      <c r="N21" s="26"/>
+    </row>
+    <row r="22" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23"/>
+      <c r="I22" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="J22" s="24"/>
+      <c r="K22" s="24"/>
+      <c r="L22" s="24"/>
+      <c r="M22" s="24"/>
+      <c r="N22" s="24"/>
+    </row>
+    <row r="24" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19"/>
+      <c r="J24" s="19"/>
+      <c r="K24" s="19"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="19"/>
+      <c r="N24" s="19"/>
+    </row>
+    <row r="25" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="J7" s="25"/>
-      <c r="K7" s="25"/>
-      <c r="L7" s="25"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
-    </row>
-    <row r="8" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="22" t="s">
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="J25" s="24"/>
+      <c r="K25" s="24"/>
+      <c r="L25" s="24"/>
+      <c r="M25" s="24"/>
+      <c r="N25" s="24"/>
+    </row>
+    <row r="26" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="22"/>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
-      <c r="N8" s="23"/>
-    </row>
-    <row r="9" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="J9" s="25"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="25"/>
-      <c r="M9" s="25"/>
-      <c r="N9" s="25"/>
-    </row>
-    <row r="11" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="19"/>
-      <c r="L11" s="19"/>
-      <c r="M11" s="19"/>
-      <c r="N11" s="19"/>
-    </row>
-    <row r="12" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
-      <c r="I12" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="J12" s="23"/>
-      <c r="K12" s="23"/>
-      <c r="L12" s="23"/>
-      <c r="M12" s="23"/>
-      <c r="N12" s="23"/>
-    </row>
-    <row r="13" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="25"/>
-      <c r="M13" s="25"/>
-      <c r="N13" s="25"/>
-    </row>
-    <row r="14" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22"/>
-      <c r="I14" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="23"/>
-      <c r="M14" s="23"/>
-      <c r="N14" s="23"/>
-    </row>
-    <row r="15" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="25"/>
-      <c r="M15" s="25"/>
-      <c r="N15" s="25"/>
-    </row>
-    <row r="17" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="19"/>
-      <c r="K17" s="19"/>
-      <c r="L17" s="19"/>
-      <c r="M17" s="19"/>
-      <c r="N17" s="19"/>
-    </row>
-    <row r="18" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="J18" s="23"/>
-      <c r="K18" s="23"/>
-      <c r="L18" s="23"/>
-      <c r="M18" s="23"/>
-      <c r="N18" s="23"/>
-    </row>
-    <row r="19" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="J19" s="25"/>
-      <c r="K19" s="25"/>
-      <c r="L19" s="25"/>
-      <c r="M19" s="25"/>
-      <c r="N19" s="25"/>
-    </row>
-    <row r="20" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="J20" s="23"/>
-      <c r="K20" s="23"/>
-      <c r="L20" s="23"/>
-      <c r="M20" s="23"/>
-      <c r="N20" s="23"/>
-    </row>
-    <row r="22" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="19"/>
-      <c r="J22" s="19"/>
-      <c r="K22" s="19"/>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19"/>
-      <c r="N22" s="19"/>
-    </row>
-    <row r="23" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="J23" s="23"/>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="23"/>
-      <c r="N23" s="23"/>
-    </row>
-    <row r="24" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="J24" s="25"/>
-      <c r="K24" s="25"/>
-      <c r="L24" s="25"/>
-      <c r="M24" s="25"/>
-      <c r="N24" s="25"/>
-    </row>
-    <row r="25" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="22" t="s">
+      <c r="B26" s="25"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
+      <c r="I26" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="J26" s="26"/>
+      <c r="K26" s="26"/>
+      <c r="L26" s="26"/>
+      <c r="M26" s="26"/>
+      <c r="N26" s="26"/>
+    </row>
+    <row r="27" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="22"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="J25" s="23"/>
-      <c r="K25" s="23"/>
-      <c r="L25" s="23"/>
-      <c r="M25" s="23"/>
-      <c r="N25" s="23"/>
-    </row>
-    <row r="26" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="24" t="s">
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="23"/>
+      <c r="I27" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="J27" s="24"/>
+      <c r="K27" s="24"/>
+      <c r="L27" s="24"/>
+      <c r="M27" s="24"/>
+      <c r="N27" s="24"/>
+    </row>
+    <row r="28" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B26" s="24"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="24"/>
-      <c r="I26" s="25" t="s">
+      <c r="B28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="J26" s="25"/>
-      <c r="K26" s="25"/>
-      <c r="L26" s="25"/>
-      <c r="M26" s="25"/>
-      <c r="N26" s="25"/>
-    </row>
-    <row r="27" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="22" t="s">
+      <c r="J28" s="26"/>
+      <c r="K28" s="26"/>
+      <c r="L28" s="26"/>
+      <c r="M28" s="26"/>
+      <c r="N28" s="26"/>
+    </row>
+    <row r="29" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="23" t="s">
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
+      <c r="I29" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="J27" s="23"/>
-      <c r="K27" s="23"/>
-      <c r="L27" s="23"/>
-      <c r="M27" s="23"/>
-      <c r="N27" s="23"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="24"/>
+      <c r="L29" s="24"/>
+      <c r="M29" s="24"/>
+      <c r="N29" s="24"/>
     </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="39">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A5:N5"/>
@@ -2299,35 +2279,36 @@
     <mergeCell ref="I7:N7"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="I8:N8"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="I9:N9"/>
-    <mergeCell ref="A11:N11"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="I12:N12"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="I13:N13"/>
+    <mergeCell ref="A10:N10"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="I11:N11"/>
+    <mergeCell ref="A13:N13"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="I14:N14"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="I15:N15"/>
-    <mergeCell ref="A17:N17"/>
-    <mergeCell ref="A18:H18"/>
-    <mergeCell ref="I18:N18"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="I19:N19"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="I16:N16"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="I17:N17"/>
+    <mergeCell ref="A19:N19"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="I20:N20"/>
-    <mergeCell ref="A22:N22"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="I23:N23"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="I24:N24"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="I21:N21"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="I22:N22"/>
+    <mergeCell ref="A24:N24"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="I25:N25"/>
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="I26:N26"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="I27:N27"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="I28:N28"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="I29:N29"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.25" footer="0.3"/>
@@ -2351,7 +2332,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -2369,7 +2350,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2403,7 +2384,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -2693,7 +2674,7 @@
     </row>
     <row r="23" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B23" s="19"/>
       <c r="C23" s="19"/>
@@ -2710,388 +2691,388 @@
       <c r="N23" s="19"/>
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" s="26"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27" t="s">
+      <c r="A24" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="H24" s="28"/>
+      <c r="I24" s="28"/>
+      <c r="J24" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="K24" s="28"/>
+      <c r="L24" s="28"/>
+      <c r="M24" s="28"/>
+      <c r="N24" s="28"/>
+    </row>
+    <row r="25" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="H25" s="29"/>
+      <c r="I25" s="29"/>
+      <c r="J25" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="K25" s="30"/>
+      <c r="L25" s="30"/>
+      <c r="M25" s="30"/>
+      <c r="N25" s="30"/>
+    </row>
+    <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="B26" s="31"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="32" t="s">
+        <v>62</v>
+      </c>
+      <c r="K26" s="32"/>
+      <c r="L26" s="32"/>
+      <c r="M26" s="32"/>
+      <c r="N26" s="32"/>
+    </row>
+    <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="H27" s="29"/>
+      <c r="I27" s="29"/>
+      <c r="J27" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="K27" s="30"/>
+      <c r="L27" s="30"/>
+      <c r="M27" s="30"/>
+      <c r="N27" s="30"/>
+    </row>
+    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="H28" s="31"/>
+      <c r="I28" s="31"/>
+      <c r="J28" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="K28" s="32"/>
+      <c r="L28" s="32"/>
+      <c r="M28" s="32"/>
+      <c r="N28" s="32"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="H29" s="29"/>
+      <c r="I29" s="29"/>
+      <c r="J29" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="K29" s="30"/>
+      <c r="L29" s="30"/>
+      <c r="M29" s="30"/>
+      <c r="N29" s="30"/>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="B30" s="31"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="H30" s="31"/>
+      <c r="I30" s="31"/>
+      <c r="J30" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="K30" s="32"/>
+      <c r="L30" s="32"/>
+      <c r="M30" s="32"/>
+      <c r="N30" s="32"/>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="H31" s="29"/>
+      <c r="I31" s="29"/>
+      <c r="J31" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="K31" s="30"/>
+      <c r="L31" s="30"/>
+      <c r="M31" s="30"/>
+      <c r="N31" s="30"/>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B32" s="31"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="E32" s="31"/>
+      <c r="F32" s="31"/>
+      <c r="G32" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="H32" s="31"/>
+      <c r="I32" s="31"/>
+      <c r="J32" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="K32" s="32"/>
+      <c r="L32" s="32"/>
+      <c r="M32" s="32"/>
+      <c r="N32" s="32"/>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="B33" s="29"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="H33" s="29"/>
+      <c r="I33" s="29"/>
+      <c r="J33" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="K33" s="30"/>
+      <c r="L33" s="30"/>
+      <c r="M33" s="30"/>
+      <c r="N33" s="30"/>
+    </row>
+    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" s="31"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="E34" s="31"/>
+      <c r="F34" s="31"/>
+      <c r="G34" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="H34" s="31"/>
+      <c r="I34" s="31"/>
+      <c r="J34" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="K34" s="32"/>
+      <c r="L34" s="32"/>
+      <c r="M34" s="32"/>
+      <c r="N34" s="32"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="B35" s="29"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="E35" s="29"/>
+      <c r="F35" s="29"/>
+      <c r="G35" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="H35" s="29"/>
+      <c r="I35" s="29"/>
+      <c r="J35" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="K35" s="30"/>
+      <c r="L35" s="30"/>
+      <c r="M35" s="30"/>
+      <c r="N35" s="30"/>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="31" t="s">
+        <v>83</v>
+      </c>
+      <c r="B36" s="31"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="E36" s="31"/>
+      <c r="F36" s="31"/>
+      <c r="G36" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="H36" s="31"/>
+      <c r="I36" s="31"/>
+      <c r="J36" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="K36" s="32"/>
+      <c r="L36" s="32"/>
+      <c r="M36" s="32"/>
+      <c r="N36" s="32"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="B37" s="29"/>
+      <c r="C37" s="29"/>
+      <c r="D37" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="E37" s="29"/>
+      <c r="F37" s="29"/>
+      <c r="G37" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="H37" s="29"/>
+      <c r="I37" s="29"/>
+      <c r="J37" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="K37" s="30"/>
+      <c r="L37" s="30"/>
+      <c r="M37" s="30"/>
+      <c r="N37" s="30"/>
+    </row>
+    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="31" t="s">
+        <v>87</v>
+      </c>
+      <c r="B38" s="31"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="E38" s="31"/>
+      <c r="F38" s="31"/>
+      <c r="G38" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="H38" s="31"/>
+      <c r="I38" s="31"/>
+      <c r="J38" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="K38" s="32"/>
+      <c r="L38" s="32"/>
+      <c r="M38" s="32"/>
+      <c r="N38" s="32"/>
+    </row>
+    <row r="39" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="B39" s="33"/>
+      <c r="C39" s="33"/>
+      <c r="D39" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="E39" s="33"/>
+      <c r="F39" s="33"/>
+      <c r="G39" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="H24" s="27"/>
-      <c r="I24" s="27"/>
-      <c r="J24" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="K24" s="27"/>
-      <c r="L24" s="27"/>
-      <c r="M24" s="27"/>
-      <c r="N24" s="27"/>
-    </row>
-    <row r="25" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="28" t="s">
-        <v>55</v>
-      </c>
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="E25" s="28"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="28" t="s">
-        <v>57</v>
-      </c>
-      <c r="H25" s="28"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="K25" s="29"/>
-      <c r="L25" s="29"/>
-      <c r="M25" s="29"/>
-      <c r="N25" s="29"/>
-    </row>
-    <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="B26" s="30"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="E26" s="30"/>
-      <c r="F26" s="30"/>
-      <c r="G26" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="H26" s="30"/>
-      <c r="I26" s="30"/>
-      <c r="J26" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="K26" s="31"/>
-      <c r="L26" s="31"/>
-      <c r="M26" s="31"/>
-      <c r="N26" s="31"/>
-    </row>
-    <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="B27" s="28"/>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="E27" s="28"/>
-      <c r="F27" s="28"/>
-      <c r="G27" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="H27" s="28"/>
-      <c r="I27" s="28"/>
-      <c r="J27" s="29" t="s">
-        <v>64</v>
-      </c>
-      <c r="K27" s="29"/>
-      <c r="L27" s="29"/>
-      <c r="M27" s="29"/>
-      <c r="N27" s="29"/>
-    </row>
-    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="B28" s="30"/>
-      <c r="C28" s="30"/>
-      <c r="D28" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="E28" s="30"/>
-      <c r="F28" s="30"/>
-      <c r="G28" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="H28" s="30"/>
-      <c r="I28" s="30"/>
-      <c r="J28" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="K28" s="31"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="31"/>
-    </row>
-    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="28" t="s">
-        <v>68</v>
-      </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28" t="s">
-        <v>57</v>
-      </c>
-      <c r="H29" s="28"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="K29" s="29"/>
-      <c r="L29" s="29"/>
-      <c r="M29" s="29"/>
-      <c r="N29" s="29"/>
-    </row>
-    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="30" t="s">
-        <v>70</v>
-      </c>
-      <c r="B30" s="30"/>
-      <c r="C30" s="30"/>
-      <c r="D30" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="E30" s="30"/>
-      <c r="F30" s="30"/>
-      <c r="G30" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="H30" s="30"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="31" t="s">
-        <v>71</v>
-      </c>
-      <c r="K30" s="31"/>
-      <c r="L30" s="31"/>
-      <c r="M30" s="31"/>
-      <c r="N30" s="31"/>
-    </row>
-    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
-      <c r="D31" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="H31" s="28"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="K31" s="29"/>
-      <c r="L31" s="29"/>
-      <c r="M31" s="29"/>
-      <c r="N31" s="29"/>
-    </row>
-    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="30" t="s">
-        <v>74</v>
-      </c>
-      <c r="B32" s="30"/>
-      <c r="C32" s="30"/>
-      <c r="D32" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="E32" s="30"/>
-      <c r="F32" s="30"/>
-      <c r="G32" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="H32" s="30"/>
-      <c r="I32" s="30"/>
-      <c r="J32" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="K32" s="31"/>
-      <c r="L32" s="31"/>
-      <c r="M32" s="31"/>
-      <c r="N32" s="31"/>
-    </row>
-    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="B33" s="28"/>
-      <c r="C33" s="28"/>
-      <c r="D33" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="E33" s="28"/>
-      <c r="F33" s="28"/>
-      <c r="G33" s="28" t="s">
-        <v>57</v>
-      </c>
-      <c r="H33" s="28"/>
-      <c r="I33" s="28"/>
-      <c r="J33" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="K33" s="29"/>
-      <c r="L33" s="29"/>
-      <c r="M33" s="29"/>
-      <c r="N33" s="29"/>
-    </row>
-    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="30" t="s">
-        <v>78</v>
-      </c>
-      <c r="B34" s="30"/>
-      <c r="C34" s="30"/>
-      <c r="D34" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="E34" s="30"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="H34" s="30"/>
-      <c r="I34" s="30"/>
-      <c r="J34" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="K34" s="31"/>
-      <c r="L34" s="31"/>
-      <c r="M34" s="31"/>
-      <c r="N34" s="31"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="B35" s="28"/>
-      <c r="C35" s="28"/>
-      <c r="D35" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="E35" s="28"/>
-      <c r="F35" s="28"/>
-      <c r="G35" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="H35" s="28"/>
-      <c r="I35" s="28"/>
-      <c r="J35" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="K35" s="29"/>
-      <c r="L35" s="29"/>
-      <c r="M35" s="29"/>
-      <c r="N35" s="29"/>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="B36" s="30"/>
-      <c r="C36" s="30"/>
-      <c r="D36" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="E36" s="30"/>
-      <c r="F36" s="30"/>
-      <c r="G36" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="H36" s="30"/>
-      <c r="I36" s="30"/>
-      <c r="J36" s="31" t="s">
-        <v>83</v>
-      </c>
-      <c r="K36" s="31"/>
-      <c r="L36" s="31"/>
-      <c r="M36" s="31"/>
-      <c r="N36" s="31"/>
-    </row>
-    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="B37" s="28"/>
-      <c r="C37" s="28"/>
-      <c r="D37" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="E37" s="28"/>
-      <c r="F37" s="28"/>
-      <c r="G37" s="28" t="s">
-        <v>57</v>
-      </c>
-      <c r="H37" s="28"/>
-      <c r="I37" s="28"/>
-      <c r="J37" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="K37" s="29"/>
-      <c r="L37" s="29"/>
-      <c r="M37" s="29"/>
-      <c r="N37" s="29"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="B38" s="30"/>
-      <c r="C38" s="30"/>
-      <c r="D38" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="E38" s="30"/>
-      <c r="F38" s="30"/>
-      <c r="G38" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="H38" s="30"/>
-      <c r="I38" s="30"/>
-      <c r="J38" s="31" t="s">
-        <v>87</v>
-      </c>
-      <c r="K38" s="31"/>
-      <c r="L38" s="31"/>
-      <c r="M38" s="31"/>
-      <c r="N38" s="31"/>
-    </row>
-    <row r="39" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A39" s="32" t="s">
-        <v>5</v>
-      </c>
-      <c r="B39" s="32"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="32" t="s">
-        <v>35</v>
-      </c>
-      <c r="E39" s="32"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="H39" s="32"/>
-      <c r="I39" s="32"/>
-      <c r="J39" s="33" t="s">
-        <v>30</v>
-      </c>
-      <c r="K39" s="33"/>
-      <c r="L39" s="33"/>
-      <c r="M39" s="33"/>
-      <c r="N39" s="33"/>
+      <c r="H39" s="33"/>
+      <c r="I39" s="33"/>
+      <c r="J39" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="K39" s="34"/>
+      <c r="L39" s="34"/>
+      <c r="M39" s="34"/>
+      <c r="N39" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="68">
@@ -3187,7 +3168,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -3205,7 +3186,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3239,7 +3220,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -3545,7 +3526,7 @@
     </row>
     <row r="24" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
@@ -3562,356 +3543,356 @@
       <c r="N24" s="19"/>
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="F25" s="27"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="27"/>
-      <c r="J25" s="27" t="s">
-        <v>22</v>
-      </c>
-      <c r="K25" s="27"/>
-      <c r="L25" s="27"/>
-      <c r="M25" s="27"/>
-      <c r="N25" s="27"/>
+      <c r="A25" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="F25" s="28"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="28"/>
+      <c r="I25" s="28"/>
+      <c r="J25" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="K25" s="28"/>
+      <c r="L25" s="28"/>
+      <c r="M25" s="28"/>
+      <c r="N25" s="28"/>
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="28" t="s">
-        <v>55</v>
-      </c>
-      <c r="B26" s="28"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="29" t="s">
-        <v>91</v>
-      </c>
-      <c r="F26" s="29"/>
-      <c r="G26" s="29"/>
-      <c r="H26" s="29"/>
-      <c r="I26" s="29"/>
-      <c r="J26" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="K26" s="28"/>
-      <c r="L26" s="28"/>
-      <c r="M26" s="28"/>
-      <c r="N26" s="28"/>
+      <c r="A26" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="F26" s="30"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="30"/>
+      <c r="I26" s="30"/>
+      <c r="J26" s="29" t="s">
+        <v>44</v>
+      </c>
+      <c r="K26" s="29"/>
+      <c r="L26" s="29"/>
+      <c r="M26" s="29"/>
+      <c r="N26" s="29"/>
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="30" t="s">
+      <c r="A27" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="31" t="s">
+        <v>94</v>
+      </c>
+      <c r="K27" s="31"/>
+      <c r="L27" s="31"/>
+      <c r="M27" s="31"/>
+      <c r="N27" s="31"/>
+    </row>
+    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="29"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="30"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="K28" s="29"/>
+      <c r="L28" s="29"/>
+      <c r="M28" s="29"/>
+      <c r="N28" s="29"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="K29" s="31"/>
+      <c r="L29" s="31"/>
+      <c r="M29" s="31"/>
+      <c r="N29" s="31"/>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="F30" s="30"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="30"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="K30" s="29"/>
+      <c r="L30" s="29"/>
+      <c r="M30" s="29"/>
+      <c r="N30" s="29"/>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="31"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="31"/>
+      <c r="E31" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="K31" s="31"/>
+      <c r="L31" s="31"/>
+      <c r="M31" s="31"/>
+      <c r="N31" s="31"/>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B32" s="29"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="F32" s="30"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="30"/>
+      <c r="I32" s="30"/>
+      <c r="J32" s="29" t="s">
+        <v>94</v>
+      </c>
+      <c r="K32" s="29"/>
+      <c r="L32" s="29"/>
+      <c r="M32" s="29"/>
+      <c r="N32" s="29"/>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B33" s="31"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="31"/>
+      <c r="E33" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="K33" s="31"/>
+      <c r="L33" s="31"/>
+      <c r="M33" s="31"/>
+      <c r="N33" s="31"/>
+    </row>
+    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" s="29"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="B27" s="30"/>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30"/>
-      <c r="E27" s="31" t="s">
-        <v>92</v>
-      </c>
-      <c r="F27" s="31"/>
-      <c r="G27" s="31"/>
-      <c r="H27" s="31"/>
-      <c r="I27" s="31"/>
-      <c r="J27" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="K27" s="30"/>
-      <c r="L27" s="30"/>
-      <c r="M27" s="30"/>
-      <c r="N27" s="30"/>
-    </row>
-    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="29" t="s">
+      <c r="F34" s="30"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="30"/>
+      <c r="I34" s="30"/>
+      <c r="J34" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="K34" s="29"/>
+      <c r="L34" s="29"/>
+      <c r="M34" s="29"/>
+      <c r="N34" s="29"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="B35" s="31"/>
+      <c r="C35" s="31"/>
+      <c r="D35" s="31"/>
+      <c r="E35" s="32" t="s">
+        <v>101</v>
+      </c>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="32"/>
+      <c r="I35" s="32"/>
+      <c r="J35" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="K35" s="31"/>
+      <c r="L35" s="31"/>
+      <c r="M35" s="31"/>
+      <c r="N35" s="31"/>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="B36" s="29"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="F36" s="30"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="30"/>
+      <c r="I36" s="30"/>
+      <c r="J36" s="29" t="s">
+        <v>44</v>
+      </c>
+      <c r="K36" s="29"/>
+      <c r="L36" s="29"/>
+      <c r="M36" s="29"/>
+      <c r="N36" s="29"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="31" t="s">
+        <v>83</v>
+      </c>
+      <c r="B37" s="31"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
+      <c r="E37" s="32" t="s">
+        <v>103</v>
+      </c>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="F28" s="29"/>
-      <c r="G28" s="29"/>
-      <c r="H28" s="29"/>
-      <c r="I28" s="29"/>
-      <c r="J28" s="28" t="s">
+      <c r="K37" s="31"/>
+      <c r="L37" s="31"/>
+      <c r="M37" s="31"/>
+      <c r="N37" s="31"/>
+    </row>
+    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="F38" s="30"/>
+      <c r="G38" s="30"/>
+      <c r="H38" s="30"/>
+      <c r="I38" s="30"/>
+      <c r="J38" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="K38" s="29"/>
+      <c r="L38" s="29"/>
+      <c r="M38" s="29"/>
+      <c r="N38" s="29"/>
+    </row>
+    <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" s="31" t="s">
+        <v>87</v>
+      </c>
+      <c r="B39" s="31"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="31"/>
+      <c r="E39" s="32" t="s">
+        <v>105</v>
+      </c>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="K28" s="28"/>
-      <c r="L28" s="28"/>
-      <c r="M28" s="28"/>
-      <c r="N28" s="28"/>
-    </row>
-    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="B29" s="30"/>
-      <c r="C29" s="30"/>
-      <c r="D29" s="30"/>
-      <c r="E29" s="31" t="s">
-        <v>95</v>
-      </c>
-      <c r="F29" s="31"/>
-      <c r="G29" s="31"/>
-      <c r="H29" s="31"/>
-      <c r="I29" s="31"/>
-      <c r="J29" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="K29" s="30"/>
-      <c r="L29" s="30"/>
-      <c r="M29" s="30"/>
-      <c r="N29" s="30"/>
-    </row>
-    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="28" t="s">
-        <v>68</v>
-      </c>
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="29" t="s">
-        <v>96</v>
-      </c>
-      <c r="F30" s="29"/>
-      <c r="G30" s="29"/>
-      <c r="H30" s="29"/>
-      <c r="I30" s="29"/>
-      <c r="J30" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="K30" s="28"/>
-      <c r="L30" s="28"/>
-      <c r="M30" s="28"/>
-      <c r="N30" s="28"/>
-    </row>
-    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="30" t="s">
-        <v>70</v>
-      </c>
-      <c r="B31" s="30"/>
-      <c r="C31" s="30"/>
-      <c r="D31" s="30"/>
-      <c r="E31" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="F31" s="31"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="31"/>
-      <c r="I31" s="31"/>
-      <c r="J31" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="K31" s="30"/>
-      <c r="L31" s="30"/>
-      <c r="M31" s="30"/>
-      <c r="N31" s="30"/>
-    </row>
-    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="F32" s="29"/>
-      <c r="G32" s="29"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="29"/>
-      <c r="J32" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
-      <c r="N32" s="28"/>
-    </row>
-    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="30" t="s">
-        <v>74</v>
-      </c>
-      <c r="B33" s="30"/>
-      <c r="C33" s="30"/>
-      <c r="D33" s="30"/>
-      <c r="E33" s="31" t="s">
-        <v>99</v>
-      </c>
-      <c r="F33" s="31"/>
-      <c r="G33" s="31"/>
-      <c r="H33" s="31"/>
-      <c r="I33" s="31"/>
-      <c r="J33" s="30" t="s">
-        <v>57</v>
-      </c>
-      <c r="K33" s="30"/>
-      <c r="L33" s="30"/>
-      <c r="M33" s="30"/>
-      <c r="N33" s="30"/>
-    </row>
-    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="B34" s="28"/>
-      <c r="C34" s="28"/>
-      <c r="D34" s="28"/>
-      <c r="E34" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="F34" s="29"/>
-      <c r="G34" s="29"/>
-      <c r="H34" s="29"/>
-      <c r="I34" s="29"/>
-      <c r="J34" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="K34" s="28"/>
-      <c r="L34" s="28"/>
-      <c r="M34" s="28"/>
-      <c r="N34" s="28"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="30" t="s">
-        <v>78</v>
-      </c>
-      <c r="B35" s="30"/>
-      <c r="C35" s="30"/>
-      <c r="D35" s="30"/>
-      <c r="E35" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="F35" s="31"/>
-      <c r="G35" s="31"/>
-      <c r="H35" s="31"/>
-      <c r="I35" s="31"/>
-      <c r="J35" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="K35" s="30"/>
-      <c r="L35" s="30"/>
-      <c r="M35" s="30"/>
-      <c r="N35" s="30"/>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="B36" s="28"/>
-      <c r="C36" s="28"/>
-      <c r="D36" s="28"/>
-      <c r="E36" s="29" t="s">
-        <v>101</v>
-      </c>
-      <c r="F36" s="29"/>
-      <c r="G36" s="29"/>
-      <c r="H36" s="29"/>
-      <c r="I36" s="29"/>
-      <c r="J36" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="K36" s="28"/>
-      <c r="L36" s="28"/>
-      <c r="M36" s="28"/>
-      <c r="N36" s="28"/>
-    </row>
-    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="B37" s="30"/>
-      <c r="C37" s="30"/>
-      <c r="D37" s="30"/>
-      <c r="E37" s="31" t="s">
-        <v>102</v>
-      </c>
-      <c r="F37" s="31"/>
-      <c r="G37" s="31"/>
-      <c r="H37" s="31"/>
-      <c r="I37" s="31"/>
-      <c r="J37" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="K37" s="30"/>
-      <c r="L37" s="30"/>
-      <c r="M37" s="30"/>
-      <c r="N37" s="30"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="B38" s="28"/>
-      <c r="C38" s="28"/>
-      <c r="D38" s="28"/>
-      <c r="E38" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="F38" s="29"/>
-      <c r="G38" s="29"/>
-      <c r="H38" s="29"/>
-      <c r="I38" s="29"/>
-      <c r="J38" s="28" t="s">
-        <v>57</v>
-      </c>
-      <c r="K38" s="28"/>
-      <c r="L38" s="28"/>
-      <c r="M38" s="28"/>
-      <c r="N38" s="28"/>
-    </row>
-    <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A39" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="B39" s="30"/>
-      <c r="C39" s="30"/>
-      <c r="D39" s="30"/>
-      <c r="E39" s="31" t="s">
-        <v>104</v>
-      </c>
-      <c r="F39" s="31"/>
-      <c r="G39" s="31"/>
-      <c r="H39" s="31"/>
-      <c r="I39" s="31"/>
-      <c r="J39" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="K39" s="30"/>
-      <c r="L39" s="30"/>
-      <c r="M39" s="30"/>
-      <c r="N39" s="30"/>
+      <c r="K39" s="31"/>
+      <c r="L39" s="31"/>
+      <c r="M39" s="31"/>
+      <c r="N39" s="31"/>
     </row>
     <row r="40" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A40" s="32" t="s">
+      <c r="A40" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="B40" s="32"/>
-      <c r="C40" s="32"/>
-      <c r="D40" s="32"/>
-      <c r="E40" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="F40" s="33"/>
-      <c r="G40" s="33"/>
-      <c r="H40" s="33"/>
-      <c r="I40" s="33"/>
-      <c r="J40" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="K40" s="32"/>
-      <c r="L40" s="32"/>
-      <c r="M40" s="32"/>
-      <c r="N40" s="32"/>
+      <c r="B40" s="33"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="33"/>
+      <c r="E40" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="F40" s="34"/>
+      <c r="G40" s="34"/>
+      <c r="H40" s="34"/>
+      <c r="I40" s="34"/>
+      <c r="J40" s="33" t="s">
+        <v>26</v>
+      </c>
+      <c r="K40" s="33"/>
+      <c r="L40" s="33"/>
+      <c r="M40" s="33"/>
+      <c r="N40" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="52">

</xml_diff>

<commit_message>
feat(reporting): improve executive summary user experience
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="117">
   <si>
     <t>MINEUQR</t>
   </si>
@@ -59,7 +59,7 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>18 Jul 2026, 21:58</t>
+    <t>18 Jul 2026, 22:10</t>
   </si>
   <si>
     <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Order Sales  ·  Check Revenue Trends</t>
@@ -71,49 +71,82 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 21:58</t>
+    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 22:10</t>
   </si>
   <si>
     <t>AT A GLANCE</t>
   </si>
   <si>
-    <t>How the restaurant performed this period — details follow in later sections.</t>
+    <t>How did the restaurant perform this period?</t>
+  </si>
+  <si>
+    <t>MONEY COLLECTED</t>
+  </si>
+  <si>
+    <t>From paid guest checks — your Check Revenue story.</t>
   </si>
   <si>
     <t>Check Revenue</t>
   </si>
   <si>
+    <t>Paid Checks</t>
+  </si>
+  <si>
+    <t>Average Check</t>
+  </si>
+  <si>
+    <t>14,612.50 ر.س</t>
+  </si>
+  <si>
+    <t>68</t>
+  </si>
+  <si>
+    <t>214.89 ر.س</t>
+  </si>
+  <si>
+    <t>What guests paid on settled checks</t>
+  </si>
+  <si>
+    <t>How many checks were paid</t>
+  </si>
+  <si>
+    <t>Typical size of a paid check</t>
+  </si>
+  <si>
+    <t>ORDERS SERVED</t>
+  </si>
+  <si>
+    <t>From completed kitchen orders — your Order Sales story.</t>
+  </si>
+  <si>
     <t>Order Sales</t>
   </si>
   <si>
-    <t>Paid Checks</t>
-  </si>
-  <si>
-    <t>14,612.50 ر.س</t>
+    <t>Orders</t>
+  </si>
+  <si>
+    <t>Average Order</t>
   </si>
   <si>
     <t>19,222.00 ر.س</t>
   </si>
   <si>
-    <t>68</t>
-  </si>
-  <si>
-    <t>Orders</t>
-  </si>
-  <si>
-    <t>Average Check</t>
-  </si>
-  <si>
-    <t>Average Order</t>
-  </si>
-  <si>
     <t>103</t>
   </si>
   <si>
-    <t>214.89 ر.س</t>
-  </si>
-  <si>
     <t>215.98 ر.س</t>
+  </si>
+  <si>
+    <t>Value of orders that were completed (served)</t>
+  </si>
+  <si>
+    <t>How many orders were placed</t>
+  </si>
+  <si>
+    <t>Typical size of a completed order</t>
+  </si>
+  <si>
+    <t>These two money totals measure different things and can differ. Check Revenue is money collected on paid checks; Order Sales is the value of completed orders. Average Check uses Check Revenue; Average Order uses Order Sales.</t>
   </si>
   <si>
     <t>Financial Summary</t>
@@ -339,7 +372,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -423,8 +456,24 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF1E293B"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FF0C1222"/>
       <sz val="20"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF94A3B8"/>
+      <sz val="9"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF64748B"/>
+      <sz val="9"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -546,7 +595,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -597,43 +646,52 @@
     <xf numFmtId="49" fontId="13" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="49" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="49" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="19" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="21" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="21" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="20" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="22" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="23" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1527,7 +1585,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="10.2" customWidth="1"/>
@@ -1637,138 +1695,279 @@
       <c r="M6" s="20"/>
       <c r="N6" s="20"/>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
+    <row r="8" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="21"/>
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
-      <c r="F8" s="21" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
-      <c r="I8" s="21"/>
-      <c r="K8" s="21" t="s">
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="21"/>
+      <c r="L9" s="21"/>
+      <c r="M9" s="21"/>
+      <c r="N9" s="21"/>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="L8" s="21"/>
-      <c r="M8" s="21"/>
-      <c r="N8" s="21"/>
-    </row>
-    <row r="9" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="22" t="s">
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="F10" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="22"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="F9" s="22" t="s">
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+      <c r="K10" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="K9" s="22" t="s">
+      <c r="L10" s="22"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+    </row>
+    <row r="11" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="L9" s="22"/>
-      <c r="M9" s="22"/>
-      <c r="N9" s="22"/>
-    </row>
-    <row r="10" ht="5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="F11" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="21"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="F12" s="21" t="s">
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="K11" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
-      <c r="I12" s="21"/>
-      <c r="K12" s="21" t="s">
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
+      <c r="N11" s="23"/>
+    </row>
+    <row r="12" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="L12" s="21"/>
-      <c r="M12" s="21"/>
-      <c r="N12" s="21"/>
-    </row>
-    <row r="13" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="22" t="s">
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="F12" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="22"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="F13" s="22" t="s">
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="K12" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
-      <c r="I13" s="22"/>
-      <c r="K13" s="22" t="s">
+      <c r="L12" s="24"/>
+      <c r="M12" s="24"/>
+      <c r="N12" s="24"/>
+    </row>
+    <row r="13" ht="5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
+    </row>
+    <row r="16" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="L13" s="22"/>
-      <c r="M13" s="22"/>
-      <c r="N13" s="22"/>
-    </row>
-    <row r="14" ht="5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="21"/>
+      <c r="J17" s="21"/>
+      <c r="K17" s="21"/>
+      <c r="L17" s="21"/>
+      <c r="M17" s="21"/>
+      <c r="N17" s="21"/>
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="F18" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="22"/>
+      <c r="K18" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="L18" s="22"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="22"/>
+    </row>
+    <row r="19" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="F19" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="K19" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="L19" s="23"/>
+      <c r="M19" s="23"/>
+      <c r="N19" s="23"/>
+    </row>
+    <row r="20" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="F20" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="24"/>
+      <c r="K20" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="L20" s="24"/>
+      <c r="M20" s="24"/>
+      <c r="N20" s="24"/>
+    </row>
+    <row r="21" ht="5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+    </row>
+    <row r="24" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" s="25"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="25"/>
+      <c r="I24" s="25"/>
+      <c r="J24" s="25"/>
+      <c r="K24" s="25"/>
+      <c r="L24" s="25"/>
+      <c r="M24" s="25"/>
+      <c r="N24" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="33">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A5:N5"/>
     <mergeCell ref="A6:N6"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="A8:N8"/>
+    <mergeCell ref="A9:N9"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="K10:N10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="F11:I11"/>
+    <mergeCell ref="K11:N11"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="F12:I12"/>
     <mergeCell ref="K12:N12"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="F13:I13"/>
     <mergeCell ref="K13:N13"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="K14:N14"/>
+    <mergeCell ref="A16:N16"/>
+    <mergeCell ref="A17:N17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="K18:N18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="K19:N19"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="K20:N20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="K21:N21"/>
+    <mergeCell ref="A24:N24"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.25" footer="0.3"/>
@@ -1792,7 +1991,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -1810,7 +2009,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1860,7 +2059,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -1877,68 +2076,68 @@
       <c r="N5" s="19"/>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="24" t="s">
+      <c r="A6" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="27"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="27"/>
+      <c r="M6" s="27"/>
+      <c r="N6" s="27"/>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="24"/>
-      <c r="K6" s="24"/>
-      <c r="L6" s="24"/>
-      <c r="M6" s="24"/>
-      <c r="N6" s="24"/>
-    </row>
-    <row r="7" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="J7" s="26"/>
-      <c r="K7" s="26"/>
-      <c r="L7" s="26"/>
-      <c r="M7" s="26"/>
-      <c r="N7" s="26"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="29"/>
+      <c r="K7" s="29"/>
+      <c r="L7" s="29"/>
+      <c r="M7" s="29"/>
+      <c r="N7" s="29"/>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="23" t="s">
+      <c r="A8" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="J8" s="24"/>
-      <c r="K8" s="24"/>
-      <c r="L8" s="24"/>
-      <c r="M8" s="24"/>
-      <c r="N8" s="24"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+      <c r="M8" s="27"/>
+      <c r="N8" s="27"/>
     </row>
     <row r="10" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="B10" s="19"/>
       <c r="C10" s="19"/>
@@ -1955,28 +2154,28 @@
       <c r="N10" s="19"/>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="J11" s="24"/>
-      <c r="K11" s="24"/>
-      <c r="L11" s="24"/>
-      <c r="M11" s="24"/>
-      <c r="N11" s="24"/>
+      <c r="A11" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="J11" s="27"/>
+      <c r="K11" s="27"/>
+      <c r="L11" s="27"/>
+      <c r="M11" s="27"/>
+      <c r="N11" s="27"/>
     </row>
     <row r="13" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="B13" s="19"/>
       <c r="C13" s="19"/>
@@ -1993,88 +2192,88 @@
       <c r="N13" s="19"/>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="J14" s="24"/>
-      <c r="K14" s="24"/>
-      <c r="L14" s="24"/>
-      <c r="M14" s="24"/>
-      <c r="N14" s="24"/>
+      <c r="A14" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="J14" s="27"/>
+      <c r="K14" s="27"/>
+      <c r="L14" s="27"/>
+      <c r="M14" s="27"/>
+      <c r="N14" s="27"/>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="J15" s="26"/>
-      <c r="K15" s="26"/>
-      <c r="L15" s="26"/>
-      <c r="M15" s="26"/>
-      <c r="N15" s="26"/>
+      <c r="A15" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="J15" s="29"/>
+      <c r="K15" s="29"/>
+      <c r="L15" s="29"/>
+      <c r="M15" s="29"/>
+      <c r="N15" s="29"/>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="J16" s="24"/>
-      <c r="K16" s="24"/>
-      <c r="L16" s="24"/>
-      <c r="M16" s="24"/>
-      <c r="N16" s="24"/>
+      <c r="A16" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="J16" s="27"/>
+      <c r="K16" s="27"/>
+      <c r="L16" s="27"/>
+      <c r="M16" s="27"/>
+      <c r="N16" s="27"/>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="J17" s="26"/>
-      <c r="K17" s="26"/>
-      <c r="L17" s="26"/>
-      <c r="M17" s="26"/>
-      <c r="N17" s="26"/>
+      <c r="A17" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="J17" s="29"/>
+      <c r="K17" s="29"/>
+      <c r="L17" s="29"/>
+      <c r="M17" s="29"/>
+      <c r="N17" s="29"/>
     </row>
     <row r="19" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="B19" s="19"/>
       <c r="C19" s="19"/>
@@ -2091,68 +2290,68 @@
       <c r="N19" s="19"/>
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="J20" s="24"/>
-      <c r="K20" s="24"/>
-      <c r="L20" s="24"/>
-      <c r="M20" s="24"/>
-      <c r="N20" s="24"/>
+      <c r="A20" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="J20" s="27"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="27"/>
+      <c r="M20" s="27"/>
+      <c r="N20" s="27"/>
     </row>
     <row r="21" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="J21" s="26"/>
-      <c r="K21" s="26"/>
-      <c r="L21" s="26"/>
-      <c r="M21" s="26"/>
-      <c r="N21" s="26"/>
+      <c r="A21" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="28"/>
+      <c r="H21" s="28"/>
+      <c r="I21" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="J21" s="29"/>
+      <c r="K21" s="29"/>
+      <c r="L21" s="29"/>
+      <c r="M21" s="29"/>
+      <c r="N21" s="29"/>
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="23"/>
-      <c r="G22" s="23"/>
-      <c r="H22" s="23"/>
-      <c r="I22" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="J22" s="24"/>
-      <c r="K22" s="24"/>
-      <c r="L22" s="24"/>
-      <c r="M22" s="24"/>
-      <c r="N22" s="24"/>
+      <c r="A22" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="26"/>
+      <c r="I22" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
+      <c r="L22" s="27"/>
+      <c r="M22" s="27"/>
+      <c r="N22" s="27"/>
     </row>
     <row r="24" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
@@ -2169,104 +2368,104 @@
       <c r="N24" s="19"/>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="J25" s="24"/>
-      <c r="K25" s="24"/>
-      <c r="L25" s="24"/>
-      <c r="M25" s="24"/>
-      <c r="N25" s="24"/>
+      <c r="A25" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="26"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="26"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="26"/>
+      <c r="I25" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="J25" s="27"/>
+      <c r="K25" s="27"/>
+      <c r="L25" s="27"/>
+      <c r="M25" s="27"/>
+      <c r="N25" s="27"/>
     </row>
     <row r="26" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="B26" s="25"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="25"/>
-      <c r="I26" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="J26" s="26"/>
-      <c r="K26" s="26"/>
-      <c r="L26" s="26"/>
-      <c r="M26" s="26"/>
-      <c r="N26" s="26"/>
+      <c r="A26" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="28"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="28"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="28"/>
+      <c r="H26" s="28"/>
+      <c r="I26" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="J26" s="29"/>
+      <c r="K26" s="29"/>
+      <c r="L26" s="29"/>
+      <c r="M26" s="29"/>
+      <c r="N26" s="29"/>
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="23" t="s">
+      <c r="A27" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
-      <c r="H27" s="23"/>
-      <c r="I27" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="J27" s="24"/>
-      <c r="K27" s="24"/>
-      <c r="L27" s="24"/>
-      <c r="M27" s="24"/>
-      <c r="N27" s="24"/>
+      <c r="B27" s="26"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="J27" s="27"/>
+      <c r="K27" s="27"/>
+      <c r="L27" s="27"/>
+      <c r="M27" s="27"/>
+      <c r="N27" s="27"/>
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="25"/>
-      <c r="I28" s="26" t="s">
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="J28" s="26"/>
-      <c r="K28" s="26"/>
-      <c r="L28" s="26"/>
-      <c r="M28" s="26"/>
-      <c r="N28" s="26"/>
+      <c r="J28" s="29"/>
+      <c r="K28" s="29"/>
+      <c r="L28" s="29"/>
+      <c r="M28" s="29"/>
+      <c r="N28" s="29"/>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="23" t="s">
+      <c r="A29" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="B29" s="23"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="24" t="s">
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="26"/>
+      <c r="I29" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="J29" s="24"/>
-      <c r="K29" s="24"/>
-      <c r="L29" s="24"/>
-      <c r="M29" s="24"/>
-      <c r="N29" s="24"/>
+      <c r="J29" s="27"/>
+      <c r="K29" s="27"/>
+      <c r="L29" s="27"/>
+      <c r="M29" s="27"/>
+      <c r="N29" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="39">
@@ -2332,7 +2531,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -2350,7 +2549,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2384,7 +2583,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -2674,7 +2873,7 @@
     </row>
     <row r="23" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="B23" s="19"/>
       <c r="C23" s="19"/>
@@ -2691,388 +2890,388 @@
       <c r="N23" s="19"/>
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="27" t="s">
-        <v>55</v>
-      </c>
-      <c r="B24" s="27"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="H24" s="28"/>
-      <c r="I24" s="28"/>
-      <c r="J24" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="K24" s="28"/>
-      <c r="L24" s="28"/>
-      <c r="M24" s="28"/>
-      <c r="N24" s="28"/>
+      <c r="A24" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="31" t="s">
+        <v>51</v>
+      </c>
+      <c r="H24" s="31"/>
+      <c r="I24" s="31"/>
+      <c r="J24" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="K24" s="31"/>
+      <c r="L24" s="31"/>
+      <c r="M24" s="31"/>
+      <c r="N24" s="31"/>
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="B25" s="29"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="E25" s="29"/>
-      <c r="F25" s="29"/>
-      <c r="G25" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="H25" s="29"/>
-      <c r="I25" s="29"/>
-      <c r="J25" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="K25" s="30"/>
-      <c r="L25" s="30"/>
-      <c r="M25" s="30"/>
-      <c r="N25" s="30"/>
+      <c r="A25" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="33" t="s">
+        <v>70</v>
+      </c>
+      <c r="K25" s="33"/>
+      <c r="L25" s="33"/>
+      <c r="M25" s="33"/>
+      <c r="N25" s="33"/>
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="31" t="s">
-        <v>60</v>
-      </c>
-      <c r="B26" s="31"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="31" t="s">
-        <v>57</v>
-      </c>
-      <c r="H26" s="31"/>
-      <c r="I26" s="31"/>
-      <c r="J26" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="K26" s="32"/>
-      <c r="L26" s="32"/>
-      <c r="M26" s="32"/>
-      <c r="N26" s="32"/>
+      <c r="A26" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="B26" s="34"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="H26" s="34"/>
+      <c r="I26" s="34"/>
+      <c r="J26" s="35" t="s">
+        <v>73</v>
+      </c>
+      <c r="K26" s="35"/>
+      <c r="L26" s="35"/>
+      <c r="M26" s="35"/>
+      <c r="N26" s="35"/>
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29" t="s">
-        <v>64</v>
-      </c>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="H27" s="29"/>
-      <c r="I27" s="29"/>
-      <c r="J27" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="K27" s="30"/>
-      <c r="L27" s="30"/>
-      <c r="M27" s="30"/>
-      <c r="N27" s="30"/>
+      <c r="A27" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="B27" s="32"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="K27" s="33"/>
+      <c r="L27" s="33"/>
+      <c r="M27" s="33"/>
+      <c r="N27" s="33"/>
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="B28" s="31"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="H28" s="31"/>
-      <c r="I28" s="31"/>
-      <c r="J28" s="32" t="s">
+      <c r="A28" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B28" s="34"/>
+      <c r="C28" s="34"/>
+      <c r="D28" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
+      <c r="G28" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="H28" s="34"/>
+      <c r="I28" s="34"/>
+      <c r="J28" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="K28" s="35"/>
+      <c r="L28" s="35"/>
+      <c r="M28" s="35"/>
+      <c r="N28" s="35"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29" s="32"/>
+      <c r="C29" s="32"/>
+      <c r="D29" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="K28" s="32"/>
-      <c r="L28" s="32"/>
-      <c r="M28" s="32"/>
-      <c r="N28" s="32"/>
-    </row>
-    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="29" t="s">
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
-      <c r="G29" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="H29" s="29"/>
-      <c r="I29" s="29"/>
-      <c r="J29" s="30" t="s">
-        <v>70</v>
-      </c>
-      <c r="K29" s="30"/>
-      <c r="L29" s="30"/>
-      <c r="M29" s="30"/>
-      <c r="N29" s="30"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="K29" s="33"/>
+      <c r="L29" s="33"/>
+      <c r="M29" s="33"/>
+      <c r="N29" s="33"/>
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="31" t="s">
-        <v>71</v>
-      </c>
-      <c r="B30" s="31"/>
-      <c r="C30" s="31"/>
-      <c r="D30" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="E30" s="31"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="31" t="s">
-        <v>57</v>
-      </c>
-      <c r="H30" s="31"/>
-      <c r="I30" s="31"/>
-      <c r="J30" s="32" t="s">
+      <c r="A30" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="B30" s="34"/>
+      <c r="C30" s="34"/>
+      <c r="D30" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="K30" s="32"/>
-      <c r="L30" s="32"/>
-      <c r="M30" s="32"/>
-      <c r="N30" s="32"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="H30" s="34"/>
+      <c r="I30" s="34"/>
+      <c r="J30" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="K30" s="35"/>
+      <c r="L30" s="35"/>
+      <c r="M30" s="35"/>
+      <c r="N30" s="35"/>
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="B31" s="29"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29" t="s">
-        <v>64</v>
-      </c>
-      <c r="E31" s="29"/>
-      <c r="F31" s="29"/>
-      <c r="G31" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="H31" s="29"/>
-      <c r="I31" s="29"/>
-      <c r="J31" s="30" t="s">
-        <v>74</v>
-      </c>
-      <c r="K31" s="30"/>
-      <c r="L31" s="30"/>
-      <c r="M31" s="30"/>
-      <c r="N31" s="30"/>
+      <c r="A31" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="B31" s="32"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="K31" s="33"/>
+      <c r="L31" s="33"/>
+      <c r="M31" s="33"/>
+      <c r="N31" s="33"/>
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="31" t="s">
+      <c r="A32" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="B32" s="34"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="E32" s="34"/>
+      <c r="F32" s="34"/>
+      <c r="G32" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="B32" s="31"/>
-      <c r="C32" s="31"/>
-      <c r="D32" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="E32" s="31"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="H32" s="31"/>
-      <c r="I32" s="31"/>
-      <c r="J32" s="32" t="s">
-        <v>76</v>
-      </c>
-      <c r="K32" s="32"/>
-      <c r="L32" s="32"/>
-      <c r="M32" s="32"/>
-      <c r="N32" s="32"/>
+      <c r="H32" s="34"/>
+      <c r="I32" s="34"/>
+      <c r="J32" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="K32" s="35"/>
+      <c r="L32" s="35"/>
+      <c r="M32" s="35"/>
+      <c r="N32" s="35"/>
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="B33" s="29"/>
-      <c r="C33" s="29"/>
-      <c r="D33" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="E33" s="29"/>
-      <c r="F33" s="29"/>
-      <c r="G33" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="H33" s="29"/>
-      <c r="I33" s="29"/>
-      <c r="J33" s="30" t="s">
+      <c r="A33" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="B33" s="32"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="K33" s="33"/>
+      <c r="L33" s="33"/>
+      <c r="M33" s="33"/>
+      <c r="N33" s="33"/>
+    </row>
+    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="B34" s="34"/>
+      <c r="C34" s="34"/>
+      <c r="D34" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="E34" s="34"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="H34" s="34"/>
+      <c r="I34" s="34"/>
+      <c r="J34" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="K34" s="35"/>
+      <c r="L34" s="35"/>
+      <c r="M34" s="35"/>
+      <c r="N34" s="35"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="B35" s="32"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="H35" s="32"/>
+      <c r="I35" s="32"/>
+      <c r="J35" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="K35" s="33"/>
+      <c r="L35" s="33"/>
+      <c r="M35" s="33"/>
+      <c r="N35" s="33"/>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="B36" s="34"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="K33" s="30"/>
-      <c r="L33" s="30"/>
-      <c r="M33" s="30"/>
-      <c r="N33" s="30"/>
-    </row>
-    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="B34" s="31"/>
-      <c r="C34" s="31"/>
-      <c r="D34" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="E34" s="31"/>
-      <c r="F34" s="31"/>
-      <c r="G34" s="31" t="s">
-        <v>57</v>
-      </c>
-      <c r="H34" s="31"/>
-      <c r="I34" s="31"/>
-      <c r="J34" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="K34" s="32"/>
-      <c r="L34" s="32"/>
-      <c r="M34" s="32"/>
-      <c r="N34" s="32"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="B35" s="29"/>
-      <c r="C35" s="29"/>
-      <c r="D35" s="29" t="s">
-        <v>64</v>
-      </c>
-      <c r="E35" s="29"/>
-      <c r="F35" s="29"/>
-      <c r="G35" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="H35" s="29"/>
-      <c r="I35" s="29"/>
-      <c r="J35" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="K35" s="30"/>
-      <c r="L35" s="30"/>
-      <c r="M35" s="30"/>
-      <c r="N35" s="30"/>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" s="31" t="s">
-        <v>83</v>
-      </c>
-      <c r="B36" s="31"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="H36" s="31"/>
-      <c r="I36" s="31"/>
-      <c r="J36" s="32" t="s">
-        <v>84</v>
-      </c>
-      <c r="K36" s="32"/>
-      <c r="L36" s="32"/>
-      <c r="M36" s="32"/>
-      <c r="N36" s="32"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="H36" s="34"/>
+      <c r="I36" s="34"/>
+      <c r="J36" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="K36" s="35"/>
+      <c r="L36" s="35"/>
+      <c r="M36" s="35"/>
+      <c r="N36" s="35"/>
     </row>
     <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="B37" s="29"/>
-      <c r="C37" s="29"/>
-      <c r="D37" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="E37" s="29"/>
-      <c r="F37" s="29"/>
-      <c r="G37" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="H37" s="29"/>
-      <c r="I37" s="29"/>
-      <c r="J37" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="K37" s="30"/>
-      <c r="L37" s="30"/>
-      <c r="M37" s="30"/>
-      <c r="N37" s="30"/>
+      <c r="A37" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="B37" s="32"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="H37" s="32"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="K37" s="33"/>
+      <c r="L37" s="33"/>
+      <c r="M37" s="33"/>
+      <c r="N37" s="33"/>
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="31" t="s">
-        <v>87</v>
-      </c>
-      <c r="B38" s="31"/>
-      <c r="C38" s="31"/>
-      <c r="D38" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="E38" s="31"/>
-      <c r="F38" s="31"/>
-      <c r="G38" s="31" t="s">
-        <v>57</v>
-      </c>
-      <c r="H38" s="31"/>
-      <c r="I38" s="31"/>
-      <c r="J38" s="32" t="s">
-        <v>88</v>
-      </c>
-      <c r="K38" s="32"/>
-      <c r="L38" s="32"/>
-      <c r="M38" s="32"/>
-      <c r="N38" s="32"/>
+      <c r="A38" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="B38" s="34"/>
+      <c r="C38" s="34"/>
+      <c r="D38" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="E38" s="34"/>
+      <c r="F38" s="34"/>
+      <c r="G38" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="H38" s="34"/>
+      <c r="I38" s="34"/>
+      <c r="J38" s="35" t="s">
+        <v>99</v>
+      </c>
+      <c r="K38" s="35"/>
+      <c r="L38" s="35"/>
+      <c r="M38" s="35"/>
+      <c r="N38" s="35"/>
     </row>
     <row r="39" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A39" s="33" t="s">
+      <c r="A39" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="B39" s="33"/>
-      <c r="C39" s="33"/>
-      <c r="D39" s="33" t="s">
-        <v>30</v>
-      </c>
-      <c r="E39" s="33"/>
-      <c r="F39" s="33"/>
-      <c r="G39" s="33" t="s">
-        <v>41</v>
-      </c>
-      <c r="H39" s="33"/>
-      <c r="I39" s="33"/>
-      <c r="J39" s="34" t="s">
-        <v>25</v>
-      </c>
-      <c r="K39" s="34"/>
-      <c r="L39" s="34"/>
-      <c r="M39" s="34"/>
-      <c r="N39" s="34"/>
+      <c r="B39" s="36"/>
+      <c r="C39" s="36"/>
+      <c r="D39" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="E39" s="36"/>
+      <c r="F39" s="36"/>
+      <c r="G39" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="H39" s="36"/>
+      <c r="I39" s="36"/>
+      <c r="J39" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="K39" s="37"/>
+      <c r="L39" s="37"/>
+      <c r="M39" s="37"/>
+      <c r="N39" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="68">
@@ -3168,7 +3367,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -3186,7 +3385,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3220,7 +3419,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -3526,7 +3725,7 @@
     </row>
     <row r="24" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
@@ -3543,356 +3742,356 @@
       <c r="N24" s="19"/>
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="27" t="s">
+      <c r="A25" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="B25" s="30"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" s="31"/>
+      <c r="G25" s="31"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="31"/>
+      <c r="J25" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="K25" s="31"/>
+      <c r="L25" s="31"/>
+      <c r="M25" s="31"/>
+      <c r="N25" s="31"/>
+    </row>
+    <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="33" t="s">
+        <v>103</v>
+      </c>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="33"/>
+      <c r="J26" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="B25" s="27"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="28" t="s">
-        <v>21</v>
-      </c>
-      <c r="F25" s="28"/>
-      <c r="G25" s="28"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="K25" s="28"/>
-      <c r="L25" s="28"/>
-      <c r="M25" s="28"/>
-      <c r="N25" s="28"/>
-    </row>
-    <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="B26" s="29"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="30" t="s">
+      <c r="K26" s="32"/>
+      <c r="L26" s="32"/>
+      <c r="M26" s="32"/>
+      <c r="N26" s="32"/>
+    </row>
+    <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35"/>
+      <c r="H27" s="35"/>
+      <c r="I27" s="35"/>
+      <c r="J27" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
+      <c r="M27" s="34"/>
+      <c r="N27" s="34"/>
+    </row>
+    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="B28" s="32"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="33" t="s">
+        <v>106</v>
+      </c>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="33"/>
+      <c r="J28" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="K28" s="32"/>
+      <c r="L28" s="32"/>
+      <c r="M28" s="32"/>
+      <c r="N28" s="32"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B29" s="34"/>
+      <c r="C29" s="34"/>
+      <c r="D29" s="34"/>
+      <c r="E29" s="35" t="s">
+        <v>107</v>
+      </c>
+      <c r="F29" s="35"/>
+      <c r="G29" s="35"/>
+      <c r="H29" s="35"/>
+      <c r="I29" s="35"/>
+      <c r="J29" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
+      <c r="M29" s="34"/>
+      <c r="N29" s="34"/>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="B30" s="32"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="33"/>
+      <c r="J30" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="K30" s="32"/>
+      <c r="L30" s="32"/>
+      <c r="M30" s="32"/>
+      <c r="N30" s="32"/>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="B31" s="34"/>
+      <c r="C31" s="34"/>
+      <c r="D31" s="34"/>
+      <c r="E31" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F31" s="35"/>
+      <c r="G31" s="35"/>
+      <c r="H31" s="35"/>
+      <c r="I31" s="35"/>
+      <c r="J31" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="K31" s="34"/>
+      <c r="L31" s="34"/>
+      <c r="M31" s="34"/>
+      <c r="N31" s="34"/>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="B32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="33" t="s">
+        <v>110</v>
+      </c>
+      <c r="F32" s="33"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="33"/>
+      <c r="I32" s="33"/>
+      <c r="J32" s="32" t="s">
+        <v>105</v>
+      </c>
+      <c r="K32" s="32"/>
+      <c r="L32" s="32"/>
+      <c r="M32" s="32"/>
+      <c r="N32" s="32"/>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="B33" s="34"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="35" t="s">
+        <v>111</v>
+      </c>
+      <c r="F33" s="35"/>
+      <c r="G33" s="35"/>
+      <c r="H33" s="35"/>
+      <c r="I33" s="35"/>
+      <c r="J33" s="34" t="s">
+        <v>69</v>
+      </c>
+      <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
+      <c r="M33" s="34"/>
+      <c r="N33" s="34"/>
+    </row>
+    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="B34" s="32"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="33" t="s">
+        <v>70</v>
+      </c>
+      <c r="F34" s="33"/>
+      <c r="G34" s="33"/>
+      <c r="H34" s="33"/>
+      <c r="I34" s="33"/>
+      <c r="J34" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="K34" s="32"/>
+      <c r="L34" s="32"/>
+      <c r="M34" s="32"/>
+      <c r="N34" s="32"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="B35" s="34"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="34"/>
+      <c r="E35" s="35" t="s">
+        <v>112</v>
+      </c>
+      <c r="F35" s="35"/>
+      <c r="G35" s="35"/>
+      <c r="H35" s="35"/>
+      <c r="I35" s="35"/>
+      <c r="J35" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="K35" s="34"/>
+      <c r="L35" s="34"/>
+      <c r="M35" s="34"/>
+      <c r="N35" s="34"/>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="F26" s="30"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="30"/>
-      <c r="J26" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="K26" s="29"/>
-      <c r="L26" s="29"/>
-      <c r="M26" s="29"/>
-      <c r="N26" s="29"/>
-    </row>
-    <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="31" t="s">
-        <v>60</v>
-      </c>
-      <c r="B27" s="31"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="32" t="s">
-        <v>93</v>
-      </c>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="32"/>
-      <c r="I27" s="32"/>
-      <c r="J27" s="31" t="s">
+      <c r="B36" s="32"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="F36" s="33"/>
+      <c r="G36" s="33"/>
+      <c r="H36" s="33"/>
+      <c r="I36" s="33"/>
+      <c r="J36" s="32" t="s">
+        <v>55</v>
+      </c>
+      <c r="K36" s="32"/>
+      <c r="L36" s="32"/>
+      <c r="M36" s="32"/>
+      <c r="N36" s="32"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="K27" s="31"/>
-      <c r="L27" s="31"/>
-      <c r="M27" s="31"/>
-      <c r="N27" s="31"/>
-    </row>
-    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="B28" s="29"/>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="F28" s="30"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="30"/>
-      <c r="I28" s="30"/>
-      <c r="J28" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="K28" s="29"/>
-      <c r="L28" s="29"/>
-      <c r="M28" s="29"/>
-      <c r="N28" s="29"/>
-    </row>
-    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="B29" s="31"/>
-      <c r="C29" s="31"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="32" t="s">
+      <c r="B37" s="34"/>
+      <c r="C37" s="34"/>
+      <c r="D37" s="34"/>
+      <c r="E37" s="35" t="s">
+        <v>114</v>
+      </c>
+      <c r="F37" s="35"/>
+      <c r="G37" s="35"/>
+      <c r="H37" s="35"/>
+      <c r="I37" s="35"/>
+      <c r="J37" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="K37" s="34"/>
+      <c r="L37" s="34"/>
+      <c r="M37" s="34"/>
+      <c r="N37" s="34"/>
+    </row>
+    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="32" t="s">
         <v>96</v>
       </c>
-      <c r="F29" s="32"/>
-      <c r="G29" s="32"/>
-      <c r="H29" s="32"/>
-      <c r="I29" s="32"/>
-      <c r="J29" s="31" t="s">
-        <v>57</v>
-      </c>
-      <c r="K29" s="31"/>
-      <c r="L29" s="31"/>
-      <c r="M29" s="31"/>
-      <c r="N29" s="31"/>
-    </row>
-    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="29" t="s">
+      <c r="B38" s="32"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="F38" s="33"/>
+      <c r="G38" s="33"/>
+      <c r="H38" s="33"/>
+      <c r="I38" s="33"/>
+      <c r="J38" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="B30" s="29"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="30" t="s">
-        <v>97</v>
-      </c>
-      <c r="F30" s="30"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="30"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="K30" s="29"/>
-      <c r="L30" s="29"/>
-      <c r="M30" s="29"/>
-      <c r="N30" s="29"/>
-    </row>
-    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="31" t="s">
-        <v>71</v>
-      </c>
-      <c r="B31" s="31"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="32" t="s">
+      <c r="K38" s="32"/>
+      <c r="L38" s="32"/>
+      <c r="M38" s="32"/>
+      <c r="N38" s="32"/>
+    </row>
+    <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="F31" s="32"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="32"/>
-      <c r="I31" s="32"/>
-      <c r="J31" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="K31" s="31"/>
-      <c r="L31" s="31"/>
-      <c r="M31" s="31"/>
-      <c r="N31" s="31"/>
-    </row>
-    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="B32" s="29"/>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="30" t="s">
-        <v>99</v>
-      </c>
-      <c r="F32" s="30"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="30"/>
-      <c r="I32" s="30"/>
-      <c r="J32" s="29" t="s">
-        <v>94</v>
-      </c>
-      <c r="K32" s="29"/>
-      <c r="L32" s="29"/>
-      <c r="M32" s="29"/>
-      <c r="N32" s="29"/>
-    </row>
-    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="B33" s="31"/>
-      <c r="C33" s="31"/>
-      <c r="D33" s="31"/>
-      <c r="E33" s="32" t="s">
-        <v>100</v>
-      </c>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="32"/>
-      <c r="I33" s="32"/>
-      <c r="J33" s="31" t="s">
-        <v>58</v>
-      </c>
-      <c r="K33" s="31"/>
-      <c r="L33" s="31"/>
-      <c r="M33" s="31"/>
-      <c r="N33" s="31"/>
-    </row>
-    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="B34" s="29"/>
-      <c r="C34" s="29"/>
-      <c r="D34" s="29"/>
-      <c r="E34" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="F34" s="30"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="30"/>
-      <c r="I34" s="30"/>
-      <c r="J34" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="K34" s="29"/>
-      <c r="L34" s="29"/>
-      <c r="M34" s="29"/>
-      <c r="N34" s="29"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="B35" s="31"/>
-      <c r="C35" s="31"/>
-      <c r="D35" s="31"/>
-      <c r="E35" s="32" t="s">
-        <v>101</v>
-      </c>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
-      <c r="H35" s="32"/>
-      <c r="I35" s="32"/>
-      <c r="J35" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="K35" s="31"/>
-      <c r="L35" s="31"/>
-      <c r="M35" s="31"/>
-      <c r="N35" s="31"/>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="B36" s="29"/>
-      <c r="C36" s="29"/>
-      <c r="D36" s="29"/>
-      <c r="E36" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="F36" s="30"/>
-      <c r="G36" s="30"/>
-      <c r="H36" s="30"/>
-      <c r="I36" s="30"/>
-      <c r="J36" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="K36" s="29"/>
-      <c r="L36" s="29"/>
-      <c r="M36" s="29"/>
-      <c r="N36" s="29"/>
-    </row>
-    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="31" t="s">
-        <v>83</v>
-      </c>
-      <c r="B37" s="31"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="31"/>
-      <c r="E37" s="32" t="s">
-        <v>103</v>
-      </c>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
-      <c r="H37" s="32"/>
-      <c r="I37" s="32"/>
-      <c r="J37" s="31" t="s">
-        <v>94</v>
-      </c>
-      <c r="K37" s="31"/>
-      <c r="L37" s="31"/>
-      <c r="M37" s="31"/>
-      <c r="N37" s="31"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="B38" s="29"/>
-      <c r="C38" s="29"/>
-      <c r="D38" s="29"/>
-      <c r="E38" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="F38" s="30"/>
-      <c r="G38" s="30"/>
-      <c r="H38" s="30"/>
-      <c r="I38" s="30"/>
-      <c r="J38" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="K38" s="29"/>
-      <c r="L38" s="29"/>
-      <c r="M38" s="29"/>
-      <c r="N38" s="29"/>
-    </row>
-    <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A39" s="31" t="s">
-        <v>87</v>
-      </c>
-      <c r="B39" s="31"/>
-      <c r="C39" s="31"/>
-      <c r="D39" s="31"/>
-      <c r="E39" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="F39" s="32"/>
-      <c r="G39" s="32"/>
-      <c r="H39" s="32"/>
-      <c r="I39" s="32"/>
-      <c r="J39" s="31" t="s">
-        <v>57</v>
-      </c>
-      <c r="K39" s="31"/>
-      <c r="L39" s="31"/>
-      <c r="M39" s="31"/>
-      <c r="N39" s="31"/>
+      <c r="B39" s="34"/>
+      <c r="C39" s="34"/>
+      <c r="D39" s="34"/>
+      <c r="E39" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="F39" s="35"/>
+      <c r="G39" s="35"/>
+      <c r="H39" s="35"/>
+      <c r="I39" s="35"/>
+      <c r="J39" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="K39" s="34"/>
+      <c r="L39" s="34"/>
+      <c r="M39" s="34"/>
+      <c r="N39" s="34"/>
     </row>
     <row r="40" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A40" s="33" t="s">
+      <c r="A40" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="B40" s="33"/>
-      <c r="C40" s="33"/>
-      <c r="D40" s="33"/>
-      <c r="E40" s="34" t="s">
-        <v>24</v>
-      </c>
-      <c r="F40" s="34"/>
-      <c r="G40" s="34"/>
-      <c r="H40" s="34"/>
-      <c r="I40" s="34"/>
-      <c r="J40" s="33" t="s">
+      <c r="B40" s="36"/>
+      <c r="C40" s="36"/>
+      <c r="D40" s="36"/>
+      <c r="E40" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="K40" s="33"/>
-      <c r="L40" s="33"/>
-      <c r="M40" s="33"/>
-      <c r="N40" s="33"/>
+      <c r="F40" s="37"/>
+      <c r="G40" s="37"/>
+      <c r="H40" s="37"/>
+      <c r="I40" s="37"/>
+      <c r="J40" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="K40" s="36"/>
+      <c r="L40" s="36"/>
+      <c r="M40" s="36"/>
+      <c r="N40" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="52">

</xml_diff>

<commit_message>
feat(reporting): introduce payment method analytics
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -7,15 +7,16 @@
     <sheet sheetId="1" name="Cover" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Executive Summary" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Financial Summary" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Order Sales" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Check Revenue Trends" state="visible" r:id="rId8"/>
+    <sheet sheetId="4" name="Payment Method Analysis" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Order Sales" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Check Revenue Trends" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="139">
   <si>
     <t>MINEUQR</t>
   </si>
@@ -59,10 +60,10 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>18 Jul 2026, 22:10</t>
-  </si>
-  <si>
-    <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Order Sales  ·  Check Revenue Trends</t>
+    <t>18 Jul 2026, 22:22</t>
+  </si>
+  <si>
+    <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Payment Method Analysis  ·  Order Sales  ·  Check Revenue Trends</t>
   </si>
   <si>
     <t>Confidential — Internal Use  ·  Prepared by MineuQR</t>
@@ -71,7 +72,7 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 22:10</t>
+    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 22:22</t>
   </si>
   <si>
     <t>AT A GLANCE</t>
@@ -207,6 +208,72 @@
   </si>
   <si>
     <t>SAR (ر.س)</t>
+  </si>
+  <si>
+    <t>Payment Method Analysis</t>
+  </si>
+  <si>
+    <t>Payment mix is from settlement tenders. Check Revenue remains the official revenue total from paid checks.</t>
+  </si>
+  <si>
+    <t>PAYMENT MIX</t>
+  </si>
+  <si>
+    <t>Monetary Tender Total</t>
+  </si>
+  <si>
+    <t>Complimentary</t>
+  </si>
+  <si>
+    <t>PAYMENT METHOD ANALYSIS</t>
+  </si>
+  <si>
+    <t>Payment Method</t>
+  </si>
+  <si>
+    <t>Tender Amount</t>
+  </si>
+  <si>
+    <t>Paid Checks (by method)</t>
+  </si>
+  <si>
+    <t>Average Check (by method)</t>
+  </si>
+  <si>
+    <t>Mix %</t>
+  </si>
+  <si>
+    <t>Transactions</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>5,845.00 ر.س</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>216.48 ر.س</t>
+  </si>
+  <si>
+    <t>40.00%</t>
+  </si>
+  <si>
+    <t>Mada</t>
+  </si>
+  <si>
+    <t>8,767.50 ر.س</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>213.84 ر.س</t>
+  </si>
+  <si>
+    <t>60.00%</t>
   </si>
   <si>
     <t>Monthly Report  ·  Daily Order Sales — July 2026</t>
@@ -372,7 +439,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -489,6 +556,17 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF1E293B"/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF0C1222"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -595,7 +673,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -676,22 +754,25 @@
     <xf numFmtId="49" fontId="19" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="21" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="22" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="23" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="23" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="23" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="24" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="25" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2523,7 +2604,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="10.2" customWidth="1"/>
@@ -2531,7 +2612,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -2549,7 +2630,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2581,9 +2662,305 @@
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
     </row>
+    <row r="4" ht="10" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="21"/>
+      <c r="N5" s="21"/>
+    </row>
+    <row r="7" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="19"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+    </row>
+    <row r="8" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="J8" s="27"/>
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+      <c r="M8" s="27"/>
+      <c r="N8" s="27"/>
+    </row>
+    <row r="9" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="J9" s="29"/>
+      <c r="K9" s="29"/>
+      <c r="L9" s="29"/>
+      <c r="M9" s="29"/>
+      <c r="N9" s="29"/>
+    </row>
+    <row r="11" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
+      <c r="L11" s="19"/>
+      <c r="M11" s="19"/>
+      <c r="N11" s="19"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="30"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="H12" s="30"/>
+      <c r="I12" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="J12" s="30"/>
+      <c r="K12" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="L12" s="30"/>
+      <c r="M12" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="N12" s="30"/>
+    </row>
+    <row r="13" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="31" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="32" t="s">
+        <v>77</v>
+      </c>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="31" t="s">
+        <v>78</v>
+      </c>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="J13" s="31"/>
+      <c r="K13" s="31" t="s">
+        <v>80</v>
+      </c>
+      <c r="L13" s="31"/>
+      <c r="M13" s="31" t="s">
+        <v>78</v>
+      </c>
+      <c r="N13" s="31"/>
+    </row>
+    <row r="14" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="31" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="31"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="31" t="s">
+        <v>83</v>
+      </c>
+      <c r="H14" s="31"/>
+      <c r="I14" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31" t="s">
+        <v>85</v>
+      </c>
+      <c r="L14" s="31"/>
+      <c r="M14" s="31" t="s">
+        <v>83</v>
+      </c>
+      <c r="N14" s="31"/>
+    </row>
+  </sheetData>
+  <mergeCells count="27">
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A5:N5"/>
+    <mergeCell ref="A7:N7"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="I8:N8"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="I9:N9"/>
+    <mergeCell ref="A11:N11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="K12:L12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="M14:N14"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.25" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddFooter>&amp;LMineuQR Executive Report&amp;RPage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:N39"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="14" width="10.2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+    </row>
+    <row r="3" ht="4" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+    </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -2890,388 +3267,388 @@
       <c r="N23" s="19"/>
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="B24" s="30"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="31" t="s">
+      <c r="A24" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="33"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="E24" s="31"/>
-      <c r="F24" s="31"/>
-      <c r="G24" s="31" t="s">
+      <c r="E24" s="34"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="H24" s="31"/>
-      <c r="I24" s="31"/>
-      <c r="J24" s="31" t="s">
+      <c r="H24" s="34"/>
+      <c r="I24" s="34"/>
+      <c r="J24" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="K24" s="31"/>
-      <c r="L24" s="31"/>
-      <c r="M24" s="31"/>
-      <c r="N24" s="31"/>
+      <c r="K24" s="34"/>
+      <c r="L24" s="34"/>
+      <c r="M24" s="34"/>
+      <c r="N24" s="34"/>
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32" t="s">
-        <v>68</v>
-      </c>
-      <c r="E25" s="32"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="H25" s="32"/>
-      <c r="I25" s="32"/>
-      <c r="J25" s="33" t="s">
-        <v>70</v>
-      </c>
-      <c r="K25" s="33"/>
-      <c r="L25" s="33"/>
-      <c r="M25" s="33"/>
-      <c r="N25" s="33"/>
+      <c r="A25" s="35" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="E25" s="35"/>
+      <c r="F25" s="35"/>
+      <c r="G25" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="H25" s="35"/>
+      <c r="I25" s="35"/>
+      <c r="J25" s="36" t="s">
+        <v>92</v>
+      </c>
+      <c r="K25" s="36"/>
+      <c r="L25" s="36"/>
+      <c r="M25" s="36"/>
+      <c r="N25" s="36"/>
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="34" t="s">
-        <v>71</v>
-      </c>
-      <c r="B26" s="34"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="E26" s="34"/>
-      <c r="F26" s="34"/>
-      <c r="G26" s="34" t="s">
-        <v>68</v>
-      </c>
-      <c r="H26" s="34"/>
-      <c r="I26" s="34"/>
-      <c r="J26" s="35" t="s">
-        <v>73</v>
-      </c>
-      <c r="K26" s="35"/>
-      <c r="L26" s="35"/>
-      <c r="M26" s="35"/>
-      <c r="N26" s="35"/>
+      <c r="A26" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="B26" s="37"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="E26" s="37"/>
+      <c r="F26" s="37"/>
+      <c r="G26" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="H26" s="37"/>
+      <c r="I26" s="37"/>
+      <c r="J26" s="38" t="s">
+        <v>95</v>
+      </c>
+      <c r="K26" s="38"/>
+      <c r="L26" s="38"/>
+      <c r="M26" s="38"/>
+      <c r="N26" s="38"/>
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="B27" s="32"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="H27" s="32"/>
-      <c r="I27" s="32"/>
-      <c r="J27" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="K27" s="33"/>
-      <c r="L27" s="33"/>
-      <c r="M27" s="33"/>
-      <c r="N27" s="33"/>
+      <c r="A27" s="35" t="s">
+        <v>96</v>
+      </c>
+      <c r="B27" s="35"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="35" t="s">
+        <v>97</v>
+      </c>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="H27" s="35"/>
+      <c r="I27" s="35"/>
+      <c r="J27" s="36" t="s">
+        <v>98</v>
+      </c>
+      <c r="K27" s="36"/>
+      <c r="L27" s="36"/>
+      <c r="M27" s="36"/>
+      <c r="N27" s="36"/>
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B28" s="34"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="E28" s="34"/>
-      <c r="F28" s="34"/>
-      <c r="G28" s="34" t="s">
-        <v>75</v>
-      </c>
-      <c r="H28" s="34"/>
-      <c r="I28" s="34"/>
-      <c r="J28" s="35" t="s">
-        <v>79</v>
-      </c>
-      <c r="K28" s="35"/>
-      <c r="L28" s="35"/>
-      <c r="M28" s="35"/>
-      <c r="N28" s="35"/>
+      <c r="A28" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" s="37"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="E28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="H28" s="37"/>
+      <c r="I28" s="37"/>
+      <c r="J28" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="K28" s="38"/>
+      <c r="L28" s="38"/>
+      <c r="M28" s="38"/>
+      <c r="N28" s="38"/>
     </row>
     <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="B29" s="32"/>
-      <c r="C29" s="32"/>
-      <c r="D29" s="32" t="s">
-        <v>68</v>
-      </c>
-      <c r="E29" s="32"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="H29" s="32"/>
-      <c r="I29" s="32"/>
-      <c r="J29" s="33" t="s">
-        <v>81</v>
-      </c>
-      <c r="K29" s="33"/>
-      <c r="L29" s="33"/>
-      <c r="M29" s="33"/>
-      <c r="N29" s="33"/>
+      <c r="A29" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="B29" s="35"/>
+      <c r="C29" s="35"/>
+      <c r="D29" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="E29" s="35"/>
+      <c r="F29" s="35"/>
+      <c r="G29" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="H29" s="35"/>
+      <c r="I29" s="35"/>
+      <c r="J29" s="36" t="s">
+        <v>103</v>
+      </c>
+      <c r="K29" s="36"/>
+      <c r="L29" s="36"/>
+      <c r="M29" s="36"/>
+      <c r="N29" s="36"/>
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="34" t="s">
-        <v>82</v>
-      </c>
-      <c r="B30" s="34"/>
-      <c r="C30" s="34"/>
-      <c r="D30" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="E30" s="34"/>
-      <c r="F30" s="34"/>
-      <c r="G30" s="34" t="s">
-        <v>68</v>
-      </c>
-      <c r="H30" s="34"/>
-      <c r="I30" s="34"/>
-      <c r="J30" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="K30" s="35"/>
-      <c r="L30" s="35"/>
-      <c r="M30" s="35"/>
-      <c r="N30" s="35"/>
+      <c r="A30" s="37" t="s">
+        <v>104</v>
+      </c>
+      <c r="B30" s="37"/>
+      <c r="C30" s="37"/>
+      <c r="D30" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="E30" s="37"/>
+      <c r="F30" s="37"/>
+      <c r="G30" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="H30" s="37"/>
+      <c r="I30" s="37"/>
+      <c r="J30" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="K30" s="38"/>
+      <c r="L30" s="38"/>
+      <c r="M30" s="38"/>
+      <c r="N30" s="38"/>
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="32" t="s">
-        <v>84</v>
-      </c>
-      <c r="B31" s="32"/>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="H31" s="32"/>
-      <c r="I31" s="32"/>
-      <c r="J31" s="33" t="s">
-        <v>85</v>
-      </c>
-      <c r="K31" s="33"/>
-      <c r="L31" s="33"/>
-      <c r="M31" s="33"/>
-      <c r="N31" s="33"/>
+      <c r="A31" s="35" t="s">
+        <v>106</v>
+      </c>
+      <c r="B31" s="35"/>
+      <c r="C31" s="35"/>
+      <c r="D31" s="35" t="s">
+        <v>97</v>
+      </c>
+      <c r="E31" s="35"/>
+      <c r="F31" s="35"/>
+      <c r="G31" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="H31" s="35"/>
+      <c r="I31" s="35"/>
+      <c r="J31" s="36" t="s">
+        <v>107</v>
+      </c>
+      <c r="K31" s="36"/>
+      <c r="L31" s="36"/>
+      <c r="M31" s="36"/>
+      <c r="N31" s="36"/>
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="B32" s="34"/>
-      <c r="C32" s="34"/>
-      <c r="D32" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="E32" s="34"/>
-      <c r="F32" s="34"/>
-      <c r="G32" s="34" t="s">
-        <v>75</v>
-      </c>
-      <c r="H32" s="34"/>
-      <c r="I32" s="34"/>
-      <c r="J32" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="K32" s="35"/>
-      <c r="L32" s="35"/>
-      <c r="M32" s="35"/>
-      <c r="N32" s="35"/>
+      <c r="A32" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="B32" s="37"/>
+      <c r="C32" s="37"/>
+      <c r="D32" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="E32" s="37"/>
+      <c r="F32" s="37"/>
+      <c r="G32" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="H32" s="37"/>
+      <c r="I32" s="37"/>
+      <c r="J32" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="K32" s="38"/>
+      <c r="L32" s="38"/>
+      <c r="M32" s="38"/>
+      <c r="N32" s="38"/>
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="32" t="s">
-        <v>88</v>
-      </c>
-      <c r="B33" s="32"/>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32" t="s">
-        <v>68</v>
-      </c>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="H33" s="32"/>
-      <c r="I33" s="32"/>
-      <c r="J33" s="33" t="s">
-        <v>89</v>
-      </c>
-      <c r="K33" s="33"/>
-      <c r="L33" s="33"/>
-      <c r="M33" s="33"/>
-      <c r="N33" s="33"/>
+      <c r="A33" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="B33" s="35"/>
+      <c r="C33" s="35"/>
+      <c r="D33" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="E33" s="35"/>
+      <c r="F33" s="35"/>
+      <c r="G33" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="H33" s="35"/>
+      <c r="I33" s="35"/>
+      <c r="J33" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="K33" s="36"/>
+      <c r="L33" s="36"/>
+      <c r="M33" s="36"/>
+      <c r="N33" s="36"/>
     </row>
     <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="34" t="s">
+      <c r="A34" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="B34" s="37"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="E34" s="37"/>
+      <c r="F34" s="37"/>
+      <c r="G34" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="B34" s="34"/>
-      <c r="C34" s="34"/>
-      <c r="D34" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="E34" s="34"/>
-      <c r="F34" s="34"/>
-      <c r="G34" s="34" t="s">
-        <v>68</v>
-      </c>
-      <c r="H34" s="34"/>
-      <c r="I34" s="34"/>
-      <c r="J34" s="35" t="s">
+      <c r="H34" s="37"/>
+      <c r="I34" s="37"/>
+      <c r="J34" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="K34" s="38"/>
+      <c r="L34" s="38"/>
+      <c r="M34" s="38"/>
+      <c r="N34" s="38"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="35" t="s">
+        <v>114</v>
+      </c>
+      <c r="B35" s="35"/>
+      <c r="C35" s="35"/>
+      <c r="D35" s="35" t="s">
+        <v>97</v>
+      </c>
+      <c r="E35" s="35"/>
+      <c r="F35" s="35"/>
+      <c r="G35" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="H35" s="35"/>
+      <c r="I35" s="35"/>
+      <c r="J35" s="36" t="s">
+        <v>115</v>
+      </c>
+      <c r="K35" s="36"/>
+      <c r="L35" s="36"/>
+      <c r="M35" s="36"/>
+      <c r="N35" s="36"/>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="37" t="s">
+        <v>116</v>
+      </c>
+      <c r="B36" s="37"/>
+      <c r="C36" s="37"/>
+      <c r="D36" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="E36" s="37"/>
+      <c r="F36" s="37"/>
+      <c r="G36" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="H36" s="37"/>
+      <c r="I36" s="37"/>
+      <c r="J36" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="K36" s="38"/>
+      <c r="L36" s="38"/>
+      <c r="M36" s="38"/>
+      <c r="N36" s="38"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="35" t="s">
+        <v>118</v>
+      </c>
+      <c r="B37" s="35"/>
+      <c r="C37" s="35"/>
+      <c r="D37" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="E37" s="35"/>
+      <c r="F37" s="35"/>
+      <c r="G37" s="35" t="s">
         <v>91</v>
       </c>
-      <c r="K34" s="35"/>
-      <c r="L34" s="35"/>
-      <c r="M34" s="35"/>
-      <c r="N34" s="35"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="B35" s="32"/>
-      <c r="C35" s="32"/>
-      <c r="D35" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="E35" s="32"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="H35" s="32"/>
-      <c r="I35" s="32"/>
-      <c r="J35" s="33" t="s">
-        <v>93</v>
-      </c>
-      <c r="K35" s="33"/>
-      <c r="L35" s="33"/>
-      <c r="M35" s="33"/>
-      <c r="N35" s="33"/>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" s="34" t="s">
+      <c r="H37" s="35"/>
+      <c r="I37" s="35"/>
+      <c r="J37" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="K37" s="36"/>
+      <c r="L37" s="36"/>
+      <c r="M37" s="36"/>
+      <c r="N37" s="36"/>
+    </row>
+    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="37" t="s">
+        <v>120</v>
+      </c>
+      <c r="B38" s="37"/>
+      <c r="C38" s="37"/>
+      <c r="D38" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="B36" s="34"/>
-      <c r="C36" s="34"/>
-      <c r="D36" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="E36" s="34"/>
-      <c r="F36" s="34"/>
-      <c r="G36" s="34" t="s">
-        <v>75</v>
-      </c>
-      <c r="H36" s="34"/>
-      <c r="I36" s="34"/>
-      <c r="J36" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="K36" s="35"/>
-      <c r="L36" s="35"/>
-      <c r="M36" s="35"/>
-      <c r="N36" s="35"/>
-    </row>
-    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="32" t="s">
-        <v>68</v>
-      </c>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="H37" s="32"/>
-      <c r="I37" s="32"/>
-      <c r="J37" s="33" t="s">
-        <v>97</v>
-      </c>
-      <c r="K37" s="33"/>
-      <c r="L37" s="33"/>
-      <c r="M37" s="33"/>
-      <c r="N37" s="33"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="B38" s="34"/>
-      <c r="C38" s="34"/>
-      <c r="D38" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="E38" s="34"/>
-      <c r="F38" s="34"/>
-      <c r="G38" s="34" t="s">
-        <v>68</v>
-      </c>
-      <c r="H38" s="34"/>
-      <c r="I38" s="34"/>
-      <c r="J38" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="K38" s="35"/>
-      <c r="L38" s="35"/>
-      <c r="M38" s="35"/>
-      <c r="N38" s="35"/>
+      <c r="E38" s="37"/>
+      <c r="F38" s="37"/>
+      <c r="G38" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="H38" s="37"/>
+      <c r="I38" s="37"/>
+      <c r="J38" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="K38" s="38"/>
+      <c r="L38" s="38"/>
+      <c r="M38" s="38"/>
+      <c r="N38" s="38"/>
     </row>
     <row r="39" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A39" s="36" t="s">
+      <c r="A39" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="B39" s="36"/>
-      <c r="C39" s="36"/>
-      <c r="D39" s="36" t="s">
+      <c r="B39" s="39"/>
+      <c r="C39" s="39"/>
+      <c r="D39" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="E39" s="36"/>
-      <c r="F39" s="36"/>
-      <c r="G39" s="36" t="s">
+      <c r="E39" s="39"/>
+      <c r="F39" s="39"/>
+      <c r="G39" s="39" t="s">
         <v>52</v>
       </c>
-      <c r="H39" s="36"/>
-      <c r="I39" s="36"/>
-      <c r="J39" s="37" t="s">
+      <c r="H39" s="39"/>
+      <c r="I39" s="39"/>
+      <c r="J39" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="K39" s="37"/>
-      <c r="L39" s="37"/>
-      <c r="M39" s="37"/>
-      <c r="N39" s="37"/>
+      <c r="K39" s="40"/>
+      <c r="L39" s="40"/>
+      <c r="M39" s="40"/>
+      <c r="N39" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="68">
@@ -3354,7 +3731,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3367,7 +3744,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -3385,7 +3762,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3419,7 +3796,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>102</v>
+        <v>124</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -3742,356 +4119,356 @@
       <c r="N24" s="19"/>
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="B25" s="30"/>
-      <c r="C25" s="30"/>
-      <c r="D25" s="30"/>
-      <c r="E25" s="31" t="s">
+      <c r="A25" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="B25" s="33"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="F25" s="31"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
-      <c r="I25" s="31"/>
-      <c r="J25" s="31" t="s">
+      <c r="F25" s="34"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="34"/>
+      <c r="I25" s="34"/>
+      <c r="J25" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="K25" s="31"/>
-      <c r="L25" s="31"/>
-      <c r="M25" s="31"/>
-      <c r="N25" s="31"/>
+      <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
+      <c r="M25" s="34"/>
+      <c r="N25" s="34"/>
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="B26" s="32"/>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="33" t="s">
-        <v>103</v>
-      </c>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="33"/>
-      <c r="J26" s="32" t="s">
+      <c r="A26" s="35" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" s="35"/>
+      <c r="C26" s="35"/>
+      <c r="D26" s="35"/>
+      <c r="E26" s="36" t="s">
+        <v>125</v>
+      </c>
+      <c r="F26" s="36"/>
+      <c r="G26" s="36"/>
+      <c r="H26" s="36"/>
+      <c r="I26" s="36"/>
+      <c r="J26" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="K26" s="32"/>
-      <c r="L26" s="32"/>
-      <c r="M26" s="32"/>
-      <c r="N26" s="32"/>
+      <c r="K26" s="35"/>
+      <c r="L26" s="35"/>
+      <c r="M26" s="35"/>
+      <c r="N26" s="35"/>
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="34" t="s">
-        <v>71</v>
-      </c>
-      <c r="B27" s="34"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="35" t="s">
+      <c r="A27" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="F27" s="38"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="38"/>
+      <c r="J27" s="37" t="s">
+        <v>127</v>
+      </c>
+      <c r="K27" s="37"/>
+      <c r="L27" s="37"/>
+      <c r="M27" s="37"/>
+      <c r="N27" s="37"/>
+    </row>
+    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="35" t="s">
+        <v>96</v>
+      </c>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="36" t="s">
+        <v>128</v>
+      </c>
+      <c r="F28" s="36"/>
+      <c r="G28" s="36"/>
+      <c r="H28" s="36"/>
+      <c r="I28" s="36"/>
+      <c r="J28" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="K28" s="35"/>
+      <c r="L28" s="35"/>
+      <c r="M28" s="35"/>
+      <c r="N28" s="35"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="B29" s="37"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="37"/>
+      <c r="E29" s="38" t="s">
+        <v>129</v>
+      </c>
+      <c r="F29" s="38"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="38"/>
+      <c r="I29" s="38"/>
+      <c r="J29" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="K29" s="37"/>
+      <c r="L29" s="37"/>
+      <c r="M29" s="37"/>
+      <c r="N29" s="37"/>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="B30" s="35"/>
+      <c r="C30" s="35"/>
+      <c r="D30" s="35"/>
+      <c r="E30" s="36" t="s">
+        <v>130</v>
+      </c>
+      <c r="F30" s="36"/>
+      <c r="G30" s="36"/>
+      <c r="H30" s="36"/>
+      <c r="I30" s="36"/>
+      <c r="J30" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="K30" s="35"/>
+      <c r="L30" s="35"/>
+      <c r="M30" s="35"/>
+      <c r="N30" s="35"/>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="37" t="s">
         <v>104</v>
       </c>
-      <c r="F27" s="35"/>
-      <c r="G27" s="35"/>
-      <c r="H27" s="35"/>
-      <c r="I27" s="35"/>
-      <c r="J27" s="34" t="s">
-        <v>105</v>
-      </c>
-      <c r="K27" s="34"/>
-      <c r="L27" s="34"/>
-      <c r="M27" s="34"/>
-      <c r="N27" s="34"/>
-    </row>
-    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="B28" s="32"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="33" t="s">
+      <c r="B31" s="37"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="38" t="s">
+        <v>131</v>
+      </c>
+      <c r="F31" s="38"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="38"/>
+      <c r="J31" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="K31" s="37"/>
+      <c r="L31" s="37"/>
+      <c r="M31" s="37"/>
+      <c r="N31" s="37"/>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="35" t="s">
         <v>106</v>
       </c>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="K28" s="32"/>
-      <c r="L28" s="32"/>
-      <c r="M28" s="32"/>
-      <c r="N28" s="32"/>
-    </row>
-    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="B29" s="34"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="35" t="s">
-        <v>107</v>
-      </c>
-      <c r="F29" s="35"/>
-      <c r="G29" s="35"/>
-      <c r="H29" s="35"/>
-      <c r="I29" s="35"/>
-      <c r="J29" s="34" t="s">
-        <v>68</v>
-      </c>
-      <c r="K29" s="34"/>
-      <c r="L29" s="34"/>
-      <c r="M29" s="34"/>
-      <c r="N29" s="34"/>
-    </row>
-    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="B30" s="32"/>
-      <c r="C30" s="32"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="33" t="s">
+      <c r="B32" s="35"/>
+      <c r="C32" s="35"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="F32" s="36"/>
+      <c r="G32" s="36"/>
+      <c r="H32" s="36"/>
+      <c r="I32" s="36"/>
+      <c r="J32" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="K32" s="35"/>
+      <c r="L32" s="35"/>
+      <c r="M32" s="35"/>
+      <c r="N32" s="35"/>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="F30" s="33"/>
-      <c r="G30" s="33"/>
-      <c r="H30" s="33"/>
-      <c r="I30" s="33"/>
-      <c r="J30" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="K30" s="32"/>
-      <c r="L30" s="32"/>
-      <c r="M30" s="32"/>
-      <c r="N30" s="32"/>
-    </row>
-    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="34" t="s">
-        <v>82</v>
-      </c>
-      <c r="B31" s="34"/>
-      <c r="C31" s="34"/>
-      <c r="D31" s="34"/>
-      <c r="E31" s="35" t="s">
-        <v>109</v>
-      </c>
-      <c r="F31" s="35"/>
-      <c r="G31" s="35"/>
-      <c r="H31" s="35"/>
-      <c r="I31" s="35"/>
-      <c r="J31" s="34" t="s">
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="38" t="s">
+        <v>133</v>
+      </c>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="38"/>
+      <c r="I33" s="38"/>
+      <c r="J33" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="K33" s="37"/>
+      <c r="L33" s="37"/>
+      <c r="M33" s="37"/>
+      <c r="N33" s="37"/>
+    </row>
+    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="B34" s="35"/>
+      <c r="C34" s="35"/>
+      <c r="D34" s="35"/>
+      <c r="E34" s="36" t="s">
+        <v>92</v>
+      </c>
+      <c r="F34" s="36"/>
+      <c r="G34" s="36"/>
+      <c r="H34" s="36"/>
+      <c r="I34" s="36"/>
+      <c r="J34" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="K34" s="35"/>
+      <c r="L34" s="35"/>
+      <c r="M34" s="35"/>
+      <c r="N34" s="35"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="B35" s="37"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="38" t="s">
+        <v>134</v>
+      </c>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
+      <c r="I35" s="38"/>
+      <c r="J35" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="K35" s="37"/>
+      <c r="L35" s="37"/>
+      <c r="M35" s="37"/>
+      <c r="N35" s="37"/>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="35" t="s">
+        <v>114</v>
+      </c>
+      <c r="B36" s="35"/>
+      <c r="C36" s="35"/>
+      <c r="D36" s="35"/>
+      <c r="E36" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="F36" s="36"/>
+      <c r="G36" s="36"/>
+      <c r="H36" s="36"/>
+      <c r="I36" s="36"/>
+      <c r="J36" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="K31" s="34"/>
-      <c r="L31" s="34"/>
-      <c r="M31" s="34"/>
-      <c r="N31" s="34"/>
-    </row>
-    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="32" t="s">
-        <v>84</v>
-      </c>
-      <c r="B32" s="32"/>
-      <c r="C32" s="32"/>
-      <c r="D32" s="32"/>
-      <c r="E32" s="33" t="s">
-        <v>110</v>
-      </c>
-      <c r="F32" s="33"/>
-      <c r="G32" s="33"/>
-      <c r="H32" s="33"/>
-      <c r="I32" s="33"/>
-      <c r="J32" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="K32" s="32"/>
-      <c r="L32" s="32"/>
-      <c r="M32" s="32"/>
-      <c r="N32" s="32"/>
-    </row>
-    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="35" t="s">
-        <v>111</v>
-      </c>
-      <c r="F33" s="35"/>
-      <c r="G33" s="35"/>
-      <c r="H33" s="35"/>
-      <c r="I33" s="35"/>
-      <c r="J33" s="34" t="s">
-        <v>69</v>
-      </c>
-      <c r="K33" s="34"/>
-      <c r="L33" s="34"/>
-      <c r="M33" s="34"/>
-      <c r="N33" s="34"/>
-    </row>
-    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="32" t="s">
-        <v>88</v>
-      </c>
-      <c r="B34" s="32"/>
-      <c r="C34" s="32"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="33" t="s">
-        <v>70</v>
-      </c>
-      <c r="F34" s="33"/>
-      <c r="G34" s="33"/>
-      <c r="H34" s="33"/>
-      <c r="I34" s="33"/>
-      <c r="J34" s="32" t="s">
-        <v>68</v>
-      </c>
-      <c r="K34" s="32"/>
-      <c r="L34" s="32"/>
-      <c r="M34" s="32"/>
-      <c r="N34" s="32"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="34" t="s">
+      <c r="K36" s="35"/>
+      <c r="L36" s="35"/>
+      <c r="M36" s="35"/>
+      <c r="N36" s="35"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="37" t="s">
+        <v>116</v>
+      </c>
+      <c r="B37" s="37"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="37"/>
+      <c r="E37" s="38" t="s">
+        <v>136</v>
+      </c>
+      <c r="F37" s="38"/>
+      <c r="G37" s="38"/>
+      <c r="H37" s="38"/>
+      <c r="I37" s="38"/>
+      <c r="J37" s="37" t="s">
+        <v>127</v>
+      </c>
+      <c r="K37" s="37"/>
+      <c r="L37" s="37"/>
+      <c r="M37" s="37"/>
+      <c r="N37" s="37"/>
+    </row>
+    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="35" t="s">
+        <v>118</v>
+      </c>
+      <c r="B38" s="35"/>
+      <c r="C38" s="35"/>
+      <c r="D38" s="35"/>
+      <c r="E38" s="36" t="s">
+        <v>137</v>
+      </c>
+      <c r="F38" s="36"/>
+      <c r="G38" s="36"/>
+      <c r="H38" s="36"/>
+      <c r="I38" s="36"/>
+      <c r="J38" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="K38" s="35"/>
+      <c r="L38" s="35"/>
+      <c r="M38" s="35"/>
+      <c r="N38" s="35"/>
+    </row>
+    <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" s="37" t="s">
+        <v>120</v>
+      </c>
+      <c r="B39" s="37"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="37"/>
+      <c r="E39" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="F39" s="38"/>
+      <c r="G39" s="38"/>
+      <c r="H39" s="38"/>
+      <c r="I39" s="38"/>
+      <c r="J39" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="B35" s="34"/>
-      <c r="C35" s="34"/>
-      <c r="D35" s="34"/>
-      <c r="E35" s="35" t="s">
-        <v>112</v>
-      </c>
-      <c r="F35" s="35"/>
-      <c r="G35" s="35"/>
-      <c r="H35" s="35"/>
-      <c r="I35" s="35"/>
-      <c r="J35" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="K35" s="34"/>
-      <c r="L35" s="34"/>
-      <c r="M35" s="34"/>
-      <c r="N35" s="34"/>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="33" t="s">
-        <v>113</v>
-      </c>
-      <c r="F36" s="33"/>
-      <c r="G36" s="33"/>
-      <c r="H36" s="33"/>
-      <c r="I36" s="33"/>
-      <c r="J36" s="32" t="s">
-        <v>55</v>
-      </c>
-      <c r="K36" s="32"/>
-      <c r="L36" s="32"/>
-      <c r="M36" s="32"/>
-      <c r="N36" s="32"/>
-    </row>
-    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="B37" s="34"/>
-      <c r="C37" s="34"/>
-      <c r="D37" s="34"/>
-      <c r="E37" s="35" t="s">
-        <v>114</v>
-      </c>
-      <c r="F37" s="35"/>
-      <c r="G37" s="35"/>
-      <c r="H37" s="35"/>
-      <c r="I37" s="35"/>
-      <c r="J37" s="34" t="s">
-        <v>105</v>
-      </c>
-      <c r="K37" s="34"/>
-      <c r="L37" s="34"/>
-      <c r="M37" s="34"/>
-      <c r="N37" s="34"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="33" t="s">
-        <v>115</v>
-      </c>
-      <c r="F38" s="33"/>
-      <c r="G38" s="33"/>
-      <c r="H38" s="33"/>
-      <c r="I38" s="33"/>
-      <c r="J38" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="K38" s="32"/>
-      <c r="L38" s="32"/>
-      <c r="M38" s="32"/>
-      <c r="N38" s="32"/>
-    </row>
-    <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A39" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="B39" s="34"/>
-      <c r="C39" s="34"/>
-      <c r="D39" s="34"/>
-      <c r="E39" s="35" t="s">
-        <v>116</v>
-      </c>
-      <c r="F39" s="35"/>
-      <c r="G39" s="35"/>
-      <c r="H39" s="35"/>
-      <c r="I39" s="35"/>
-      <c r="J39" s="34" t="s">
-        <v>68</v>
-      </c>
-      <c r="K39" s="34"/>
-      <c r="L39" s="34"/>
-      <c r="M39" s="34"/>
-      <c r="N39" s="34"/>
+      <c r="K39" s="37"/>
+      <c r="L39" s="37"/>
+      <c r="M39" s="37"/>
+      <c r="N39" s="37"/>
     </row>
     <row r="40" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A40" s="36" t="s">
+      <c r="A40" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="B40" s="36"/>
-      <c r="C40" s="36"/>
-      <c r="D40" s="36"/>
-      <c r="E40" s="37" t="s">
+      <c r="B40" s="39"/>
+      <c r="C40" s="39"/>
+      <c r="D40" s="39"/>
+      <c r="E40" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="F40" s="37"/>
-      <c r="G40" s="37"/>
-      <c r="H40" s="37"/>
-      <c r="I40" s="37"/>
-      <c r="J40" s="36" t="s">
+      <c r="F40" s="40"/>
+      <c r="G40" s="40"/>
+      <c r="H40" s="40"/>
+      <c r="I40" s="40"/>
+      <c r="J40" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="K40" s="36"/>
-      <c r="L40" s="36"/>
-      <c r="M40" s="36"/>
-      <c r="N40" s="36"/>
+      <c r="K40" s="39"/>
+      <c r="L40" s="39"/>
+      <c r="M40" s="39"/>
+      <c r="N40" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="52">

</xml_diff>

<commit_message>
refactor(reporting): simplify executive summary presentation
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="137">
   <si>
     <t>MINEUQR</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>18 Jul 2026, 22:22</t>
+    <t>18 Jul 2026, 22:35</t>
   </si>
   <si>
     <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Payment Method Analysis  ·  Order Sales  ·  Check Revenue Trends</t>
@@ -72,94 +72,88 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 22:22</t>
+    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 22:35</t>
   </si>
   <si>
     <t>AT A GLANCE</t>
   </si>
   <si>
-    <t>How did the restaurant perform this period?</t>
+    <t>How is the restaurant performing operationally?</t>
+  </si>
+  <si>
+    <t>ORDERS SERVED</t>
+  </si>
+  <si>
+    <t>From completed kitchen orders — your Order Sales story for this period.</t>
+  </si>
+  <si>
+    <t>Order Sales</t>
+  </si>
+  <si>
+    <t>Orders</t>
+  </si>
+  <si>
+    <t>Average Order</t>
+  </si>
+  <si>
+    <t>19,222.00 ر.س</t>
+  </si>
+  <si>
+    <t>103</t>
+  </si>
+  <si>
+    <t>215.98 ر.س</t>
+  </si>
+  <si>
+    <t>Value of orders that were completed (served)</t>
+  </si>
+  <si>
+    <t>How many orders were placed</t>
+  </si>
+  <si>
+    <t>Typical size of a completed order</t>
+  </si>
+  <si>
+    <t>Check Revenue, Paid Checks, Average Check, and Tax Collected are in Financial Summary. Payment mix is in Payment Method Analysis.</t>
+  </si>
+  <si>
+    <t>Financial Summary</t>
+  </si>
+  <si>
+    <t>Monthly Report  ·  July 2026</t>
   </si>
   <si>
     <t>MONEY COLLECTED</t>
   </si>
   <si>
-    <t>From paid guest checks — your Check Revenue story.</t>
+    <t>Paid guest checks for this reporting period — Check Revenue story.</t>
+  </si>
+  <si>
+    <t>CHECK REVENUE DETAIL</t>
   </si>
   <si>
     <t>Check Revenue</t>
   </si>
   <si>
+    <t>14,612.50 ر.س</t>
+  </si>
+  <si>
     <t>Paid Checks</t>
   </si>
   <si>
+    <t>68</t>
+  </si>
+  <si>
     <t>Average Check</t>
   </si>
   <si>
-    <t>14,612.50 ر.س</t>
-  </si>
-  <si>
-    <t>68</t>
-  </si>
-  <si>
     <t>214.89 ر.س</t>
   </si>
   <si>
-    <t>What guests paid on settled checks</t>
-  </si>
-  <si>
-    <t>How many checks were paid</t>
-  </si>
-  <si>
-    <t>Typical size of a paid check</t>
-  </si>
-  <si>
-    <t>ORDERS SERVED</t>
-  </si>
-  <si>
-    <t>From completed kitchen orders — your Order Sales story.</t>
-  </si>
-  <si>
-    <t>Order Sales</t>
-  </si>
-  <si>
-    <t>Orders</t>
-  </si>
-  <si>
-    <t>Average Order</t>
-  </si>
-  <si>
-    <t>19,222.00 ر.س</t>
-  </si>
-  <si>
-    <t>103</t>
-  </si>
-  <si>
-    <t>215.98 ر.س</t>
-  </si>
-  <si>
-    <t>Value of orders that were completed (served)</t>
-  </si>
-  <si>
-    <t>How many orders were placed</t>
-  </si>
-  <si>
-    <t>Typical size of a completed order</t>
-  </si>
-  <si>
-    <t>These two money totals measure different things and can differ. Check Revenue is money collected on paid checks; Order Sales is the value of completed orders. Average Check uses Check Revenue; Average Order uses Order Sales.</t>
-  </si>
-  <si>
-    <t>Financial Summary</t>
-  </si>
-  <si>
-    <t>Monthly Report  ·  July 2026</t>
-  </si>
-  <si>
-    <t>CHECK REVENUE DETAIL</t>
-  </si>
-  <si>
     <t>TAX</t>
+  </si>
+  <si>
+    <t>Tax Collected is the total tax from all paid checks in this reporting period (not a subset of sections).</t>
   </si>
   <si>
     <t>Tax Collected</t>
@@ -673,7 +667,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -752,6 +746,12 @@
       <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="19" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="49" fontId="20" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1666,7 +1666,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="10.2" customWidth="1"/>
@@ -1886,136 +1886,26 @@
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
     </row>
-    <row r="16" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="19" t="s">
+    <row r="16" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
-      <c r="L16" s="19"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="19"/>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="21"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="21"/>
-      <c r="K17" s="21"/>
-      <c r="L17" s="21"/>
-      <c r="M17" s="21"/>
-      <c r="N17" s="21"/>
-    </row>
-    <row r="18" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="F18" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="K18" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-    </row>
-    <row r="19" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="F19" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="G19" s="23"/>
-      <c r="H19" s="23"/>
-      <c r="I19" s="23"/>
-      <c r="K19" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="L19" s="23"/>
-      <c r="M19" s="23"/>
-      <c r="N19" s="23"/>
-    </row>
-    <row r="20" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="F20" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-      <c r="K20" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="L20" s="24"/>
-      <c r="M20" s="24"/>
-      <c r="N20" s="24"/>
-    </row>
-    <row r="21" ht="5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
-      <c r="M21" s="3"/>
-      <c r="N21" s="3"/>
-    </row>
-    <row r="24" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="25" t="s">
-        <v>43</v>
-      </c>
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="25"/>
-      <c r="J24" s="25"/>
-      <c r="K24" s="25"/>
-      <c r="L24" s="25"/>
-      <c r="M24" s="25"/>
-      <c r="N24" s="25"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="25"/>
+      <c r="K16" s="25"/>
+      <c r="L16" s="25"/>
+      <c r="M16" s="25"/>
+      <c r="N16" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="19">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A5:N5"/>
@@ -2035,20 +1925,6 @@
     <mergeCell ref="F13:I13"/>
     <mergeCell ref="K13:N13"/>
     <mergeCell ref="A16:N16"/>
-    <mergeCell ref="A17:N17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="K18:N18"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="K19:N19"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="F20:I20"/>
-    <mergeCell ref="K20:N20"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="F21:I21"/>
-    <mergeCell ref="K21:N21"/>
-    <mergeCell ref="A24:N24"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.25" footer="0.3"/>
@@ -2064,7 +1940,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="10.2" customWidth="1"/>
@@ -2072,7 +1948,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -2090,7 +1966,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2140,7 +2016,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -2156,49 +2032,45 @@
       <c r="M5" s="19"/>
       <c r="N5" s="19"/>
     </row>
-    <row r="6" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="27"/>
-      <c r="M6" s="27"/>
-      <c r="N6" s="27"/>
-    </row>
-    <row r="7" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="28" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
-      <c r="I7" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="29"/>
-      <c r="K7" s="29"/>
-      <c r="L7" s="29"/>
-      <c r="M7" s="29"/>
-      <c r="N7" s="29"/>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+    </row>
+    <row r="7" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="19"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="B8" s="26"/>
       <c r="C8" s="26"/>
@@ -2208,7 +2080,7 @@
       <c r="G8" s="26"/>
       <c r="H8" s="26"/>
       <c r="I8" s="27" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="J8" s="27"/>
       <c r="K8" s="27"/>
@@ -2216,241 +2088,261 @@
       <c r="M8" s="27"/>
       <c r="N8" s="27"/>
     </row>
-    <row r="10" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
+    <row r="9" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="J9" s="29"/>
+      <c r="K9" s="29"/>
+      <c r="L9" s="29"/>
+      <c r="M9" s="29"/>
+      <c r="N9" s="29"/>
+    </row>
+    <row r="10" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="J10" s="27"/>
+      <c r="K10" s="27"/>
+      <c r="L10" s="27"/>
+      <c r="M10" s="27"/>
+      <c r="N10" s="27"/>
+    </row>
+    <row r="12" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="19"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="19"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="21"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="21"/>
+      <c r="K13" s="21"/>
+      <c r="L13" s="21"/>
+      <c r="M13" s="21"/>
+      <c r="N13" s="21"/>
+    </row>
+    <row r="14" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
-      <c r="N10" s="19"/>
-    </row>
-    <row r="11" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="26" t="s">
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
+      <c r="M14" s="31"/>
+      <c r="N14" s="31"/>
+    </row>
+    <row r="16" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="27" t="s">
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
+    </row>
+    <row r="17" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27"/>
+      <c r="L17" s="27"/>
+      <c r="M17" s="27"/>
+      <c r="N17" s="27"/>
+    </row>
+    <row r="18" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="J18" s="29"/>
+      <c r="K18" s="29"/>
+      <c r="L18" s="29"/>
+      <c r="M18" s="29"/>
+      <c r="N18" s="29"/>
+    </row>
+    <row r="19" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
+      <c r="L19" s="27"/>
+      <c r="M19" s="27"/>
+      <c r="N19" s="27"/>
+    </row>
+    <row r="20" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="J11" s="27"/>
-      <c r="K11" s="27"/>
-      <c r="L11" s="27"/>
-      <c r="M11" s="27"/>
-      <c r="N11" s="27"/>
-    </row>
-    <row r="13" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="19"/>
-      <c r="J13" s="19"/>
-      <c r="K13" s="19"/>
-      <c r="L13" s="19"/>
-      <c r="M13" s="19"/>
-      <c r="N13" s="19"/>
-    </row>
-    <row r="14" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="26" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="27" t="s">
-        <v>37</v>
-      </c>
-      <c r="J14" s="27"/>
-      <c r="K14" s="27"/>
-      <c r="L14" s="27"/>
-      <c r="M14" s="27"/>
-      <c r="N14" s="27"/>
-    </row>
-    <row r="15" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="J15" s="29"/>
-      <c r="K15" s="29"/>
-      <c r="L15" s="29"/>
-      <c r="M15" s="29"/>
-      <c r="N15" s="29"/>
-    </row>
-    <row r="16" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="J16" s="27"/>
-      <c r="K16" s="27"/>
-      <c r="L16" s="27"/>
-      <c r="M16" s="27"/>
-      <c r="N16" s="27"/>
-    </row>
-    <row r="17" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="28" t="s">
+      <c r="J20" s="29"/>
+      <c r="K20" s="29"/>
+      <c r="L20" s="29"/>
+      <c r="M20" s="29"/>
+      <c r="N20" s="29"/>
+    </row>
+    <row r="22" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="29" t="s">
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="19"/>
+      <c r="K22" s="19"/>
+      <c r="L22" s="19"/>
+      <c r="M22" s="19"/>
+      <c r="N22" s="19"/>
+    </row>
+    <row r="23" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="J17" s="29"/>
-      <c r="K17" s="29"/>
-      <c r="L17" s="29"/>
-      <c r="M17" s="29"/>
-      <c r="N17" s="29"/>
-    </row>
-    <row r="19" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="19"/>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="19"/>
-      <c r="N19" s="19"/>
-    </row>
-    <row r="20" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="26" t="s">
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
+      <c r="L23" s="27"/>
+      <c r="M23" s="27"/>
+      <c r="N23" s="27"/>
+    </row>
+    <row r="24" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="26"/>
-      <c r="C20" s="26"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="27" t="s">
+      <c r="B24" s="28"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="28"/>
+      <c r="H24" s="28"/>
+      <c r="I24" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="J20" s="27"/>
-      <c r="K20" s="27"/>
-      <c r="L20" s="27"/>
-      <c r="M20" s="27"/>
-      <c r="N20" s="27"/>
-    </row>
-    <row r="21" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="28"/>
-      <c r="I21" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="J21" s="29"/>
-      <c r="K21" s="29"/>
-      <c r="L21" s="29"/>
-      <c r="M21" s="29"/>
-      <c r="N21" s="29"/>
-    </row>
-    <row r="22" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="B22" s="26"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="26"/>
-      <c r="I22" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="J22" s="27"/>
-      <c r="K22" s="27"/>
-      <c r="L22" s="27"/>
-      <c r="M22" s="27"/>
-      <c r="N22" s="27"/>
-    </row>
-    <row r="24" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="19"/>
-      <c r="I24" s="19"/>
-      <c r="J24" s="19"/>
-      <c r="K24" s="19"/>
-      <c r="L24" s="19"/>
-      <c r="M24" s="19"/>
-      <c r="N24" s="19"/>
+      <c r="J24" s="29"/>
+      <c r="K24" s="29"/>
+      <c r="L24" s="29"/>
+      <c r="M24" s="29"/>
+      <c r="N24" s="29"/>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="26" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="26"/>
@@ -2460,7 +2352,7 @@
       <c r="G25" s="26"/>
       <c r="H25" s="26"/>
       <c r="I25" s="27" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="J25" s="27"/>
       <c r="K25" s="27"/>
@@ -2468,127 +2360,168 @@
       <c r="M25" s="27"/>
       <c r="N25" s="27"/>
     </row>
-    <row r="26" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="B26" s="28"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="28"/>
-      <c r="I26" s="29" t="s">
-        <v>62</v>
-      </c>
-      <c r="J26" s="29"/>
-      <c r="K26" s="29"/>
-      <c r="L26" s="29"/>
-      <c r="M26" s="29"/>
-      <c r="N26" s="29"/>
-    </row>
-    <row r="27" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="26" t="s">
+    <row r="27" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="19"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="19"/>
+      <c r="K27" s="19"/>
+      <c r="L27" s="19"/>
+      <c r="M27" s="19"/>
+      <c r="N27" s="19"/>
+    </row>
+    <row r="28" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28" s="26"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="26"/>
+      <c r="H28" s="26"/>
+      <c r="I28" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="J28" s="27"/>
+      <c r="K28" s="27"/>
+      <c r="L28" s="27"/>
+      <c r="M28" s="27"/>
+      <c r="N28" s="27"/>
+    </row>
+    <row r="29" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="28"/>
+      <c r="I29" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="J29" s="29"/>
+      <c r="K29" s="29"/>
+      <c r="L29" s="29"/>
+      <c r="M29" s="29"/>
+      <c r="N29" s="29"/>
+    </row>
+    <row r="30" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B27" s="26"/>
-      <c r="C27" s="26"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="27" t="s">
-        <v>63</v>
-      </c>
-      <c r="J27" s="27"/>
-      <c r="K27" s="27"/>
-      <c r="L27" s="27"/>
-      <c r="M27" s="27"/>
-      <c r="N27" s="27"/>
-    </row>
-    <row r="28" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="28" t="s">
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="J30" s="27"/>
+      <c r="K30" s="27"/>
+      <c r="L30" s="27"/>
+      <c r="M30" s="27"/>
+      <c r="N30" s="27"/>
+    </row>
+    <row r="31" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="29" t="s">
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="28"/>
+      <c r="I31" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="J28" s="29"/>
-      <c r="K28" s="29"/>
-      <c r="L28" s="29"/>
-      <c r="M28" s="29"/>
-      <c r="N28" s="29"/>
-    </row>
-    <row r="29" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="26" t="s">
+      <c r="J31" s="29"/>
+      <c r="K31" s="29"/>
+      <c r="L31" s="29"/>
+      <c r="M31" s="29"/>
+      <c r="N31" s="29"/>
+    </row>
+    <row r="32" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="27" t="s">
+      <c r="B32" s="26"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="26"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="26"/>
+      <c r="I32" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="J29" s="27"/>
-      <c r="K29" s="27"/>
-      <c r="L29" s="27"/>
-      <c r="M29" s="27"/>
-      <c r="N29" s="27"/>
+      <c r="J32" s="27"/>
+      <c r="K32" s="27"/>
+      <c r="L32" s="27"/>
+      <c r="M32" s="27"/>
+      <c r="N32" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="39">
+  <mergeCells count="42">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A5:N5"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="I6:N6"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="I7:N7"/>
+    <mergeCell ref="A6:N6"/>
+    <mergeCell ref="A7:N7"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="I8:N8"/>
-    <mergeCell ref="A10:N10"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="I11:N11"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="I9:N9"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="I10:N10"/>
+    <mergeCell ref="A12:N12"/>
     <mergeCell ref="A13:N13"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="I14:N14"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="I15:N15"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="I16:N16"/>
+    <mergeCell ref="A16:N16"/>
     <mergeCell ref="A17:H17"/>
     <mergeCell ref="I17:N17"/>
-    <mergeCell ref="A19:N19"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="I18:N18"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="I19:N19"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="I20:N20"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="I21:N21"/>
-    <mergeCell ref="A22:H22"/>
-    <mergeCell ref="I22:N22"/>
-    <mergeCell ref="A24:N24"/>
+    <mergeCell ref="A22:N22"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="I23:N23"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="I24:N24"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="I25:N25"/>
-    <mergeCell ref="A26:H26"/>
-    <mergeCell ref="I26:N26"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="I27:N27"/>
+    <mergeCell ref="A27:N27"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="I28:N28"/>
     <mergeCell ref="A29:H29"/>
     <mergeCell ref="I29:N29"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="I30:N30"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="I31:N31"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="I32:N32"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.25" footer="0.3"/>
@@ -2612,7 +2545,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -2630,7 +2563,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2680,7 +2613,7 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B5" s="21"/>
       <c r="C5" s="21"/>
@@ -2698,7 +2631,7 @@
     </row>
     <row r="7" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="19"/>
@@ -2716,7 +2649,7 @@
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B8" s="26"/>
       <c r="C8" s="26"/>
@@ -2726,7 +2659,7 @@
       <c r="G8" s="26"/>
       <c r="H8" s="26"/>
       <c r="I8" s="27" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="J8" s="27"/>
       <c r="K8" s="27"/>
@@ -2736,7 +2669,7 @@
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B9" s="28"/>
       <c r="C9" s="28"/>
@@ -2746,7 +2679,7 @@
       <c r="G9" s="28"/>
       <c r="H9" s="28"/>
       <c r="I9" s="29" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J9" s="29"/>
       <c r="K9" s="29"/>
@@ -2756,7 +2689,7 @@
     </row>
     <row r="11" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B11" s="19"/>
       <c r="C11" s="19"/>
@@ -2773,88 +2706,88 @@
       <c r="N11" s="19"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B12" s="30"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30" t="s">
+      <c r="H12" s="32"/>
+      <c r="I12" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30" t="s">
+      <c r="J12" s="32"/>
+      <c r="K12" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30" t="s">
+      <c r="L12" s="32"/>
+      <c r="M12" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="J12" s="30"/>
-      <c r="K12" s="30" t="s">
+      <c r="N12" s="32"/>
+    </row>
+    <row r="13" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="L12" s="30"/>
-      <c r="M12" s="30" t="s">
+      <c r="B13" s="33"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="N12" s="30"/>
-    </row>
-    <row r="13" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="31" t="s">
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="B13" s="31"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="32" t="s">
+      <c r="H13" s="33"/>
+      <c r="I13" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="E13" s="32"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="31" t="s">
+      <c r="J13" s="33"/>
+      <c r="K13" s="33" t="s">
         <v>78</v>
       </c>
-      <c r="H13" s="31"/>
-      <c r="I13" s="31" t="s">
+      <c r="L13" s="33"/>
+      <c r="M13" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="N13" s="33"/>
+    </row>
+    <row r="14" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="J13" s="31"/>
-      <c r="K13" s="31" t="s">
+      <c r="B14" s="33"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="L13" s="31"/>
-      <c r="M13" s="31" t="s">
-        <v>78</v>
-      </c>
-      <c r="N13" s="31"/>
-    </row>
-    <row r="14" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="31" t="s">
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="B14" s="31"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="32" t="s">
+      <c r="H14" s="33"/>
+      <c r="I14" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="E14" s="32"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="31" t="s">
+      <c r="J14" s="33"/>
+      <c r="K14" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="31"/>
-      <c r="I14" s="31" t="s">
-        <v>84</v>
-      </c>
-      <c r="J14" s="31"/>
-      <c r="K14" s="31" t="s">
-        <v>85</v>
-      </c>
-      <c r="L14" s="31"/>
-      <c r="M14" s="31" t="s">
-        <v>83</v>
-      </c>
-      <c r="N14" s="31"/>
+      <c r="L14" s="33"/>
+      <c r="M14" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="N14" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="27">
@@ -2908,7 +2841,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -2926,7 +2859,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2960,7 +2893,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -3250,7 +3183,7 @@
     </row>
     <row r="23" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B23" s="19"/>
       <c r="C23" s="19"/>
@@ -3267,388 +3200,388 @@
       <c r="N23" s="19"/>
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="33" t="s">
+      <c r="A24" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="H24" s="36"/>
+      <c r="I24" s="36"/>
+      <c r="J24" s="36" t="s">
+        <v>23</v>
+      </c>
+      <c r="K24" s="36"/>
+      <c r="L24" s="36"/>
+      <c r="M24" s="36"/>
+      <c r="N24" s="36"/>
+    </row>
+    <row r="25" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="B24" s="33"/>
-      <c r="C24" s="33"/>
-      <c r="D24" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="E24" s="34"/>
-      <c r="F24" s="34"/>
-      <c r="G24" s="34" t="s">
-        <v>51</v>
-      </c>
-      <c r="H24" s="34"/>
-      <c r="I24" s="34"/>
-      <c r="J24" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="K24" s="34"/>
-      <c r="L24" s="34"/>
-      <c r="M24" s="34"/>
-      <c r="N24" s="34"/>
-    </row>
-    <row r="25" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="35" t="s">
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
+      <c r="G25" s="37" t="s">
         <v>89</v>
       </c>
-      <c r="B25" s="35"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="35" t="s">
+      <c r="H25" s="37"/>
+      <c r="I25" s="37"/>
+      <c r="J25" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="E25" s="35"/>
-      <c r="F25" s="35"/>
-      <c r="G25" s="35" t="s">
+      <c r="K25" s="38"/>
+      <c r="L25" s="38"/>
+      <c r="M25" s="38"/>
+      <c r="N25" s="38"/>
+    </row>
+    <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="39" t="s">
         <v>91</v>
       </c>
-      <c r="H25" s="35"/>
-      <c r="I25" s="35"/>
-      <c r="J25" s="36" t="s">
+      <c r="B26" s="39"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="39" t="s">
         <v>92</v>
       </c>
-      <c r="K25" s="36"/>
-      <c r="L25" s="36"/>
-      <c r="M25" s="36"/>
-      <c r="N25" s="36"/>
-    </row>
-    <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="37" t="s">
+      <c r="E26" s="39"/>
+      <c r="F26" s="39"/>
+      <c r="G26" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="H26" s="39"/>
+      <c r="I26" s="39"/>
+      <c r="J26" s="40" t="s">
         <v>93</v>
       </c>
-      <c r="B26" s="37"/>
-      <c r="C26" s="37"/>
-      <c r="D26" s="37" t="s">
+      <c r="K26" s="40"/>
+      <c r="L26" s="40"/>
+      <c r="M26" s="40"/>
+      <c r="N26" s="40"/>
+    </row>
+    <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="E26" s="37"/>
-      <c r="F26" s="37"/>
-      <c r="G26" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="H26" s="37"/>
-      <c r="I26" s="37"/>
-      <c r="J26" s="38" t="s">
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="37" t="s">
         <v>95</v>
       </c>
-      <c r="K26" s="38"/>
-      <c r="L26" s="38"/>
-      <c r="M26" s="38"/>
-      <c r="N26" s="38"/>
-    </row>
-    <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="35" t="s">
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="H27" s="37"/>
+      <c r="I27" s="37"/>
+      <c r="J27" s="38" t="s">
         <v>96</v>
       </c>
-      <c r="B27" s="35"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="35" t="s">
+      <c r="K27" s="38"/>
+      <c r="L27" s="38"/>
+      <c r="M27" s="38"/>
+      <c r="N27" s="38"/>
+    </row>
+    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
-      <c r="G27" s="35" t="s">
-        <v>94</v>
-      </c>
-      <c r="H27" s="35"/>
-      <c r="I27" s="35"/>
-      <c r="J27" s="36" t="s">
+      <c r="B28" s="39"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="39" t="s">
         <v>98</v>
       </c>
-      <c r="K27" s="36"/>
-      <c r="L27" s="36"/>
-      <c r="M27" s="36"/>
-      <c r="N27" s="36"/>
-    </row>
-    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="37" t="s">
+      <c r="E28" s="39"/>
+      <c r="F28" s="39"/>
+      <c r="G28" s="39" t="s">
+        <v>95</v>
+      </c>
+      <c r="H28" s="39"/>
+      <c r="I28" s="39"/>
+      <c r="J28" s="40" t="s">
         <v>99</v>
       </c>
-      <c r="B28" s="37"/>
-      <c r="C28" s="37"/>
-      <c r="D28" s="37" t="s">
+      <c r="K28" s="40"/>
+      <c r="L28" s="40"/>
+      <c r="M28" s="40"/>
+      <c r="N28" s="40"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="E28" s="37"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="37" t="s">
-        <v>97</v>
-      </c>
-      <c r="H28" s="37"/>
-      <c r="I28" s="37"/>
-      <c r="J28" s="38" t="s">
+      <c r="B29" s="37"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="E29" s="37"/>
+      <c r="F29" s="37"/>
+      <c r="G29" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="H29" s="37"/>
+      <c r="I29" s="37"/>
+      <c r="J29" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="K28" s="38"/>
-      <c r="L28" s="38"/>
-      <c r="M28" s="38"/>
-      <c r="N28" s="38"/>
-    </row>
-    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="35" t="s">
+      <c r="K29" s="38"/>
+      <c r="L29" s="38"/>
+      <c r="M29" s="38"/>
+      <c r="N29" s="38"/>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="39" t="s">
         <v>102</v>
       </c>
-      <c r="B29" s="35"/>
-      <c r="C29" s="35"/>
-      <c r="D29" s="35" t="s">
-        <v>90</v>
-      </c>
-      <c r="E29" s="35"/>
-      <c r="F29" s="35"/>
-      <c r="G29" s="35" t="s">
-        <v>91</v>
-      </c>
-      <c r="H29" s="35"/>
-      <c r="I29" s="35"/>
-      <c r="J29" s="36" t="s">
+      <c r="B30" s="39"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="E30" s="39"/>
+      <c r="F30" s="39"/>
+      <c r="G30" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="H30" s="39"/>
+      <c r="I30" s="39"/>
+      <c r="J30" s="40" t="s">
         <v>103</v>
       </c>
-      <c r="K29" s="36"/>
-      <c r="L29" s="36"/>
-      <c r="M29" s="36"/>
-      <c r="N29" s="36"/>
-    </row>
-    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="37" t="s">
+      <c r="K30" s="40"/>
+      <c r="L30" s="40"/>
+      <c r="M30" s="40"/>
+      <c r="N30" s="40"/>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="37" t="s">
         <v>104</v>
       </c>
-      <c r="B30" s="37"/>
-      <c r="C30" s="37"/>
-      <c r="D30" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="E30" s="37"/>
-      <c r="F30" s="37"/>
-      <c r="G30" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="H30" s="37"/>
-      <c r="I30" s="37"/>
-      <c r="J30" s="38" t="s">
+      <c r="B31" s="37"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="E31" s="37"/>
+      <c r="F31" s="37"/>
+      <c r="G31" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="H31" s="37"/>
+      <c r="I31" s="37"/>
+      <c r="J31" s="38" t="s">
         <v>105</v>
       </c>
-      <c r="K30" s="38"/>
-      <c r="L30" s="38"/>
-      <c r="M30" s="38"/>
-      <c r="N30" s="38"/>
-    </row>
-    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="35" t="s">
+      <c r="K31" s="38"/>
+      <c r="L31" s="38"/>
+      <c r="M31" s="38"/>
+      <c r="N31" s="38"/>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="B31" s="35"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="35" t="s">
-        <v>97</v>
-      </c>
-      <c r="E31" s="35"/>
-      <c r="F31" s="35"/>
-      <c r="G31" s="35" t="s">
-        <v>94</v>
-      </c>
-      <c r="H31" s="35"/>
-      <c r="I31" s="35"/>
-      <c r="J31" s="36" t="s">
+      <c r="B32" s="39"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="E32" s="39"/>
+      <c r="F32" s="39"/>
+      <c r="G32" s="39" t="s">
+        <v>95</v>
+      </c>
+      <c r="H32" s="39"/>
+      <c r="I32" s="39"/>
+      <c r="J32" s="40" t="s">
         <v>107</v>
       </c>
-      <c r="K31" s="36"/>
-      <c r="L31" s="36"/>
-      <c r="M31" s="36"/>
-      <c r="N31" s="36"/>
-    </row>
-    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="37" t="s">
+      <c r="K32" s="40"/>
+      <c r="L32" s="40"/>
+      <c r="M32" s="40"/>
+      <c r="N32" s="40"/>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="B32" s="37"/>
-      <c r="C32" s="37"/>
-      <c r="D32" s="37" t="s">
-        <v>100</v>
-      </c>
-      <c r="E32" s="37"/>
-      <c r="F32" s="37"/>
-      <c r="G32" s="37" t="s">
-        <v>97</v>
-      </c>
-      <c r="H32" s="37"/>
-      <c r="I32" s="37"/>
-      <c r="J32" s="38" t="s">
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="H33" s="37"/>
+      <c r="I33" s="37"/>
+      <c r="J33" s="38" t="s">
         <v>109</v>
       </c>
-      <c r="K32" s="38"/>
-      <c r="L32" s="38"/>
-      <c r="M32" s="38"/>
-      <c r="N32" s="38"/>
-    </row>
-    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="35" t="s">
+      <c r="K33" s="38"/>
+      <c r="L33" s="38"/>
+      <c r="M33" s="38"/>
+      <c r="N33" s="38"/>
+    </row>
+    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="39" t="s">
         <v>110</v>
       </c>
-      <c r="B33" s="35"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35" t="s">
-        <v>90</v>
-      </c>
-      <c r="E33" s="35"/>
-      <c r="F33" s="35"/>
-      <c r="G33" s="35" t="s">
-        <v>91</v>
-      </c>
-      <c r="H33" s="35"/>
-      <c r="I33" s="35"/>
-      <c r="J33" s="36" t="s">
+      <c r="B34" s="39"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="E34" s="39"/>
+      <c r="F34" s="39"/>
+      <c r="G34" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="H34" s="39"/>
+      <c r="I34" s="39"/>
+      <c r="J34" s="40" t="s">
         <v>111</v>
       </c>
-      <c r="K33" s="36"/>
-      <c r="L33" s="36"/>
-      <c r="M33" s="36"/>
-      <c r="N33" s="36"/>
-    </row>
-    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="37" t="s">
+      <c r="K34" s="40"/>
+      <c r="L34" s="40"/>
+      <c r="M34" s="40"/>
+      <c r="N34" s="40"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="B34" s="37"/>
-      <c r="C34" s="37"/>
-      <c r="D34" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="E34" s="37"/>
-      <c r="F34" s="37"/>
-      <c r="G34" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="H34" s="37"/>
-      <c r="I34" s="37"/>
-      <c r="J34" s="38" t="s">
+      <c r="B35" s="37"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="H35" s="37"/>
+      <c r="I35" s="37"/>
+      <c r="J35" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="K34" s="38"/>
-      <c r="L34" s="38"/>
-      <c r="M34" s="38"/>
-      <c r="N34" s="38"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="35" t="s">
+      <c r="K35" s="38"/>
+      <c r="L35" s="38"/>
+      <c r="M35" s="38"/>
+      <c r="N35" s="38"/>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="39" t="s">
         <v>114</v>
       </c>
-      <c r="B35" s="35"/>
-      <c r="C35" s="35"/>
-      <c r="D35" s="35" t="s">
-        <v>97</v>
-      </c>
-      <c r="E35" s="35"/>
-      <c r="F35" s="35"/>
-      <c r="G35" s="35" t="s">
-        <v>94</v>
-      </c>
-      <c r="H35" s="35"/>
-      <c r="I35" s="35"/>
-      <c r="J35" s="36" t="s">
+      <c r="B36" s="39"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="E36" s="39"/>
+      <c r="F36" s="39"/>
+      <c r="G36" s="39" t="s">
+        <v>95</v>
+      </c>
+      <c r="H36" s="39"/>
+      <c r="I36" s="39"/>
+      <c r="J36" s="40" t="s">
         <v>115</v>
       </c>
-      <c r="K35" s="36"/>
-      <c r="L35" s="36"/>
-      <c r="M35" s="36"/>
-      <c r="N35" s="36"/>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" s="37" t="s">
+      <c r="K36" s="40"/>
+      <c r="L36" s="40"/>
+      <c r="M36" s="40"/>
+      <c r="N36" s="40"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="37" t="s">
         <v>116</v>
       </c>
-      <c r="B36" s="37"/>
-      <c r="C36" s="37"/>
-      <c r="D36" s="37" t="s">
-        <v>100</v>
-      </c>
-      <c r="E36" s="37"/>
-      <c r="F36" s="37"/>
-      <c r="G36" s="37" t="s">
-        <v>97</v>
-      </c>
-      <c r="H36" s="37"/>
-      <c r="I36" s="37"/>
-      <c r="J36" s="38" t="s">
+      <c r="B37" s="37"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="E37" s="37"/>
+      <c r="F37" s="37"/>
+      <c r="G37" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="H37" s="37"/>
+      <c r="I37" s="37"/>
+      <c r="J37" s="38" t="s">
         <v>117</v>
       </c>
-      <c r="K36" s="38"/>
-      <c r="L36" s="38"/>
-      <c r="M36" s="38"/>
-      <c r="N36" s="38"/>
-    </row>
-    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="35" t="s">
+      <c r="K37" s="38"/>
+      <c r="L37" s="38"/>
+      <c r="M37" s="38"/>
+      <c r="N37" s="38"/>
+    </row>
+    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="39" t="s">
         <v>118</v>
       </c>
-      <c r="B37" s="35"/>
-      <c r="C37" s="35"/>
-      <c r="D37" s="35" t="s">
-        <v>90</v>
-      </c>
-      <c r="E37" s="35"/>
-      <c r="F37" s="35"/>
-      <c r="G37" s="35" t="s">
-        <v>91</v>
-      </c>
-      <c r="H37" s="35"/>
-      <c r="I37" s="35"/>
-      <c r="J37" s="36" t="s">
+      <c r="B38" s="39"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="E38" s="39"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="H38" s="39"/>
+      <c r="I38" s="39"/>
+      <c r="J38" s="40" t="s">
         <v>119</v>
       </c>
-      <c r="K37" s="36"/>
-      <c r="L37" s="36"/>
-      <c r="M37" s="36"/>
-      <c r="N37" s="36"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="37" t="s">
-        <v>120</v>
-      </c>
-      <c r="B38" s="37"/>
-      <c r="C38" s="37"/>
-      <c r="D38" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="E38" s="37"/>
-      <c r="F38" s="37"/>
-      <c r="G38" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="H38" s="37"/>
-      <c r="I38" s="37"/>
-      <c r="J38" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="K38" s="38"/>
-      <c r="L38" s="38"/>
-      <c r="M38" s="38"/>
-      <c r="N38" s="38"/>
+      <c r="K38" s="40"/>
+      <c r="L38" s="40"/>
+      <c r="M38" s="40"/>
+      <c r="N38" s="40"/>
     </row>
     <row r="39" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A39" s="39" t="s">
+      <c r="A39" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="B39" s="39"/>
-      <c r="C39" s="39"/>
-      <c r="D39" s="39" t="s">
-        <v>38</v>
-      </c>
-      <c r="E39" s="39"/>
-      <c r="F39" s="39"/>
-      <c r="G39" s="39" t="s">
-        <v>52</v>
-      </c>
-      <c r="H39" s="39"/>
-      <c r="I39" s="39"/>
-      <c r="J39" s="40" t="s">
-        <v>37</v>
-      </c>
-      <c r="K39" s="40"/>
-      <c r="L39" s="40"/>
-      <c r="M39" s="40"/>
-      <c r="N39" s="40"/>
+      <c r="B39" s="41"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="E39" s="41"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="41" t="s">
+        <v>50</v>
+      </c>
+      <c r="H39" s="41"/>
+      <c r="I39" s="41"/>
+      <c r="J39" s="42" t="s">
+        <v>26</v>
+      </c>
+      <c r="K39" s="42"/>
+      <c r="L39" s="42"/>
+      <c r="M39" s="42"/>
+      <c r="N39" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="68">
@@ -3744,7 +3677,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -3762,7 +3695,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3796,7 +3729,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -4102,7 +4035,7 @@
     </row>
     <row r="24" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
@@ -4119,356 +4052,356 @@
       <c r="N24" s="19"/>
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="33" t="s">
+      <c r="A25" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="F25" s="36"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="36"/>
+      <c r="J25" s="36" t="s">
+        <v>40</v>
+      </c>
+      <c r="K25" s="36"/>
+      <c r="L25" s="36"/>
+      <c r="M25" s="36"/>
+      <c r="N25" s="36"/>
+    </row>
+    <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="B26" s="37"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="37"/>
+      <c r="E26" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="F26" s="38"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="38"/>
+      <c r="I26" s="38"/>
+      <c r="J26" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="K26" s="37"/>
+      <c r="L26" s="37"/>
+      <c r="M26" s="37"/>
+      <c r="N26" s="37"/>
+    </row>
+    <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="39" t="s">
+        <v>91</v>
+      </c>
+      <c r="B27" s="39"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="F27" s="40"/>
+      <c r="G27" s="40"/>
+      <c r="H27" s="40"/>
+      <c r="I27" s="40"/>
+      <c r="J27" s="39" t="s">
+        <v>125</v>
+      </c>
+      <c r="K27" s="39"/>
+      <c r="L27" s="39"/>
+      <c r="M27" s="39"/>
+      <c r="N27" s="39"/>
+    </row>
+    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="B28" s="37"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="F28" s="38"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="38"/>
+      <c r="J28" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="K28" s="37"/>
+      <c r="L28" s="37"/>
+      <c r="M28" s="37"/>
+      <c r="N28" s="37"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="B29" s="39"/>
+      <c r="C29" s="39"/>
+      <c r="D29" s="39"/>
+      <c r="E29" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="F29" s="40"/>
+      <c r="G29" s="40"/>
+      <c r="H29" s="40"/>
+      <c r="I29" s="40"/>
+      <c r="J29" s="39" t="s">
         <v>88</v>
       </c>
-      <c r="B25" s="33"/>
-      <c r="C25" s="33"/>
-      <c r="D25" s="33"/>
-      <c r="E25" s="34" t="s">
-        <v>23</v>
-      </c>
-      <c r="F25" s="34"/>
-      <c r="G25" s="34"/>
-      <c r="H25" s="34"/>
-      <c r="I25" s="34"/>
-      <c r="J25" s="34" t="s">
-        <v>24</v>
-      </c>
-      <c r="K25" s="34"/>
-      <c r="L25" s="34"/>
-      <c r="M25" s="34"/>
-      <c r="N25" s="34"/>
-    </row>
-    <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="35" t="s">
+      <c r="K29" s="39"/>
+      <c r="L29" s="39"/>
+      <c r="M29" s="39"/>
+      <c r="N29" s="39"/>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="B30" s="37"/>
+      <c r="C30" s="37"/>
+      <c r="D30" s="37"/>
+      <c r="E30" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="F30" s="38"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="38"/>
+      <c r="J30" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="K30" s="37"/>
+      <c r="L30" s="37"/>
+      <c r="M30" s="37"/>
+      <c r="N30" s="37"/>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="39" t="s">
+        <v>102</v>
+      </c>
+      <c r="B31" s="39"/>
+      <c r="C31" s="39"/>
+      <c r="D31" s="39"/>
+      <c r="E31" s="40" t="s">
+        <v>129</v>
+      </c>
+      <c r="F31" s="40"/>
+      <c r="G31" s="40"/>
+      <c r="H31" s="40"/>
+      <c r="I31" s="40"/>
+      <c r="J31" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="K31" s="39"/>
+      <c r="L31" s="39"/>
+      <c r="M31" s="39"/>
+      <c r="N31" s="39"/>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="37" t="s">
+        <v>104</v>
+      </c>
+      <c r="B32" s="37"/>
+      <c r="C32" s="37"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="F32" s="38"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="38"/>
+      <c r="I32" s="38"/>
+      <c r="J32" s="37" t="s">
+        <v>125</v>
+      </c>
+      <c r="K32" s="37"/>
+      <c r="L32" s="37"/>
+      <c r="M32" s="37"/>
+      <c r="N32" s="37"/>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="B33" s="39"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="39"/>
+      <c r="E33" s="40" t="s">
+        <v>131</v>
+      </c>
+      <c r="F33" s="40"/>
+      <c r="G33" s="40"/>
+      <c r="H33" s="40"/>
+      <c r="I33" s="40"/>
+      <c r="J33" s="39" t="s">
         <v>89</v>
       </c>
-      <c r="B26" s="35"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="35"/>
-      <c r="E26" s="36" t="s">
+      <c r="K33" s="39"/>
+      <c r="L33" s="39"/>
+      <c r="M33" s="39"/>
+      <c r="N33" s="39"/>
+    </row>
+    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="B34" s="37"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
+      <c r="I34" s="38"/>
+      <c r="J34" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="K34" s="37"/>
+      <c r="L34" s="37"/>
+      <c r="M34" s="37"/>
+      <c r="N34" s="37"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="B35" s="39"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="39"/>
+      <c r="E35" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="F35" s="40"/>
+      <c r="G35" s="40"/>
+      <c r="H35" s="40"/>
+      <c r="I35" s="40"/>
+      <c r="J35" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="K35" s="39"/>
+      <c r="L35" s="39"/>
+      <c r="M35" s="39"/>
+      <c r="N35" s="39"/>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="B36" s="37"/>
+      <c r="C36" s="37"/>
+      <c r="D36" s="37"/>
+      <c r="E36" s="38" t="s">
+        <v>133</v>
+      </c>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="38"/>
+      <c r="J36" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="K36" s="37"/>
+      <c r="L36" s="37"/>
+      <c r="M36" s="37"/>
+      <c r="N36" s="37"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="39" t="s">
+        <v>114</v>
+      </c>
+      <c r="B37" s="39"/>
+      <c r="C37" s="39"/>
+      <c r="D37" s="39"/>
+      <c r="E37" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="F37" s="40"/>
+      <c r="G37" s="40"/>
+      <c r="H37" s="40"/>
+      <c r="I37" s="40"/>
+      <c r="J37" s="39" t="s">
         <v>125</v>
       </c>
-      <c r="F26" s="36"/>
-      <c r="G26" s="36"/>
-      <c r="H26" s="36"/>
-      <c r="I26" s="36"/>
-      <c r="J26" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="K26" s="35"/>
-      <c r="L26" s="35"/>
-      <c r="M26" s="35"/>
-      <c r="N26" s="35"/>
-    </row>
-    <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="37" t="s">
-        <v>93</v>
-      </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="37"/>
-      <c r="D27" s="37"/>
-      <c r="E27" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="F27" s="38"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="38"/>
-      <c r="I27" s="38"/>
-      <c r="J27" s="37" t="s">
-        <v>127</v>
-      </c>
-      <c r="K27" s="37"/>
-      <c r="L27" s="37"/>
-      <c r="M27" s="37"/>
-      <c r="N27" s="37"/>
-    </row>
-    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="35" t="s">
-        <v>96</v>
-      </c>
-      <c r="B28" s="35"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="35"/>
-      <c r="E28" s="36" t="s">
-        <v>128</v>
-      </c>
-      <c r="F28" s="36"/>
-      <c r="G28" s="36"/>
-      <c r="H28" s="36"/>
-      <c r="I28" s="36"/>
-      <c r="J28" s="35" t="s">
-        <v>91</v>
-      </c>
-      <c r="K28" s="35"/>
-      <c r="L28" s="35"/>
-      <c r="M28" s="35"/>
-      <c r="N28" s="35"/>
-    </row>
-    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="37" t="s">
-        <v>99</v>
-      </c>
-      <c r="B29" s="37"/>
-      <c r="C29" s="37"/>
-      <c r="D29" s="37"/>
-      <c r="E29" s="38" t="s">
-        <v>129</v>
-      </c>
-      <c r="F29" s="38"/>
-      <c r="G29" s="38"/>
-      <c r="H29" s="38"/>
-      <c r="I29" s="38"/>
-      <c r="J29" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="K29" s="37"/>
-      <c r="L29" s="37"/>
-      <c r="M29" s="37"/>
-      <c r="N29" s="37"/>
-    </row>
-    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="35" t="s">
-        <v>102</v>
-      </c>
-      <c r="B30" s="35"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="36" t="s">
-        <v>130</v>
-      </c>
-      <c r="F30" s="36"/>
-      <c r="G30" s="36"/>
-      <c r="H30" s="36"/>
-      <c r="I30" s="36"/>
-      <c r="J30" s="35" t="s">
-        <v>94</v>
-      </c>
-      <c r="K30" s="35"/>
-      <c r="L30" s="35"/>
-      <c r="M30" s="35"/>
-      <c r="N30" s="35"/>
-    </row>
-    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="37" t="s">
-        <v>104</v>
-      </c>
-      <c r="B31" s="37"/>
-      <c r="C31" s="37"/>
-      <c r="D31" s="37"/>
-      <c r="E31" s="38" t="s">
-        <v>131</v>
-      </c>
-      <c r="F31" s="38"/>
-      <c r="G31" s="38"/>
-      <c r="H31" s="38"/>
-      <c r="I31" s="38"/>
-      <c r="J31" s="37" t="s">
-        <v>55</v>
-      </c>
-      <c r="K31" s="37"/>
-      <c r="L31" s="37"/>
-      <c r="M31" s="37"/>
-      <c r="N31" s="37"/>
-    </row>
-    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="35" t="s">
-        <v>106</v>
-      </c>
-      <c r="B32" s="35"/>
-      <c r="C32" s="35"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="36" t="s">
-        <v>132</v>
-      </c>
-      <c r="F32" s="36"/>
-      <c r="G32" s="36"/>
-      <c r="H32" s="36"/>
-      <c r="I32" s="36"/>
-      <c r="J32" s="35" t="s">
-        <v>127</v>
-      </c>
-      <c r="K32" s="35"/>
-      <c r="L32" s="35"/>
-      <c r="M32" s="35"/>
-      <c r="N32" s="35"/>
-    </row>
-    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="37" t="s">
-        <v>108</v>
-      </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="F33" s="38"/>
-      <c r="G33" s="38"/>
-      <c r="H33" s="38"/>
-      <c r="I33" s="38"/>
-      <c r="J33" s="37" t="s">
-        <v>91</v>
-      </c>
-      <c r="K33" s="37"/>
-      <c r="L33" s="37"/>
-      <c r="M33" s="37"/>
-      <c r="N33" s="37"/>
-    </row>
-    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="35" t="s">
-        <v>110</v>
-      </c>
-      <c r="B34" s="35"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="35"/>
-      <c r="E34" s="36" t="s">
-        <v>92</v>
-      </c>
-      <c r="F34" s="36"/>
-      <c r="G34" s="36"/>
-      <c r="H34" s="36"/>
-      <c r="I34" s="36"/>
-      <c r="J34" s="35" t="s">
-        <v>90</v>
-      </c>
-      <c r="K34" s="35"/>
-      <c r="L34" s="35"/>
-      <c r="M34" s="35"/>
-      <c r="N34" s="35"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="37" t="s">
-        <v>112</v>
-      </c>
-      <c r="B35" s="37"/>
-      <c r="C35" s="37"/>
-      <c r="D35" s="37"/>
-      <c r="E35" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="F35" s="38"/>
-      <c r="G35" s="38"/>
-      <c r="H35" s="38"/>
-      <c r="I35" s="38"/>
-      <c r="J35" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="K35" s="37"/>
-      <c r="L35" s="37"/>
-      <c r="M35" s="37"/>
-      <c r="N35" s="37"/>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" s="35" t="s">
-        <v>114</v>
-      </c>
-      <c r="B36" s="35"/>
-      <c r="C36" s="35"/>
-      <c r="D36" s="35"/>
-      <c r="E36" s="36" t="s">
+      <c r="K37" s="39"/>
+      <c r="L37" s="39"/>
+      <c r="M37" s="39"/>
+      <c r="N37" s="39"/>
+    </row>
+    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="37" t="s">
+        <v>116</v>
+      </c>
+      <c r="B38" s="37"/>
+      <c r="C38" s="37"/>
+      <c r="D38" s="37"/>
+      <c r="E38" s="38" t="s">
         <v>135</v>
       </c>
-      <c r="F36" s="36"/>
-      <c r="G36" s="36"/>
-      <c r="H36" s="36"/>
-      <c r="I36" s="36"/>
-      <c r="J36" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="K36" s="35"/>
-      <c r="L36" s="35"/>
-      <c r="M36" s="35"/>
-      <c r="N36" s="35"/>
-    </row>
-    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="B37" s="37"/>
-      <c r="C37" s="37"/>
-      <c r="D37" s="37"/>
-      <c r="E37" s="38" t="s">
+      <c r="F38" s="38"/>
+      <c r="G38" s="38"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="38"/>
+      <c r="J38" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="K38" s="37"/>
+      <c r="L38" s="37"/>
+      <c r="M38" s="37"/>
+      <c r="N38" s="37"/>
+    </row>
+    <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" s="39" t="s">
+        <v>118</v>
+      </c>
+      <c r="B39" s="39"/>
+      <c r="C39" s="39"/>
+      <c r="D39" s="39"/>
+      <c r="E39" s="40" t="s">
         <v>136</v>
       </c>
-      <c r="F37" s="38"/>
-      <c r="G37" s="38"/>
-      <c r="H37" s="38"/>
-      <c r="I37" s="38"/>
-      <c r="J37" s="37" t="s">
-        <v>127</v>
-      </c>
-      <c r="K37" s="37"/>
-      <c r="L37" s="37"/>
-      <c r="M37" s="37"/>
-      <c r="N37" s="37"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="35" t="s">
-        <v>118</v>
-      </c>
-      <c r="B38" s="35"/>
-      <c r="C38" s="35"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="36" t="s">
-        <v>137</v>
-      </c>
-      <c r="F38" s="36"/>
-      <c r="G38" s="36"/>
-      <c r="H38" s="36"/>
-      <c r="I38" s="36"/>
-      <c r="J38" s="35" t="s">
-        <v>91</v>
-      </c>
-      <c r="K38" s="35"/>
-      <c r="L38" s="35"/>
-      <c r="M38" s="35"/>
-      <c r="N38" s="35"/>
-    </row>
-    <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A39" s="37" t="s">
-        <v>120</v>
-      </c>
-      <c r="B39" s="37"/>
-      <c r="C39" s="37"/>
-      <c r="D39" s="37"/>
-      <c r="E39" s="38" t="s">
-        <v>138</v>
-      </c>
-      <c r="F39" s="38"/>
-      <c r="G39" s="38"/>
-      <c r="H39" s="38"/>
-      <c r="I39" s="38"/>
-      <c r="J39" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="K39" s="37"/>
-      <c r="L39" s="37"/>
-      <c r="M39" s="37"/>
-      <c r="N39" s="37"/>
+      <c r="F39" s="40"/>
+      <c r="G39" s="40"/>
+      <c r="H39" s="40"/>
+      <c r="I39" s="40"/>
+      <c r="J39" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="K39" s="39"/>
+      <c r="L39" s="39"/>
+      <c r="M39" s="39"/>
+      <c r="N39" s="39"/>
     </row>
     <row r="40" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A40" s="39" t="s">
+      <c r="A40" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="B40" s="39"/>
-      <c r="C40" s="39"/>
-      <c r="D40" s="39"/>
-      <c r="E40" s="40" t="s">
-        <v>26</v>
-      </c>
-      <c r="F40" s="40"/>
-      <c r="G40" s="40"/>
-      <c r="H40" s="40"/>
-      <c r="I40" s="40"/>
-      <c r="J40" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="K40" s="39"/>
-      <c r="L40" s="39"/>
-      <c r="M40" s="39"/>
-      <c r="N40" s="39"/>
+      <c r="B40" s="41"/>
+      <c r="C40" s="41"/>
+      <c r="D40" s="41"/>
+      <c r="E40" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="F40" s="42"/>
+      <c r="G40" s="42"/>
+      <c r="H40" s="42"/>
+      <c r="I40" s="42"/>
+      <c r="J40" s="41" t="s">
+        <v>41</v>
+      </c>
+      <c r="K40" s="41"/>
+      <c r="L40" s="41"/>
+      <c r="M40" s="41"/>
+      <c r="N40" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="52">

</xml_diff>

<commit_message>
refactor(reporting): unify payment method presentation
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="146">
   <si>
     <t>MINEUQR</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>18 Jul 2026, 22:35</t>
+    <t>18 Jul 2026, 22:52</t>
   </si>
   <si>
     <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Payment Method Analysis  ·  Order Sales  ·  Check Revenue Trends</t>
@@ -72,7 +72,7 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 22:35</t>
+    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 22:52</t>
   </si>
   <si>
     <t>AT A GLANCE</t>
@@ -153,7 +153,7 @@
     <t>TAX</t>
   </si>
   <si>
-    <t>Tax Collected is the total tax from all paid checks in this reporting period (not a subset of sections).</t>
+    <t>Tax Collected covers the full reporting period — total tax from all paid checks in range (not a subset of sections).</t>
   </si>
   <si>
     <t>Tax Collected</t>
@@ -268,6 +268,33 @@
   </si>
   <si>
     <t>60.00%</t>
+  </si>
+  <si>
+    <t>Visa</t>
+  </si>
+  <si>
+    <t>0.00 ر.س</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0.00%</t>
+  </si>
+  <si>
+    <t>Mastercard</t>
+  </si>
+  <si>
+    <t>Apple Pay</t>
+  </si>
+  <si>
+    <t>STC Pay</t>
+  </si>
+  <si>
+    <t>Bank Transfer</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
   <si>
     <t>Monthly Report  ·  Daily Order Sales — July 2026</t>
@@ -667,7 +694,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -757,6 +784,8 @@
     <xf numFmtId="49" fontId="20" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="21" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="21" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="9" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="22" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
     </xf>
@@ -2537,7 +2566,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="10.2" customWidth="1"/>
@@ -2789,8 +2818,176 @@
       </c>
       <c r="N14" s="33"/>
     </row>
+    <row r="15" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="35" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="36" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="H15" s="35"/>
+      <c r="I15" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="J15" s="35"/>
+      <c r="K15" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="L15" s="35"/>
+      <c r="M15" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="N15" s="35"/>
+    </row>
+    <row r="16" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="35" t="s">
+        <v>88</v>
+      </c>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="36" t="s">
+        <v>85</v>
+      </c>
+      <c r="E16" s="36"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="H16" s="35"/>
+      <c r="I16" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="J16" s="35"/>
+      <c r="K16" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="L16" s="35"/>
+      <c r="M16" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="N16" s="35"/>
+    </row>
+    <row r="17" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="35" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="36" t="s">
+        <v>85</v>
+      </c>
+      <c r="E17" s="36"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="H17" s="35"/>
+      <c r="I17" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="J17" s="35"/>
+      <c r="K17" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="L17" s="35"/>
+      <c r="M17" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="N17" s="35"/>
+    </row>
+    <row r="18" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="36" t="s">
+        <v>85</v>
+      </c>
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="H18" s="35"/>
+      <c r="I18" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="J18" s="35"/>
+      <c r="K18" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="L18" s="35"/>
+      <c r="M18" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="N18" s="35"/>
+    </row>
+    <row r="19" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="36" t="s">
+        <v>85</v>
+      </c>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="H19" s="35"/>
+      <c r="I19" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="J19" s="35"/>
+      <c r="K19" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="L19" s="35"/>
+      <c r="M19" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="N19" s="35"/>
+    </row>
+    <row r="20" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="36" t="s">
+        <v>85</v>
+      </c>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="H20" s="35"/>
+      <c r="I20" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="J20" s="35"/>
+      <c r="K20" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="L20" s="35"/>
+      <c r="M20" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="N20" s="35"/>
+    </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="63">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A5:N5"/>
@@ -2818,6 +3015,42 @@
     <mergeCell ref="I14:J14"/>
     <mergeCell ref="K14:L14"/>
     <mergeCell ref="M14:N14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="M20:N20"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.25" footer="0.3"/>
@@ -2859,7 +3092,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2893,7 +3126,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -3200,388 +3433,388 @@
       <c r="N23" s="19"/>
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="36" t="s">
+      <c r="A24" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="36" t="s">
+      <c r="E24" s="38"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="H24" s="36"/>
-      <c r="I24" s="36"/>
-      <c r="J24" s="36" t="s">
+      <c r="H24" s="38"/>
+      <c r="I24" s="38"/>
+      <c r="J24" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="K24" s="36"/>
-      <c r="L24" s="36"/>
-      <c r="M24" s="36"/>
-      <c r="N24" s="36"/>
+      <c r="K24" s="38"/>
+      <c r="L24" s="38"/>
+      <c r="M24" s="38"/>
+      <c r="N24" s="38"/>
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="37" t="s">
-        <v>87</v>
-      </c>
-      <c r="B25" s="37"/>
-      <c r="C25" s="37"/>
-      <c r="D25" s="37" t="s">
-        <v>88</v>
-      </c>
-      <c r="E25" s="37"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="H25" s="37"/>
-      <c r="I25" s="37"/>
-      <c r="J25" s="38" t="s">
-        <v>90</v>
-      </c>
-      <c r="K25" s="38"/>
-      <c r="L25" s="38"/>
-      <c r="M25" s="38"/>
-      <c r="N25" s="38"/>
+      <c r="A25" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="B25" s="39"/>
+      <c r="C25" s="39"/>
+      <c r="D25" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="E25" s="39"/>
+      <c r="F25" s="39"/>
+      <c r="G25" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="H25" s="39"/>
+      <c r="I25" s="39"/>
+      <c r="J25" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="K25" s="40"/>
+      <c r="L25" s="40"/>
+      <c r="M25" s="40"/>
+      <c r="N25" s="40"/>
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="39" t="s">
-        <v>91</v>
-      </c>
-      <c r="B26" s="39"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39" t="s">
-        <v>92</v>
-      </c>
-      <c r="E26" s="39"/>
-      <c r="F26" s="39"/>
-      <c r="G26" s="39" t="s">
-        <v>88</v>
-      </c>
-      <c r="H26" s="39"/>
-      <c r="I26" s="39"/>
-      <c r="J26" s="40" t="s">
-        <v>93</v>
-      </c>
-      <c r="K26" s="40"/>
-      <c r="L26" s="40"/>
-      <c r="M26" s="40"/>
-      <c r="N26" s="40"/>
+      <c r="A26" s="41" t="s">
+        <v>100</v>
+      </c>
+      <c r="B26" s="41"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="E26" s="41"/>
+      <c r="F26" s="41"/>
+      <c r="G26" s="41" t="s">
+        <v>97</v>
+      </c>
+      <c r="H26" s="41"/>
+      <c r="I26" s="41"/>
+      <c r="J26" s="42" t="s">
+        <v>102</v>
+      </c>
+      <c r="K26" s="42"/>
+      <c r="L26" s="42"/>
+      <c r="M26" s="42"/>
+      <c r="N26" s="42"/>
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="37"/>
-      <c r="D27" s="37" t="s">
-        <v>95</v>
-      </c>
-      <c r="E27" s="37"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="37" t="s">
-        <v>92</v>
-      </c>
-      <c r="H27" s="37"/>
-      <c r="I27" s="37"/>
-      <c r="J27" s="38" t="s">
-        <v>96</v>
-      </c>
-      <c r="K27" s="38"/>
-      <c r="L27" s="38"/>
-      <c r="M27" s="38"/>
-      <c r="N27" s="38"/>
+      <c r="A27" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="B27" s="39"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="39" t="s">
+        <v>104</v>
+      </c>
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
+      <c r="G27" s="39" t="s">
+        <v>101</v>
+      </c>
+      <c r="H27" s="39"/>
+      <c r="I27" s="39"/>
+      <c r="J27" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="K27" s="40"/>
+      <c r="L27" s="40"/>
+      <c r="M27" s="40"/>
+      <c r="N27" s="40"/>
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="39" t="s">
+      <c r="A28" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="B28" s="41"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="E28" s="41"/>
+      <c r="F28" s="41"/>
+      <c r="G28" s="41" t="s">
+        <v>104</v>
+      </c>
+      <c r="H28" s="41"/>
+      <c r="I28" s="41"/>
+      <c r="J28" s="42" t="s">
+        <v>108</v>
+      </c>
+      <c r="K28" s="42"/>
+      <c r="L28" s="42"/>
+      <c r="M28" s="42"/>
+      <c r="N28" s="42"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="B29" s="39"/>
+      <c r="C29" s="39"/>
+      <c r="D29" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="B28" s="39"/>
-      <c r="C28" s="39"/>
-      <c r="D28" s="39" t="s">
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39" t="s">
         <v>98</v>
       </c>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39" t="s">
-        <v>95</v>
-      </c>
-      <c r="H28" s="39"/>
-      <c r="I28" s="39"/>
-      <c r="J28" s="40" t="s">
-        <v>99</v>
-      </c>
-      <c r="K28" s="40"/>
-      <c r="L28" s="40"/>
-      <c r="M28" s="40"/>
-      <c r="N28" s="40"/>
-    </row>
-    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="37" t="s">
-        <v>100</v>
-      </c>
-      <c r="B29" s="37"/>
-      <c r="C29" s="37"/>
-      <c r="D29" s="37" t="s">
-        <v>88</v>
-      </c>
-      <c r="E29" s="37"/>
-      <c r="F29" s="37"/>
-      <c r="G29" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="H29" s="37"/>
-      <c r="I29" s="37"/>
-      <c r="J29" s="38" t="s">
+      <c r="H29" s="39"/>
+      <c r="I29" s="39"/>
+      <c r="J29" s="40" t="s">
+        <v>110</v>
+      </c>
+      <c r="K29" s="40"/>
+      <c r="L29" s="40"/>
+      <c r="M29" s="40"/>
+      <c r="N29" s="40"/>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="41" t="s">
+        <v>111</v>
+      </c>
+      <c r="B30" s="41"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41" t="s">
         <v>101</v>
       </c>
-      <c r="K29" s="38"/>
-      <c r="L29" s="38"/>
-      <c r="M29" s="38"/>
-      <c r="N29" s="38"/>
-    </row>
-    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="B30" s="39"/>
-      <c r="C30" s="39"/>
-      <c r="D30" s="39" t="s">
-        <v>92</v>
-      </c>
-      <c r="E30" s="39"/>
-      <c r="F30" s="39"/>
-      <c r="G30" s="39" t="s">
-        <v>88</v>
-      </c>
-      <c r="H30" s="39"/>
-      <c r="I30" s="39"/>
-      <c r="J30" s="40" t="s">
-        <v>103</v>
-      </c>
-      <c r="K30" s="40"/>
-      <c r="L30" s="40"/>
-      <c r="M30" s="40"/>
-      <c r="N30" s="40"/>
+      <c r="E30" s="41"/>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41" t="s">
+        <v>97</v>
+      </c>
+      <c r="H30" s="41"/>
+      <c r="I30" s="41"/>
+      <c r="J30" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="K30" s="42"/>
+      <c r="L30" s="42"/>
+      <c r="M30" s="42"/>
+      <c r="N30" s="42"/>
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="37" t="s">
+      <c r="A31" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="B31" s="39"/>
+      <c r="C31" s="39"/>
+      <c r="D31" s="39" t="s">
         <v>104</v>
       </c>
-      <c r="B31" s="37"/>
-      <c r="C31" s="37"/>
-      <c r="D31" s="37" t="s">
-        <v>95</v>
-      </c>
-      <c r="E31" s="37"/>
-      <c r="F31" s="37"/>
-      <c r="G31" s="37" t="s">
-        <v>92</v>
-      </c>
-      <c r="H31" s="37"/>
-      <c r="I31" s="37"/>
-      <c r="J31" s="38" t="s">
-        <v>105</v>
-      </c>
-      <c r="K31" s="38"/>
-      <c r="L31" s="38"/>
-      <c r="M31" s="38"/>
-      <c r="N31" s="38"/>
+      <c r="E31" s="39"/>
+      <c r="F31" s="39"/>
+      <c r="G31" s="39" t="s">
+        <v>101</v>
+      </c>
+      <c r="H31" s="39"/>
+      <c r="I31" s="39"/>
+      <c r="J31" s="40" t="s">
+        <v>114</v>
+      </c>
+      <c r="K31" s="40"/>
+      <c r="L31" s="40"/>
+      <c r="M31" s="40"/>
+      <c r="N31" s="40"/>
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="39" t="s">
-        <v>106</v>
-      </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39" t="s">
+      <c r="A32" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="B32" s="41"/>
+      <c r="C32" s="41"/>
+      <c r="D32" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="E32" s="41"/>
+      <c r="F32" s="41"/>
+      <c r="G32" s="41" t="s">
+        <v>104</v>
+      </c>
+      <c r="H32" s="41"/>
+      <c r="I32" s="41"/>
+      <c r="J32" s="42" t="s">
+        <v>116</v>
+      </c>
+      <c r="K32" s="42"/>
+      <c r="L32" s="42"/>
+      <c r="M32" s="42"/>
+      <c r="N32" s="42"/>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="B33" s="39"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="E33" s="39"/>
+      <c r="F33" s="39"/>
+      <c r="G33" s="39" t="s">
         <v>98</v>
       </c>
-      <c r="E32" s="39"/>
-      <c r="F32" s="39"/>
-      <c r="G32" s="39" t="s">
-        <v>95</v>
-      </c>
-      <c r="H32" s="39"/>
-      <c r="I32" s="39"/>
-      <c r="J32" s="40" t="s">
+      <c r="H33" s="39"/>
+      <c r="I33" s="39"/>
+      <c r="J33" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="K33" s="40"/>
+      <c r="L33" s="40"/>
+      <c r="M33" s="40"/>
+      <c r="N33" s="40"/>
+    </row>
+    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="41" t="s">
+        <v>119</v>
+      </c>
+      <c r="B34" s="41"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="E34" s="41"/>
+      <c r="F34" s="41"/>
+      <c r="G34" s="41" t="s">
+        <v>97</v>
+      </c>
+      <c r="H34" s="41"/>
+      <c r="I34" s="41"/>
+      <c r="J34" s="42" t="s">
+        <v>120</v>
+      </c>
+      <c r="K34" s="42"/>
+      <c r="L34" s="42"/>
+      <c r="M34" s="42"/>
+      <c r="N34" s="42"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="39" t="s">
+        <v>121</v>
+      </c>
+      <c r="B35" s="39"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="39" t="s">
+        <v>104</v>
+      </c>
+      <c r="E35" s="39"/>
+      <c r="F35" s="39"/>
+      <c r="G35" s="39" t="s">
+        <v>101</v>
+      </c>
+      <c r="H35" s="39"/>
+      <c r="I35" s="39"/>
+      <c r="J35" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="K35" s="40"/>
+      <c r="L35" s="40"/>
+      <c r="M35" s="40"/>
+      <c r="N35" s="40"/>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="41" t="s">
+        <v>123</v>
+      </c>
+      <c r="B36" s="41"/>
+      <c r="C36" s="41"/>
+      <c r="D36" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="K32" s="40"/>
-      <c r="L32" s="40"/>
-      <c r="M32" s="40"/>
-      <c r="N32" s="40"/>
-    </row>
-    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="37" t="s">
-        <v>108</v>
-      </c>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37" t="s">
-        <v>88</v>
-      </c>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="H33" s="37"/>
-      <c r="I33" s="37"/>
-      <c r="J33" s="38" t="s">
-        <v>109</v>
-      </c>
-      <c r="K33" s="38"/>
-      <c r="L33" s="38"/>
-      <c r="M33" s="38"/>
-      <c r="N33" s="38"/>
-    </row>
-    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="39" t="s">
-        <v>110</v>
-      </c>
-      <c r="B34" s="39"/>
-      <c r="C34" s="39"/>
-      <c r="D34" s="39" t="s">
-        <v>92</v>
-      </c>
-      <c r="E34" s="39"/>
-      <c r="F34" s="39"/>
-      <c r="G34" s="39" t="s">
-        <v>88</v>
-      </c>
-      <c r="H34" s="39"/>
-      <c r="I34" s="39"/>
-      <c r="J34" s="40" t="s">
-        <v>111</v>
-      </c>
-      <c r="K34" s="40"/>
-      <c r="L34" s="40"/>
-      <c r="M34" s="40"/>
-      <c r="N34" s="40"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="37" t="s">
-        <v>112</v>
-      </c>
-      <c r="B35" s="37"/>
-      <c r="C35" s="37"/>
-      <c r="D35" s="37" t="s">
-        <v>95</v>
-      </c>
-      <c r="E35" s="37"/>
-      <c r="F35" s="37"/>
-      <c r="G35" s="37" t="s">
-        <v>92</v>
-      </c>
-      <c r="H35" s="37"/>
-      <c r="I35" s="37"/>
-      <c r="J35" s="38" t="s">
-        <v>113</v>
-      </c>
-      <c r="K35" s="38"/>
-      <c r="L35" s="38"/>
-      <c r="M35" s="38"/>
-      <c r="N35" s="38"/>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" s="39" t="s">
-        <v>114</v>
-      </c>
-      <c r="B36" s="39"/>
-      <c r="C36" s="39"/>
-      <c r="D36" s="39" t="s">
+      <c r="E36" s="41"/>
+      <c r="F36" s="41"/>
+      <c r="G36" s="41" t="s">
+        <v>104</v>
+      </c>
+      <c r="H36" s="41"/>
+      <c r="I36" s="41"/>
+      <c r="J36" s="42" t="s">
+        <v>124</v>
+      </c>
+      <c r="K36" s="42"/>
+      <c r="L36" s="42"/>
+      <c r="M36" s="42"/>
+      <c r="N36" s="42"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="39" t="s">
+        <v>125</v>
+      </c>
+      <c r="B37" s="39"/>
+      <c r="C37" s="39"/>
+      <c r="D37" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39" t="s">
         <v>98</v>
       </c>
-      <c r="E36" s="39"/>
-      <c r="F36" s="39"/>
-      <c r="G36" s="39" t="s">
-        <v>95</v>
-      </c>
-      <c r="H36" s="39"/>
-      <c r="I36" s="39"/>
-      <c r="J36" s="40" t="s">
-        <v>115</v>
-      </c>
-      <c r="K36" s="40"/>
-      <c r="L36" s="40"/>
-      <c r="M36" s="40"/>
-      <c r="N36" s="40"/>
-    </row>
-    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="B37" s="37"/>
-      <c r="C37" s="37"/>
-      <c r="D37" s="37" t="s">
-        <v>88</v>
-      </c>
-      <c r="E37" s="37"/>
-      <c r="F37" s="37"/>
-      <c r="G37" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="H37" s="37"/>
-      <c r="I37" s="37"/>
-      <c r="J37" s="38" t="s">
-        <v>117</v>
-      </c>
-      <c r="K37" s="38"/>
-      <c r="L37" s="38"/>
-      <c r="M37" s="38"/>
-      <c r="N37" s="38"/>
+      <c r="H37" s="39"/>
+      <c r="I37" s="39"/>
+      <c r="J37" s="40" t="s">
+        <v>126</v>
+      </c>
+      <c r="K37" s="40"/>
+      <c r="L37" s="40"/>
+      <c r="M37" s="40"/>
+      <c r="N37" s="40"/>
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="39" t="s">
-        <v>118</v>
-      </c>
-      <c r="B38" s="39"/>
-      <c r="C38" s="39"/>
-      <c r="D38" s="39" t="s">
-        <v>92</v>
-      </c>
-      <c r="E38" s="39"/>
-      <c r="F38" s="39"/>
-      <c r="G38" s="39" t="s">
-        <v>88</v>
-      </c>
-      <c r="H38" s="39"/>
-      <c r="I38" s="39"/>
-      <c r="J38" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="K38" s="40"/>
-      <c r="L38" s="40"/>
-      <c r="M38" s="40"/>
-      <c r="N38" s="40"/>
+      <c r="A38" s="41" t="s">
+        <v>127</v>
+      </c>
+      <c r="B38" s="41"/>
+      <c r="C38" s="41"/>
+      <c r="D38" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="E38" s="41"/>
+      <c r="F38" s="41"/>
+      <c r="G38" s="41" t="s">
+        <v>97</v>
+      </c>
+      <c r="H38" s="41"/>
+      <c r="I38" s="41"/>
+      <c r="J38" s="42" t="s">
+        <v>128</v>
+      </c>
+      <c r="K38" s="42"/>
+      <c r="L38" s="42"/>
+      <c r="M38" s="42"/>
+      <c r="N38" s="42"/>
     </row>
     <row r="39" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A39" s="41" t="s">
+      <c r="A39" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="B39" s="41"/>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41" t="s">
+      <c r="B39" s="43"/>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41" t="s">
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43" t="s">
         <v>50</v>
       </c>
-      <c r="H39" s="41"/>
-      <c r="I39" s="41"/>
-      <c r="J39" s="42" t="s">
+      <c r="H39" s="43"/>
+      <c r="I39" s="43"/>
+      <c r="J39" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="K39" s="42"/>
-      <c r="L39" s="42"/>
-      <c r="M39" s="42"/>
-      <c r="N39" s="42"/>
+      <c r="K39" s="44"/>
+      <c r="L39" s="44"/>
+      <c r="M39" s="44"/>
+      <c r="N39" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="68">
@@ -3677,7 +3910,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -3695,7 +3928,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3729,7 +3962,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -4052,356 +4285,356 @@
       <c r="N24" s="19"/>
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="B25" s="35"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="35"/>
-      <c r="E25" s="36" t="s">
+      <c r="A25" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="F25" s="36"/>
-      <c r="G25" s="36"/>
-      <c r="H25" s="36"/>
-      <c r="I25" s="36"/>
-      <c r="J25" s="36" t="s">
+      <c r="F25" s="38"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="38"/>
+      <c r="I25" s="38"/>
+      <c r="J25" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="K25" s="36"/>
-      <c r="L25" s="36"/>
-      <c r="M25" s="36"/>
-      <c r="N25" s="36"/>
+      <c r="K25" s="38"/>
+      <c r="L25" s="38"/>
+      <c r="M25" s="38"/>
+      <c r="N25" s="38"/>
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="37" t="s">
-        <v>87</v>
-      </c>
-      <c r="B26" s="37"/>
-      <c r="C26" s="37"/>
-      <c r="D26" s="37"/>
-      <c r="E26" s="38" t="s">
+      <c r="A26" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" s="39"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="39"/>
+      <c r="E26" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="40"/>
+      <c r="I26" s="40"/>
+      <c r="J26" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="K26" s="39"/>
+      <c r="L26" s="39"/>
+      <c r="M26" s="39"/>
+      <c r="N26" s="39"/>
+    </row>
+    <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="41" t="s">
+        <v>100</v>
+      </c>
+      <c r="B27" s="41"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="42" t="s">
+        <v>133</v>
+      </c>
+      <c r="F27" s="42"/>
+      <c r="G27" s="42"/>
+      <c r="H27" s="42"/>
+      <c r="I27" s="42"/>
+      <c r="J27" s="41" t="s">
+        <v>134</v>
+      </c>
+      <c r="K27" s="41"/>
+      <c r="L27" s="41"/>
+      <c r="M27" s="41"/>
+      <c r="N27" s="41"/>
+    </row>
+    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" s="39"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="39"/>
+      <c r="E28" s="40" t="s">
+        <v>135</v>
+      </c>
+      <c r="F28" s="40"/>
+      <c r="G28" s="40"/>
+      <c r="H28" s="40"/>
+      <c r="I28" s="40"/>
+      <c r="J28" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="K28" s="39"/>
+      <c r="L28" s="39"/>
+      <c r="M28" s="39"/>
+      <c r="N28" s="39"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="B29" s="41"/>
+      <c r="C29" s="41"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="42" t="s">
+        <v>136</v>
+      </c>
+      <c r="F29" s="42"/>
+      <c r="G29" s="42"/>
+      <c r="H29" s="42"/>
+      <c r="I29" s="42"/>
+      <c r="J29" s="41" t="s">
+        <v>97</v>
+      </c>
+      <c r="K29" s="41"/>
+      <c r="L29" s="41"/>
+      <c r="M29" s="41"/>
+      <c r="N29" s="41"/>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="B30" s="39"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="39"/>
+      <c r="E30" s="40" t="s">
+        <v>137</v>
+      </c>
+      <c r="F30" s="40"/>
+      <c r="G30" s="40"/>
+      <c r="H30" s="40"/>
+      <c r="I30" s="40"/>
+      <c r="J30" s="39" t="s">
+        <v>101</v>
+      </c>
+      <c r="K30" s="39"/>
+      <c r="L30" s="39"/>
+      <c r="M30" s="39"/>
+      <c r="N30" s="39"/>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="41" t="s">
+        <v>111</v>
+      </c>
+      <c r="B31" s="41"/>
+      <c r="C31" s="41"/>
+      <c r="D31" s="41"/>
+      <c r="E31" s="42" t="s">
+        <v>138</v>
+      </c>
+      <c r="F31" s="42"/>
+      <c r="G31" s="42"/>
+      <c r="H31" s="42"/>
+      <c r="I31" s="42"/>
+      <c r="J31" s="41" t="s">
+        <v>53</v>
+      </c>
+      <c r="K31" s="41"/>
+      <c r="L31" s="41"/>
+      <c r="M31" s="41"/>
+      <c r="N31" s="41"/>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="B32" s="39"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="39"/>
+      <c r="E32" s="40" t="s">
+        <v>139</v>
+      </c>
+      <c r="F32" s="40"/>
+      <c r="G32" s="40"/>
+      <c r="H32" s="40"/>
+      <c r="I32" s="40"/>
+      <c r="J32" s="39" t="s">
+        <v>134</v>
+      </c>
+      <c r="K32" s="39"/>
+      <c r="L32" s="39"/>
+      <c r="M32" s="39"/>
+      <c r="N32" s="39"/>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="42" t="s">
+        <v>140</v>
+      </c>
+      <c r="F33" s="42"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="41" t="s">
+        <v>98</v>
+      </c>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="41"/>
+      <c r="N33" s="41"/>
+    </row>
+    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="B34" s="39"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="39"/>
+      <c r="E34" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="F34" s="40"/>
+      <c r="G34" s="40"/>
+      <c r="H34" s="40"/>
+      <c r="I34" s="40"/>
+      <c r="J34" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="K34" s="39"/>
+      <c r="L34" s="39"/>
+      <c r="M34" s="39"/>
+      <c r="N34" s="39"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="41" t="s">
+        <v>119</v>
+      </c>
+      <c r="B35" s="41"/>
+      <c r="C35" s="41"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="42" t="s">
+        <v>141</v>
+      </c>
+      <c r="F35" s="42"/>
+      <c r="G35" s="42"/>
+      <c r="H35" s="42"/>
+      <c r="I35" s="42"/>
+      <c r="J35" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="K35" s="41"/>
+      <c r="L35" s="41"/>
+      <c r="M35" s="41"/>
+      <c r="N35" s="41"/>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="39" t="s">
+        <v>121</v>
+      </c>
+      <c r="B36" s="39"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="39"/>
+      <c r="E36" s="40" t="s">
+        <v>142</v>
+      </c>
+      <c r="F36" s="40"/>
+      <c r="G36" s="40"/>
+      <c r="H36" s="40"/>
+      <c r="I36" s="40"/>
+      <c r="J36" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="K36" s="39"/>
+      <c r="L36" s="39"/>
+      <c r="M36" s="39"/>
+      <c r="N36" s="39"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="41" t="s">
         <v>123</v>
       </c>
-      <c r="F26" s="38"/>
-      <c r="G26" s="38"/>
-      <c r="H26" s="38"/>
-      <c r="I26" s="38"/>
-      <c r="J26" s="37" t="s">
-        <v>53</v>
-      </c>
-      <c r="K26" s="37"/>
-      <c r="L26" s="37"/>
-      <c r="M26" s="37"/>
-      <c r="N26" s="37"/>
-    </row>
-    <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="39" t="s">
-        <v>91</v>
-      </c>
-      <c r="B27" s="39"/>
-      <c r="C27" s="39"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="40" t="s">
-        <v>124</v>
-      </c>
-      <c r="F27" s="40"/>
-      <c r="G27" s="40"/>
-      <c r="H27" s="40"/>
-      <c r="I27" s="40"/>
-      <c r="J27" s="39" t="s">
+      <c r="B37" s="41"/>
+      <c r="C37" s="41"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="42" t="s">
+        <v>143</v>
+      </c>
+      <c r="F37" s="42"/>
+      <c r="G37" s="42"/>
+      <c r="H37" s="42"/>
+      <c r="I37" s="42"/>
+      <c r="J37" s="41" t="s">
+        <v>134</v>
+      </c>
+      <c r="K37" s="41"/>
+      <c r="L37" s="41"/>
+      <c r="M37" s="41"/>
+      <c r="N37" s="41"/>
+    </row>
+    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="39" t="s">
         <v>125</v>
       </c>
-      <c r="K27" s="39"/>
-      <c r="L27" s="39"/>
-      <c r="M27" s="39"/>
-      <c r="N27" s="39"/>
-    </row>
-    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="B28" s="37"/>
-      <c r="C28" s="37"/>
-      <c r="D28" s="37"/>
-      <c r="E28" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="F28" s="38"/>
-      <c r="G28" s="38"/>
-      <c r="H28" s="38"/>
-      <c r="I28" s="38"/>
-      <c r="J28" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="K28" s="37"/>
-      <c r="L28" s="37"/>
-      <c r="M28" s="37"/>
-      <c r="N28" s="37"/>
-    </row>
-    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="39" t="s">
+      <c r="B38" s="39"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="39"/>
+      <c r="E38" s="40" t="s">
+        <v>144</v>
+      </c>
+      <c r="F38" s="40"/>
+      <c r="G38" s="40"/>
+      <c r="H38" s="40"/>
+      <c r="I38" s="40"/>
+      <c r="J38" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="K38" s="39"/>
+      <c r="L38" s="39"/>
+      <c r="M38" s="39"/>
+      <c r="N38" s="39"/>
+    </row>
+    <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" s="41" t="s">
+        <v>127</v>
+      </c>
+      <c r="B39" s="41"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="F39" s="42"/>
+      <c r="G39" s="42"/>
+      <c r="H39" s="42"/>
+      <c r="I39" s="42"/>
+      <c r="J39" s="41" t="s">
         <v>97</v>
       </c>
-      <c r="B29" s="39"/>
-      <c r="C29" s="39"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="40" t="s">
-        <v>127</v>
-      </c>
-      <c r="F29" s="40"/>
-      <c r="G29" s="40"/>
-      <c r="H29" s="40"/>
-      <c r="I29" s="40"/>
-      <c r="J29" s="39" t="s">
-        <v>88</v>
-      </c>
-      <c r="K29" s="39"/>
-      <c r="L29" s="39"/>
-      <c r="M29" s="39"/>
-      <c r="N29" s="39"/>
-    </row>
-    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="37" t="s">
-        <v>100</v>
-      </c>
-      <c r="B30" s="37"/>
-      <c r="C30" s="37"/>
-      <c r="D30" s="37"/>
-      <c r="E30" s="38" t="s">
-        <v>128</v>
-      </c>
-      <c r="F30" s="38"/>
-      <c r="G30" s="38"/>
-      <c r="H30" s="38"/>
-      <c r="I30" s="38"/>
-      <c r="J30" s="37" t="s">
-        <v>92</v>
-      </c>
-      <c r="K30" s="37"/>
-      <c r="L30" s="37"/>
-      <c r="M30" s="37"/>
-      <c r="N30" s="37"/>
-    </row>
-    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="B31" s="39"/>
-      <c r="C31" s="39"/>
-      <c r="D31" s="39"/>
-      <c r="E31" s="40" t="s">
-        <v>129</v>
-      </c>
-      <c r="F31" s="40"/>
-      <c r="G31" s="40"/>
-      <c r="H31" s="40"/>
-      <c r="I31" s="40"/>
-      <c r="J31" s="39" t="s">
-        <v>53</v>
-      </c>
-      <c r="K31" s="39"/>
-      <c r="L31" s="39"/>
-      <c r="M31" s="39"/>
-      <c r="N31" s="39"/>
-    </row>
-    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="37" t="s">
-        <v>104</v>
-      </c>
-      <c r="B32" s="37"/>
-      <c r="C32" s="37"/>
-      <c r="D32" s="37"/>
-      <c r="E32" s="38" t="s">
-        <v>130</v>
-      </c>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
-      <c r="H32" s="38"/>
-      <c r="I32" s="38"/>
-      <c r="J32" s="37" t="s">
-        <v>125</v>
-      </c>
-      <c r="K32" s="37"/>
-      <c r="L32" s="37"/>
-      <c r="M32" s="37"/>
-      <c r="N32" s="37"/>
-    </row>
-    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="39" t="s">
-        <v>106</v>
-      </c>
-      <c r="B33" s="39"/>
-      <c r="C33" s="39"/>
-      <c r="D33" s="39"/>
-      <c r="E33" s="40" t="s">
-        <v>131</v>
-      </c>
-      <c r="F33" s="40"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="40"/>
-      <c r="I33" s="40"/>
-      <c r="J33" s="39" t="s">
-        <v>89</v>
-      </c>
-      <c r="K33" s="39"/>
-      <c r="L33" s="39"/>
-      <c r="M33" s="39"/>
-      <c r="N33" s="39"/>
-    </row>
-    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="37" t="s">
-        <v>108</v>
-      </c>
-      <c r="B34" s="37"/>
-      <c r="C34" s="37"/>
-      <c r="D34" s="37"/>
-      <c r="E34" s="38" t="s">
-        <v>90</v>
-      </c>
-      <c r="F34" s="38"/>
-      <c r="G34" s="38"/>
-      <c r="H34" s="38"/>
-      <c r="I34" s="38"/>
-      <c r="J34" s="37" t="s">
-        <v>88</v>
-      </c>
-      <c r="K34" s="37"/>
-      <c r="L34" s="37"/>
-      <c r="M34" s="37"/>
-      <c r="N34" s="37"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="39" t="s">
-        <v>110</v>
-      </c>
-      <c r="B35" s="39"/>
-      <c r="C35" s="39"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="40" t="s">
-        <v>132</v>
-      </c>
-      <c r="F35" s="40"/>
-      <c r="G35" s="40"/>
-      <c r="H35" s="40"/>
-      <c r="I35" s="40"/>
-      <c r="J35" s="39" t="s">
-        <v>92</v>
-      </c>
-      <c r="K35" s="39"/>
-      <c r="L35" s="39"/>
-      <c r="M35" s="39"/>
-      <c r="N35" s="39"/>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" s="37" t="s">
-        <v>112</v>
-      </c>
-      <c r="B36" s="37"/>
-      <c r="C36" s="37"/>
-      <c r="D36" s="37"/>
-      <c r="E36" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="F36" s="38"/>
-      <c r="G36" s="38"/>
-      <c r="H36" s="38"/>
-      <c r="I36" s="38"/>
-      <c r="J36" s="37" t="s">
-        <v>53</v>
-      </c>
-      <c r="K36" s="37"/>
-      <c r="L36" s="37"/>
-      <c r="M36" s="37"/>
-      <c r="N36" s="37"/>
-    </row>
-    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="39" t="s">
-        <v>114</v>
-      </c>
-      <c r="B37" s="39"/>
-      <c r="C37" s="39"/>
-      <c r="D37" s="39"/>
-      <c r="E37" s="40" t="s">
-        <v>134</v>
-      </c>
-      <c r="F37" s="40"/>
-      <c r="G37" s="40"/>
-      <c r="H37" s="40"/>
-      <c r="I37" s="40"/>
-      <c r="J37" s="39" t="s">
-        <v>125</v>
-      </c>
-      <c r="K37" s="39"/>
-      <c r="L37" s="39"/>
-      <c r="M37" s="39"/>
-      <c r="N37" s="39"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="B38" s="37"/>
-      <c r="C38" s="37"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="38" t="s">
-        <v>135</v>
-      </c>
-      <c r="F38" s="38"/>
-      <c r="G38" s="38"/>
-      <c r="H38" s="38"/>
-      <c r="I38" s="38"/>
-      <c r="J38" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="K38" s="37"/>
-      <c r="L38" s="37"/>
-      <c r="M38" s="37"/>
-      <c r="N38" s="37"/>
-    </row>
-    <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A39" s="39" t="s">
-        <v>118</v>
-      </c>
-      <c r="B39" s="39"/>
-      <c r="C39" s="39"/>
-      <c r="D39" s="39"/>
-      <c r="E39" s="40" t="s">
-        <v>136</v>
-      </c>
-      <c r="F39" s="40"/>
-      <c r="G39" s="40"/>
-      <c r="H39" s="40"/>
-      <c r="I39" s="40"/>
-      <c r="J39" s="39" t="s">
-        <v>88</v>
-      </c>
-      <c r="K39" s="39"/>
-      <c r="L39" s="39"/>
-      <c r="M39" s="39"/>
-      <c r="N39" s="39"/>
+      <c r="K39" s="41"/>
+      <c r="L39" s="41"/>
+      <c r="M39" s="41"/>
+      <c r="N39" s="41"/>
     </row>
     <row r="40" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A40" s="41" t="s">
+      <c r="A40" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="B40" s="41"/>
-      <c r="C40" s="41"/>
-      <c r="D40" s="41"/>
-      <c r="E40" s="42" t="s">
+      <c r="B40" s="43"/>
+      <c r="C40" s="43"/>
+      <c r="D40" s="43"/>
+      <c r="E40" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="F40" s="42"/>
-      <c r="G40" s="42"/>
-      <c r="H40" s="42"/>
-      <c r="I40" s="42"/>
-      <c r="J40" s="41" t="s">
+      <c r="F40" s="44"/>
+      <c r="G40" s="44"/>
+      <c r="H40" s="44"/>
+      <c r="I40" s="44"/>
+      <c r="J40" s="43" t="s">
         <v>41</v>
       </c>
-      <c r="K40" s="41"/>
-      <c r="L40" s="41"/>
-      <c r="M40" s="41"/>
-      <c r="N40" s="41"/>
+      <c r="K40" s="43"/>
+      <c r="L40" s="43"/>
+      <c r="M40" s="43"/>
+      <c r="N40" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="52">

</xml_diff>

<commit_message>
feat(reporting): adopt canonical business day reporting architecture
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -60,7 +60,7 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>18 Jul 2026, 22:52</t>
+    <t>18 Jul 2026, 23:13</t>
   </si>
   <si>
     <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Payment Method Analysis  ·  Order Sales  ·  Check Revenue Trends</t>
@@ -72,7 +72,7 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 22:52</t>
+    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 23:13</t>
   </si>
   <si>
     <t>AT A GLANCE</t>

</xml_diff>

<commit_message>
refactor(reporting): align order dashboard KPI presentation
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -60,7 +60,7 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>18 Jul 2026, 23:13</t>
+    <t>19 Jul 2026, 18:38</t>
   </si>
   <si>
     <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Payment Method Analysis  ·  Order Sales  ·  Check Revenue Trends</t>
@@ -72,7 +72,7 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  18 Jul 2026, 23:13</t>
+    <t>Monthly Report  ·  July 2026  ·  19 Jul 2026, 18:38</t>
   </si>
   <si>
     <t>AT A GLANCE</t>
@@ -90,85 +90,85 @@
     <t>Order Sales</t>
   </si>
   <si>
+    <t>Completed Orders</t>
+  </si>
+  <si>
+    <t>Average Order</t>
+  </si>
+  <si>
+    <t>19,222.00 ر.س</t>
+  </si>
+  <si>
+    <t>89</t>
+  </si>
+  <si>
+    <t>215.98 ر.س</t>
+  </si>
+  <si>
+    <t>Value of orders that were completed (served)</t>
+  </si>
+  <si>
+    <t>How many orders were completed (served)</t>
+  </si>
+  <si>
+    <t>Typical size of a completed order</t>
+  </si>
+  <si>
+    <t>Check Revenue, Paid Checks, Average Check, and Tax Collected are in Financial Summary. Payment mix is in Payment Method Analysis.</t>
+  </si>
+  <si>
+    <t>Financial Summary</t>
+  </si>
+  <si>
+    <t>Monthly Report  ·  July 2026</t>
+  </si>
+  <si>
+    <t>MONEY COLLECTED</t>
+  </si>
+  <si>
+    <t>Paid guest checks for this reporting period — Check Revenue story.</t>
+  </si>
+  <si>
+    <t>CHECK REVENUE DETAIL</t>
+  </si>
+  <si>
+    <t>Check Revenue</t>
+  </si>
+  <si>
+    <t>14,612.50 ر.س</t>
+  </si>
+  <si>
+    <t>Paid Checks</t>
+  </si>
+  <si>
+    <t>68</t>
+  </si>
+  <si>
+    <t>Average Check</t>
+  </si>
+  <si>
+    <t>214.89 ر.س</t>
+  </si>
+  <si>
+    <t>TAX</t>
+  </si>
+  <si>
+    <t>Tax Collected covers the full reporting period — total tax from all paid checks in range (not a subset of sections).</t>
+  </si>
+  <si>
+    <t>Tax Collected</t>
+  </si>
+  <si>
+    <t>2,191.91 ر.س</t>
+  </si>
+  <si>
+    <t>ORDER SALES DETAIL</t>
+  </si>
+  <si>
     <t>Orders</t>
   </si>
   <si>
-    <t>Average Order</t>
-  </si>
-  <si>
-    <t>19,222.00 ر.س</t>
-  </si>
-  <si>
     <t>103</t>
-  </si>
-  <si>
-    <t>215.98 ر.س</t>
-  </si>
-  <si>
-    <t>Value of orders that were completed (served)</t>
-  </si>
-  <si>
-    <t>How many orders were placed</t>
-  </si>
-  <si>
-    <t>Typical size of a completed order</t>
-  </si>
-  <si>
-    <t>Check Revenue, Paid Checks, Average Check, and Tax Collected are in Financial Summary. Payment mix is in Payment Method Analysis.</t>
-  </si>
-  <si>
-    <t>Financial Summary</t>
-  </si>
-  <si>
-    <t>Monthly Report  ·  July 2026</t>
-  </si>
-  <si>
-    <t>MONEY COLLECTED</t>
-  </si>
-  <si>
-    <t>Paid guest checks for this reporting period — Check Revenue story.</t>
-  </si>
-  <si>
-    <t>CHECK REVENUE DETAIL</t>
-  </si>
-  <si>
-    <t>Check Revenue</t>
-  </si>
-  <si>
-    <t>14,612.50 ر.س</t>
-  </si>
-  <si>
-    <t>Paid Checks</t>
-  </si>
-  <si>
-    <t>68</t>
-  </si>
-  <si>
-    <t>Average Check</t>
-  </si>
-  <si>
-    <t>214.89 ر.س</t>
-  </si>
-  <si>
-    <t>TAX</t>
-  </si>
-  <si>
-    <t>Tax Collected covers the full reporting period — total tax from all paid checks in range (not a subset of sections).</t>
-  </si>
-  <si>
-    <t>Tax Collected</t>
-  </si>
-  <si>
-    <t>2,191.91 ر.س</t>
-  </si>
-  <si>
-    <t>ORDER SALES DETAIL</t>
-  </si>
-  <si>
-    <t>Completed Orders</t>
-  </si>
-  <si>
-    <t>89</t>
   </si>
   <si>
     <t>ADJUSTMENTS</t>
@@ -2273,7 +2273,7 @@
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="26" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
@@ -2283,7 +2283,7 @@
       <c r="G19" s="26"/>
       <c r="H19" s="26"/>
       <c r="I19" s="27" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="J19" s="27"/>
       <c r="K19" s="27"/>
@@ -2293,7 +2293,7 @@
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="28" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="B20" s="28"/>
       <c r="C20" s="28"/>
@@ -2303,7 +2303,7 @@
       <c r="G20" s="28"/>
       <c r="H20" s="28"/>
       <c r="I20" s="29" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="J20" s="29"/>
       <c r="K20" s="29"/>
@@ -3439,12 +3439,12 @@
       <c r="B24" s="37"/>
       <c r="C24" s="37"/>
       <c r="D24" s="38" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="E24" s="38"/>
       <c r="F24" s="38"/>
       <c r="G24" s="38" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="H24" s="38"/>
       <c r="I24" s="38"/>
@@ -3799,12 +3799,12 @@
       <c r="B39" s="43"/>
       <c r="C39" s="43"/>
       <c r="D39" s="43" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="E39" s="43"/>
       <c r="F39" s="43"/>
       <c r="G39" s="43" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="H39" s="43"/>
       <c r="I39" s="43"/>

</xml_diff>

<commit_message>
refactor(payments): unify canonical payment method catalog
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="141">
   <si>
     <t>MINEUQR</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>19 Jul 2026, 18:38</t>
+    <t>25 Jul 2026, 20:23</t>
   </si>
   <si>
     <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Payment Method Analysis  ·  Order Sales  ·  Check Revenue Trends</t>
@@ -72,7 +72,7 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  19 Jul 2026, 18:38</t>
+    <t>Monthly Report  ·  July 2026  ·  25 Jul 2026, 20:23</t>
   </si>
   <si>
     <t>AT A GLANCE</t>
@@ -255,7 +255,7 @@
     <t>40.00%</t>
   </si>
   <si>
-    <t>Mada</t>
+    <t>Card (network / bank)</t>
   </si>
   <si>
     <t>8,767.50 ر.س</t>
@@ -270,7 +270,7 @@
     <t>60.00%</t>
   </si>
   <si>
-    <t>Visa</t>
+    <t>Other</t>
   </si>
   <si>
     <t>0.00 ر.س</t>
@@ -280,21 +280,6 @@
   </si>
   <si>
     <t>0.00%</t>
-  </si>
-  <si>
-    <t>Mastercard</t>
-  </si>
-  <si>
-    <t>Apple Pay</t>
-  </si>
-  <si>
-    <t>STC Pay</t>
-  </si>
-  <si>
-    <t>Bank Transfer</t>
-  </si>
-  <si>
-    <t>Other</t>
   </si>
   <si>
     <t>Monthly Report  ·  Daily Order Sales — July 2026</t>
@@ -2566,7 +2551,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="10.2" customWidth="1"/>
@@ -2846,148 +2831,8 @@
       </c>
       <c r="N15" s="35"/>
     </row>
-    <row r="16" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="35" t="s">
-        <v>88</v>
-      </c>
-      <c r="B16" s="35"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="36" t="s">
-        <v>85</v>
-      </c>
-      <c r="E16" s="36"/>
-      <c r="F16" s="36"/>
-      <c r="G16" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35" t="s">
-        <v>85</v>
-      </c>
-      <c r="J16" s="35"/>
-      <c r="K16" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="L16" s="35"/>
-      <c r="M16" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="N16" s="35"/>
-    </row>
-    <row r="17" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="35" t="s">
-        <v>89</v>
-      </c>
-      <c r="B17" s="35"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="36" t="s">
-        <v>85</v>
-      </c>
-      <c r="E17" s="36"/>
-      <c r="F17" s="36"/>
-      <c r="G17" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="H17" s="35"/>
-      <c r="I17" s="35" t="s">
-        <v>85</v>
-      </c>
-      <c r="J17" s="35"/>
-      <c r="K17" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="L17" s="35"/>
-      <c r="M17" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="N17" s="35"/>
-    </row>
-    <row r="18" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="35" t="s">
-        <v>90</v>
-      </c>
-      <c r="B18" s="35"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="36" t="s">
-        <v>85</v>
-      </c>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35" t="s">
-        <v>85</v>
-      </c>
-      <c r="J18" s="35"/>
-      <c r="K18" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="L18" s="35"/>
-      <c r="M18" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="N18" s="35"/>
-    </row>
-    <row r="19" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="35" t="s">
-        <v>91</v>
-      </c>
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="36" t="s">
-        <v>85</v>
-      </c>
-      <c r="E19" s="36"/>
-      <c r="F19" s="36"/>
-      <c r="G19" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35" t="s">
-        <v>85</v>
-      </c>
-      <c r="J19" s="35"/>
-      <c r="K19" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="L19" s="35"/>
-      <c r="M19" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="N19" s="35"/>
-    </row>
-    <row r="20" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="35" t="s">
-        <v>92</v>
-      </c>
-      <c r="B20" s="35"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="36" t="s">
-        <v>85</v>
-      </c>
-      <c r="E20" s="36"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35" t="s">
-        <v>85</v>
-      </c>
-      <c r="J20" s="35"/>
-      <c r="K20" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="L20" s="35"/>
-      <c r="M20" s="35" t="s">
-        <v>86</v>
-      </c>
-      <c r="N20" s="35"/>
-    </row>
   </sheetData>
-  <mergeCells count="63">
+  <mergeCells count="33">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A5:N5"/>
@@ -3021,36 +2866,6 @@
     <mergeCell ref="I15:J15"/>
     <mergeCell ref="K15:L15"/>
     <mergeCell ref="M15:N15"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="M20:N20"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.25" footer="0.3"/>
@@ -3092,7 +2907,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3126,7 +2941,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -3434,7 +3249,7 @@
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="37" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B24" s="37"/>
       <c r="C24" s="37"/>
@@ -3458,22 +3273,22 @@
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="39" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B25" s="39"/>
       <c r="C25" s="39"/>
       <c r="D25" s="39" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E25" s="39"/>
       <c r="F25" s="39"/>
       <c r="G25" s="39" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="H25" s="39"/>
       <c r="I25" s="39"/>
       <c r="J25" s="40" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="K25" s="40"/>
       <c r="L25" s="40"/>
@@ -3482,22 +3297,22 @@
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="41" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B26" s="41"/>
       <c r="C26" s="41"/>
       <c r="D26" s="41" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E26" s="41"/>
       <c r="F26" s="41"/>
       <c r="G26" s="41" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="H26" s="41"/>
       <c r="I26" s="41"/>
       <c r="J26" s="42" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="K26" s="42"/>
       <c r="L26" s="42"/>
@@ -3506,22 +3321,22 @@
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="39" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B27" s="39"/>
       <c r="C27" s="39"/>
       <c r="D27" s="39" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E27" s="39"/>
       <c r="F27" s="39"/>
       <c r="G27" s="39" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H27" s="39"/>
       <c r="I27" s="39"/>
       <c r="J27" s="40" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="K27" s="40"/>
       <c r="L27" s="40"/>
@@ -3530,22 +3345,22 @@
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="41" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B28" s="41"/>
       <c r="C28" s="41"/>
       <c r="D28" s="41" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="E28" s="41"/>
       <c r="F28" s="41"/>
       <c r="G28" s="41" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="H28" s="41"/>
       <c r="I28" s="41"/>
       <c r="J28" s="42" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="K28" s="42"/>
       <c r="L28" s="42"/>
@@ -3554,22 +3369,22 @@
     </row>
     <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="39" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B29" s="39"/>
       <c r="C29" s="39"/>
       <c r="D29" s="39" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E29" s="39"/>
       <c r="F29" s="39"/>
       <c r="G29" s="39" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="H29" s="39"/>
       <c r="I29" s="39"/>
       <c r="J29" s="40" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="K29" s="40"/>
       <c r="L29" s="40"/>
@@ -3578,22 +3393,22 @@
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="41" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B30" s="41"/>
       <c r="C30" s="41"/>
       <c r="D30" s="41" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E30" s="41"/>
       <c r="F30" s="41"/>
       <c r="G30" s="41" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="H30" s="41"/>
       <c r="I30" s="41"/>
       <c r="J30" s="42" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="K30" s="42"/>
       <c r="L30" s="42"/>
@@ -3602,22 +3417,22 @@
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="39" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B31" s="39"/>
       <c r="C31" s="39"/>
       <c r="D31" s="39" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E31" s="39"/>
       <c r="F31" s="39"/>
       <c r="G31" s="39" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H31" s="39"/>
       <c r="I31" s="39"/>
       <c r="J31" s="40" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="K31" s="40"/>
       <c r="L31" s="40"/>
@@ -3626,22 +3441,22 @@
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="41" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B32" s="41"/>
       <c r="C32" s="41"/>
       <c r="D32" s="41" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="E32" s="41"/>
       <c r="F32" s="41"/>
       <c r="G32" s="41" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="H32" s="41"/>
       <c r="I32" s="41"/>
       <c r="J32" s="42" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="K32" s="42"/>
       <c r="L32" s="42"/>
@@ -3650,22 +3465,22 @@
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="39" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B33" s="39"/>
       <c r="C33" s="39"/>
       <c r="D33" s="39" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E33" s="39"/>
       <c r="F33" s="39"/>
       <c r="G33" s="39" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="H33" s="39"/>
       <c r="I33" s="39"/>
       <c r="J33" s="40" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="K33" s="40"/>
       <c r="L33" s="40"/>
@@ -3674,22 +3489,22 @@
     </row>
     <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="41" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B34" s="41"/>
       <c r="C34" s="41"/>
       <c r="D34" s="41" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E34" s="41"/>
       <c r="F34" s="41"/>
       <c r="G34" s="41" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="H34" s="41"/>
       <c r="I34" s="41"/>
       <c r="J34" s="42" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="K34" s="42"/>
       <c r="L34" s="42"/>
@@ -3698,22 +3513,22 @@
     </row>
     <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="39" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B35" s="39"/>
       <c r="C35" s="39"/>
       <c r="D35" s="39" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E35" s="39"/>
       <c r="F35" s="39"/>
       <c r="G35" s="39" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H35" s="39"/>
       <c r="I35" s="39"/>
       <c r="J35" s="40" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="K35" s="40"/>
       <c r="L35" s="40"/>
@@ -3722,22 +3537,22 @@
     </row>
     <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="41" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B36" s="41"/>
       <c r="C36" s="41"/>
       <c r="D36" s="41" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="E36" s="41"/>
       <c r="F36" s="41"/>
       <c r="G36" s="41" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="H36" s="41"/>
       <c r="I36" s="41"/>
       <c r="J36" s="42" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="K36" s="42"/>
       <c r="L36" s="42"/>
@@ -3746,22 +3561,22 @@
     </row>
     <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="39" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B37" s="39"/>
       <c r="C37" s="39"/>
       <c r="D37" s="39" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E37" s="39"/>
       <c r="F37" s="39"/>
       <c r="G37" s="39" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="H37" s="39"/>
       <c r="I37" s="39"/>
       <c r="J37" s="40" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="K37" s="40"/>
       <c r="L37" s="40"/>
@@ -3770,22 +3585,22 @@
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="41" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B38" s="41"/>
       <c r="C38" s="41"/>
       <c r="D38" s="41" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E38" s="41"/>
       <c r="F38" s="41"/>
       <c r="G38" s="41" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="H38" s="41"/>
       <c r="I38" s="41"/>
       <c r="J38" s="42" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="K38" s="42"/>
       <c r="L38" s="42"/>
@@ -3910,7 +3725,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -3928,7 +3743,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3962,7 +3777,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -4286,7 +4101,7 @@
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="37" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B25" s="37"/>
       <c r="C25" s="37"/>
@@ -4308,13 +4123,13 @@
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="39" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B26" s="39"/>
       <c r="C26" s="39"/>
       <c r="D26" s="39"/>
       <c r="E26" s="40" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F26" s="40"/>
       <c r="G26" s="40"/>
@@ -4330,20 +4145,20 @@
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="41" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B27" s="41"/>
       <c r="C27" s="41"/>
       <c r="D27" s="41"/>
       <c r="E27" s="42" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F27" s="42"/>
       <c r="G27" s="42"/>
       <c r="H27" s="42"/>
       <c r="I27" s="42"/>
       <c r="J27" s="41" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="K27" s="41"/>
       <c r="L27" s="41"/>
@@ -4352,20 +4167,20 @@
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B28" s="39"/>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
       <c r="E28" s="40" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F28" s="40"/>
       <c r="G28" s="40"/>
       <c r="H28" s="40"/>
       <c r="I28" s="40"/>
       <c r="J28" s="39" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="K28" s="39"/>
       <c r="L28" s="39"/>
@@ -4374,20 +4189,20 @@
     </row>
     <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="41" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B29" s="41"/>
       <c r="C29" s="41"/>
       <c r="D29" s="41"/>
       <c r="E29" s="42" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="F29" s="42"/>
       <c r="G29" s="42"/>
       <c r="H29" s="42"/>
       <c r="I29" s="42"/>
       <c r="J29" s="41" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="K29" s="41"/>
       <c r="L29" s="41"/>
@@ -4396,20 +4211,20 @@
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="39" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B30" s="39"/>
       <c r="C30" s="39"/>
       <c r="D30" s="39"/>
       <c r="E30" s="40" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="F30" s="40"/>
       <c r="G30" s="40"/>
       <c r="H30" s="40"/>
       <c r="I30" s="40"/>
       <c r="J30" s="39" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="K30" s="39"/>
       <c r="L30" s="39"/>
@@ -4418,13 +4233,13 @@
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="41" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B31" s="41"/>
       <c r="C31" s="41"/>
       <c r="D31" s="41"/>
       <c r="E31" s="42" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F31" s="42"/>
       <c r="G31" s="42"/>
@@ -4440,20 +4255,20 @@
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="39" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B32" s="39"/>
       <c r="C32" s="39"/>
       <c r="D32" s="39"/>
       <c r="E32" s="40" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="F32" s="40"/>
       <c r="G32" s="40"/>
       <c r="H32" s="40"/>
       <c r="I32" s="40"/>
       <c r="J32" s="39" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="K32" s="39"/>
       <c r="L32" s="39"/>
@@ -4462,20 +4277,20 @@
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="41" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B33" s="41"/>
       <c r="C33" s="41"/>
       <c r="D33" s="41"/>
       <c r="E33" s="42" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F33" s="42"/>
       <c r="G33" s="42"/>
       <c r="H33" s="42"/>
       <c r="I33" s="42"/>
       <c r="J33" s="41" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="K33" s="41"/>
       <c r="L33" s="41"/>
@@ -4484,20 +4299,20 @@
     </row>
     <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="39" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B34" s="39"/>
       <c r="C34" s="39"/>
       <c r="D34" s="39"/>
       <c r="E34" s="40" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="F34" s="40"/>
       <c r="G34" s="40"/>
       <c r="H34" s="40"/>
       <c r="I34" s="40"/>
       <c r="J34" s="39" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="K34" s="39"/>
       <c r="L34" s="39"/>
@@ -4506,20 +4321,20 @@
     </row>
     <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="41" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B35" s="41"/>
       <c r="C35" s="41"/>
       <c r="D35" s="41"/>
       <c r="E35" s="42" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F35" s="42"/>
       <c r="G35" s="42"/>
       <c r="H35" s="42"/>
       <c r="I35" s="42"/>
       <c r="J35" s="41" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="K35" s="41"/>
       <c r="L35" s="41"/>
@@ -4528,13 +4343,13 @@
     </row>
     <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="39" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B36" s="39"/>
       <c r="C36" s="39"/>
       <c r="D36" s="39"/>
       <c r="E36" s="40" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="F36" s="40"/>
       <c r="G36" s="40"/>
@@ -4550,20 +4365,20 @@
     </row>
     <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="41" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B37" s="41"/>
       <c r="C37" s="41"/>
       <c r="D37" s="41"/>
       <c r="E37" s="42" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F37" s="42"/>
       <c r="G37" s="42"/>
       <c r="H37" s="42"/>
       <c r="I37" s="42"/>
       <c r="J37" s="41" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="K37" s="41"/>
       <c r="L37" s="41"/>
@@ -4572,20 +4387,20 @@
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="39" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B38" s="39"/>
       <c r="C38" s="39"/>
       <c r="D38" s="39"/>
       <c r="E38" s="40" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="F38" s="40"/>
       <c r="G38" s="40"/>
       <c r="H38" s="40"/>
       <c r="I38" s="40"/>
       <c r="J38" s="39" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="K38" s="39"/>
       <c r="L38" s="39"/>
@@ -4594,20 +4409,20 @@
     </row>
     <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="41" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B39" s="41"/>
       <c r="C39" s="41"/>
       <c r="D39" s="41"/>
       <c r="E39" s="42" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="F39" s="42"/>
       <c r="G39" s="42"/>
       <c r="H39" s="42"/>
       <c r="I39" s="42"/>
       <c r="J39" s="41" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="K39" s="41"/>
       <c r="L39" s="41"/>

</xml_diff>

<commit_message>
feat(refund): adopt refund presentation workflow
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="147">
   <si>
     <t>MINEUQR</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>25 Jul 2026, 20:23</t>
+    <t>26 Jul 2026, 13:54</t>
   </si>
   <si>
     <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Payment Method Analysis  ·  Order Sales  ·  Check Revenue Trends</t>
@@ -72,7 +72,7 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  25 Jul 2026, 20:23</t>
+    <t>Monthly Report  ·  July 2026  ·  26 Jul 2026, 13:54</t>
   </si>
   <si>
     <t>AT A GLANCE</t>
@@ -114,7 +114,7 @@
     <t>Typical size of a completed order</t>
   </si>
   <si>
-    <t>Check Revenue, Paid Checks, Average Check, and Tax Collected are in Financial Summary. Payment mix is in Payment Method Analysis.</t>
+    <t>Check Revenue (Gross), Net Revenue, Refund Publications, Paid Checks, Average Check, and Tax Collected are in Financial Summary. Payment and refund mix are in Payment Method Analysis.</t>
   </si>
   <si>
     <t>Financial Summary</t>
@@ -126,7 +126,7 @@
     <t>MONEY COLLECTED</t>
   </si>
   <si>
-    <t>Paid guest checks for this reporting period — Check Revenue story.</t>
+    <t>Paid guest checks for this reporting period — Gross Check Revenue. Net Revenue subtracts Refund Publications.</t>
   </si>
   <si>
     <t>CHECK REVENUE DETAIL</t>
@@ -138,12 +138,33 @@
     <t>14,612.50 ر.س</t>
   </si>
   <si>
+    <t>Refund Publications</t>
+  </si>
+  <si>
+    <t>0.00 ر.س</t>
+  </si>
+  <si>
+    <t>Net Revenue</t>
+  </si>
+  <si>
+    <t>Refund Rate</t>
+  </si>
+  <si>
+    <t>0.00%</t>
+  </si>
+  <si>
     <t>Paid Checks</t>
   </si>
   <si>
     <t>68</t>
   </si>
   <si>
+    <t>Refund Count</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
     <t>Average Check</t>
   </si>
   <si>
@@ -207,7 +228,7 @@
     <t>Payment Method Analysis</t>
   </si>
   <si>
-    <t>Payment mix is from settlement tenders. Check Revenue remains the official revenue total from paid checks.</t>
+    <t>Payment mix is from settlement tenders. Check Revenue remains Gross from paid checks; refund tenders are listed separately and do not replace Check Revenue.</t>
   </si>
   <si>
     <t>PAYMENT MIX</t>
@@ -273,13 +294,10 @@
     <t>Other</t>
   </si>
   <si>
-    <t>0.00 ر.س</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>0.00%</t>
+    <t>REFUND MIX BY PAYMENT METHOD</t>
+  </si>
+  <si>
+    <t>Refund Tender Total</t>
   </si>
   <si>
     <t>Monthly Report  ·  Daily Order Sales — July 2026</t>
@@ -1954,7 +1972,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="10.2" customWidth="1"/>
@@ -2134,7 +2152,7 @@
       <c r="G10" s="26"/>
       <c r="H10" s="26"/>
       <c r="I10" s="27" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="J10" s="27"/>
       <c r="K10" s="27"/>
@@ -2142,65 +2160,89 @@
       <c r="M10" s="27"/>
       <c r="N10" s="27"/>
     </row>
-    <row r="12" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
+    <row r="11" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="19"/>
-      <c r="M12" s="19"/>
-      <c r="N12" s="19"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="21" t="s">
+      <c r="J11" s="29"/>
+      <c r="K11" s="29"/>
+      <c r="L11" s="29"/>
+      <c r="M11" s="29"/>
+      <c r="N11" s="29"/>
+    </row>
+    <row r="12" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="21"/>
-      <c r="I13" s="21"/>
-      <c r="J13" s="21"/>
-      <c r="K13" s="21"/>
-      <c r="L13" s="21"/>
-      <c r="M13" s="21"/>
-      <c r="N13" s="21"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="27" t="s">
+        <v>46</v>
+      </c>
+      <c r="J12" s="27"/>
+      <c r="K12" s="27"/>
+      <c r="L12" s="27"/>
+      <c r="M12" s="27"/>
+      <c r="N12" s="27"/>
+    </row>
+    <row r="13" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="J13" s="29"/>
+      <c r="K13" s="29"/>
+      <c r="L13" s="29"/>
+      <c r="M13" s="29"/>
+      <c r="N13" s="29"/>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="30" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" s="30"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
-      <c r="I14" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="J14" s="31"/>
-      <c r="K14" s="31"/>
-      <c r="L14" s="31"/>
-      <c r="M14" s="31"/>
-      <c r="N14" s="31"/>
+      <c r="A14" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="27" t="s">
+        <v>50</v>
+      </c>
+      <c r="J14" s="27"/>
+      <c r="K14" s="27"/>
+      <c r="L14" s="27"/>
+      <c r="M14" s="27"/>
+      <c r="N14" s="27"/>
     </row>
     <row r="16" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B16" s="19"/>
       <c r="C16" s="19"/>
@@ -2216,107 +2258,105 @@
       <c r="M16" s="19"/>
       <c r="N16" s="19"/>
     </row>
-    <row r="17" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="26" t="s">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="21"/>
+      <c r="J17" s="21"/>
+      <c r="K17" s="21"/>
+      <c r="L17" s="21"/>
+      <c r="M17" s="21"/>
+      <c r="N17" s="21"/>
+    </row>
+    <row r="18" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="31" t="s">
+        <v>54</v>
+      </c>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+      <c r="L18" s="31"/>
+      <c r="M18" s="31"/>
+      <c r="N18" s="31"/>
+    </row>
+    <row r="20" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="19"/>
+      <c r="N20" s="19"/>
+    </row>
+    <row r="21" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="26"/>
-      <c r="I17" s="27" t="s">
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="J17" s="27"/>
-      <c r="K17" s="27"/>
-      <c r="L17" s="27"/>
-      <c r="M17" s="27"/>
-      <c r="N17" s="27"/>
-    </row>
-    <row r="18" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="28" t="s">
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="27"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+    </row>
+    <row r="22" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="28"/>
-      <c r="H18" s="28"/>
-      <c r="I18" s="29" t="s">
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="J18" s="29"/>
-      <c r="K18" s="29"/>
-      <c r="L18" s="29"/>
-      <c r="M18" s="29"/>
-      <c r="N18" s="29"/>
-    </row>
-    <row r="19" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="J19" s="27"/>
-      <c r="K19" s="27"/>
-      <c r="L19" s="27"/>
-      <c r="M19" s="27"/>
-      <c r="N19" s="27"/>
-    </row>
-    <row r="20" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="28" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="J20" s="29"/>
-      <c r="K20" s="29"/>
-      <c r="L20" s="29"/>
-      <c r="M20" s="29"/>
-      <c r="N20" s="29"/>
-    </row>
-    <row r="22" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="19"/>
-      <c r="J22" s="19"/>
-      <c r="K22" s="19"/>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19"/>
-      <c r="N22" s="19"/>
+      <c r="J22" s="29"/>
+      <c r="K22" s="29"/>
+      <c r="L22" s="29"/>
+      <c r="M22" s="29"/>
+      <c r="N22" s="29"/>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B23" s="26"/>
       <c r="C23" s="26"/>
@@ -2326,7 +2366,7 @@
       <c r="G23" s="26"/>
       <c r="H23" s="26"/>
       <c r="I23" s="27" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="J23" s="27"/>
       <c r="K23" s="27"/>
@@ -2336,7 +2376,7 @@
     </row>
     <row r="24" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="28" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B24" s="28"/>
       <c r="C24" s="28"/>
@@ -2346,7 +2386,7 @@
       <c r="G24" s="28"/>
       <c r="H24" s="28"/>
       <c r="I24" s="29" t="s">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="J24" s="29"/>
       <c r="K24" s="29"/>
@@ -2354,127 +2394,105 @@
       <c r="M24" s="29"/>
       <c r="N24" s="29"/>
     </row>
-    <row r="25" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="26" t="s">
-        <v>56</v>
-      </c>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="J25" s="27"/>
-      <c r="K25" s="27"/>
-      <c r="L25" s="27"/>
-      <c r="M25" s="27"/>
-      <c r="N25" s="27"/>
-    </row>
-    <row r="27" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="19" t="s">
+    <row r="26" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19"/>
-      <c r="I27" s="19"/>
-      <c r="J27" s="19"/>
-      <c r="K27" s="19"/>
-      <c r="L27" s="19"/>
-      <c r="M27" s="19"/>
-      <c r="N27" s="19"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="19"/>
+      <c r="J26" s="19"/>
+      <c r="K26" s="19"/>
+      <c r="L26" s="19"/>
+      <c r="M26" s="19"/>
+      <c r="N26" s="19"/>
+    </row>
+    <row r="27" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="B27" s="26"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="J27" s="27"/>
+      <c r="K27" s="27"/>
+      <c r="L27" s="27"/>
+      <c r="M27" s="27"/>
+      <c r="N27" s="27"/>
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="J28" s="27"/>
-      <c r="K28" s="27"/>
-      <c r="L28" s="27"/>
-      <c r="M28" s="27"/>
-      <c r="N28" s="27"/>
+      <c r="A28" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="J28" s="29"/>
+      <c r="K28" s="29"/>
+      <c r="L28" s="29"/>
+      <c r="M28" s="29"/>
+      <c r="N28" s="29"/>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="J29" s="29"/>
-      <c r="K29" s="29"/>
-      <c r="L29" s="29"/>
-      <c r="M29" s="29"/>
-      <c r="N29" s="29"/>
-    </row>
-    <row r="30" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="27" t="s">
-        <v>61</v>
-      </c>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="27"/>
-      <c r="M30" s="27"/>
-      <c r="N30" s="27"/>
-    </row>
-    <row r="31" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="29" t="s">
-        <v>10</v>
-      </c>
-      <c r="J31" s="29"/>
-      <c r="K31" s="29"/>
-      <c r="L31" s="29"/>
-      <c r="M31" s="29"/>
-      <c r="N31" s="29"/>
+      <c r="A29" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="26"/>
+      <c r="I29" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="J29" s="27"/>
+      <c r="K29" s="27"/>
+      <c r="L29" s="27"/>
+      <c r="M29" s="27"/>
+      <c r="N29" s="27"/>
+    </row>
+    <row r="31" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="19"/>
+      <c r="K31" s="19"/>
+      <c r="L31" s="19"/>
+      <c r="M31" s="19"/>
+      <c r="N31" s="19"/>
     </row>
     <row r="32" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="B32" s="26"/>
       <c r="C32" s="26"/>
@@ -2484,7 +2502,7 @@
       <c r="G32" s="26"/>
       <c r="H32" s="26"/>
       <c r="I32" s="27" t="s">
-        <v>12</v>
+        <v>66</v>
       </c>
       <c r="J32" s="27"/>
       <c r="K32" s="27"/>
@@ -2492,8 +2510,88 @@
       <c r="M32" s="27"/>
       <c r="N32" s="27"/>
     </row>
+    <row r="33" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
+      <c r="I33" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="J33" s="29"/>
+      <c r="K33" s="29"/>
+      <c r="L33" s="29"/>
+      <c r="M33" s="29"/>
+      <c r="N33" s="29"/>
+    </row>
+    <row r="34" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" s="26"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="26"/>
+      <c r="F34" s="26"/>
+      <c r="G34" s="26"/>
+      <c r="H34" s="26"/>
+      <c r="I34" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="J34" s="27"/>
+      <c r="K34" s="27"/>
+      <c r="L34" s="27"/>
+      <c r="M34" s="27"/>
+      <c r="N34" s="27"/>
+    </row>
+    <row r="35" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="B35" s="28"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="28"/>
+      <c r="H35" s="28"/>
+      <c r="I35" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="J35" s="29"/>
+      <c r="K35" s="29"/>
+      <c r="L35" s="29"/>
+      <c r="M35" s="29"/>
+      <c r="N35" s="29"/>
+    </row>
+    <row r="36" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" s="26"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="26"/>
+      <c r="G36" s="26"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="J36" s="27"/>
+      <c r="K36" s="27"/>
+      <c r="L36" s="27"/>
+      <c r="M36" s="27"/>
+      <c r="N36" s="27"/>
+    </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="50">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A5:N5"/>
@@ -2505,37 +2603,45 @@
     <mergeCell ref="I9:N9"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="I10:N10"/>
-    <mergeCell ref="A12:N12"/>
-    <mergeCell ref="A13:N13"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="I11:N11"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="I12:N12"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="I13:N13"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="I14:N14"/>
     <mergeCell ref="A16:N16"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="I17:N17"/>
+    <mergeCell ref="A17:N17"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="I18:N18"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="I19:N19"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="I20:N20"/>
-    <mergeCell ref="A22:N22"/>
+    <mergeCell ref="A20:N20"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="I21:N21"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="I22:N22"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="I23:N23"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="I24:N24"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="I25:N25"/>
-    <mergeCell ref="A27:N27"/>
+    <mergeCell ref="A26:N26"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="I27:N27"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="I28:N28"/>
     <mergeCell ref="A29:H29"/>
     <mergeCell ref="I29:N29"/>
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="I30:N30"/>
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="I31:N31"/>
+    <mergeCell ref="A31:N31"/>
     <mergeCell ref="A32:H32"/>
     <mergeCell ref="I32:N32"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="I33:N33"/>
+    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="I34:N34"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="I35:N35"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="I36:N36"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.25" footer="0.3"/>
@@ -2551,7 +2657,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="10.2" customWidth="1"/>
@@ -2559,7 +2665,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -2627,7 +2733,7 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B5" s="21"/>
       <c r="C5" s="21"/>
@@ -2645,7 +2751,7 @@
     </row>
     <row r="7" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="19"/>
@@ -2663,7 +2769,7 @@
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B8" s="26"/>
       <c r="C8" s="26"/>
@@ -2683,7 +2789,7 @@
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B9" s="28"/>
       <c r="C9" s="28"/>
@@ -2693,7 +2799,7 @@
       <c r="G9" s="28"/>
       <c r="H9" s="28"/>
       <c r="I9" s="29" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="J9" s="29"/>
       <c r="K9" s="29"/>
@@ -2703,7 +2809,7 @@
     </row>
     <row r="11" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B11" s="19"/>
       <c r="C11" s="19"/>
@@ -2721,118 +2827,156 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="32" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="B12" s="32"/>
       <c r="C12" s="32"/>
       <c r="D12" s="32" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="E12" s="32"/>
       <c r="F12" s="32"/>
       <c r="G12" s="32" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="H12" s="32"/>
       <c r="I12" s="32" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="J12" s="32"/>
       <c r="K12" s="32" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="L12" s="32"/>
       <c r="M12" s="32" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="N12" s="32"/>
     </row>
     <row r="13" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="33"/>
       <c r="D13" s="34" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="E13" s="34"/>
       <c r="F13" s="34"/>
       <c r="G13" s="33" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="H13" s="33"/>
       <c r="I13" s="33" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="J13" s="33"/>
       <c r="K13" s="33" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="L13" s="33"/>
       <c r="M13" s="33" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="N13" s="33"/>
     </row>
     <row r="14" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="33" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="33"/>
       <c r="D14" s="34" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="E14" s="34"/>
       <c r="F14" s="34"/>
       <c r="G14" s="33" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H14" s="33"/>
       <c r="I14" s="33" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="J14" s="33"/>
       <c r="K14" s="33" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="L14" s="33"/>
       <c r="M14" s="33" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="N14" s="33"/>
     </row>
     <row r="15" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="35" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B15" s="35"/>
       <c r="C15" s="35"/>
       <c r="D15" s="36" t="s">
-        <v>85</v>
+        <v>41</v>
       </c>
       <c r="E15" s="36"/>
       <c r="F15" s="36"/>
       <c r="G15" s="35" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
       <c r="H15" s="35"/>
       <c r="I15" s="35" t="s">
-        <v>85</v>
+        <v>41</v>
       </c>
       <c r="J15" s="35"/>
       <c r="K15" s="35" t="s">
-        <v>87</v>
+        <v>44</v>
       </c>
       <c r="L15" s="35"/>
       <c r="M15" s="35" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
       <c r="N15" s="35"/>
     </row>
+    <row r="17" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="19"/>
+      <c r="K17" s="19"/>
+      <c r="L17" s="19"/>
+      <c r="M17" s="19"/>
+      <c r="N17" s="19"/>
+    </row>
+    <row r="18" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="26" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27"/>
+      <c r="L18" s="27"/>
+      <c r="M18" s="27"/>
+      <c r="N18" s="27"/>
+    </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="36">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A5:N5"/>
@@ -2866,6 +3010,9 @@
     <mergeCell ref="I15:J15"/>
     <mergeCell ref="K15:L15"/>
     <mergeCell ref="M15:N15"/>
+    <mergeCell ref="A17:N17"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="I18:N18"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.25" footer="0.3"/>
@@ -2907,7 +3054,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2941,7 +3088,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -3231,7 +3378,7 @@
     </row>
     <row r="23" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="B23" s="19"/>
       <c r="C23" s="19"/>
@@ -3249,12 +3396,12 @@
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="37" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B24" s="37"/>
       <c r="C24" s="37"/>
       <c r="D24" s="38" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E24" s="38"/>
       <c r="F24" s="38"/>
@@ -3273,22 +3420,22 @@
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="39" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B25" s="39"/>
       <c r="C25" s="39"/>
       <c r="D25" s="39" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E25" s="39"/>
       <c r="F25" s="39"/>
       <c r="G25" s="39" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="H25" s="39"/>
       <c r="I25" s="39"/>
       <c r="J25" s="40" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="K25" s="40"/>
       <c r="L25" s="40"/>
@@ -3297,22 +3444,22 @@
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="41" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B26" s="41"/>
       <c r="C26" s="41"/>
       <c r="D26" s="41" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E26" s="41"/>
       <c r="F26" s="41"/>
       <c r="G26" s="41" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="H26" s="41"/>
       <c r="I26" s="41"/>
       <c r="J26" s="42" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="K26" s="42"/>
       <c r="L26" s="42"/>
@@ -3321,22 +3468,22 @@
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="39" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B27" s="39"/>
       <c r="C27" s="39"/>
       <c r="D27" s="39" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E27" s="39"/>
       <c r="F27" s="39"/>
       <c r="G27" s="39" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="H27" s="39"/>
       <c r="I27" s="39"/>
       <c r="J27" s="40" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="K27" s="40"/>
       <c r="L27" s="40"/>
@@ -3345,22 +3492,22 @@
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="41" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B28" s="41"/>
       <c r="C28" s="41"/>
       <c r="D28" s="41" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E28" s="41"/>
       <c r="F28" s="41"/>
       <c r="G28" s="41" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="H28" s="41"/>
       <c r="I28" s="41"/>
       <c r="J28" s="42" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="K28" s="42"/>
       <c r="L28" s="42"/>
@@ -3369,22 +3516,22 @@
     </row>
     <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="39" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B29" s="39"/>
       <c r="C29" s="39"/>
       <c r="D29" s="39" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E29" s="39"/>
       <c r="F29" s="39"/>
       <c r="G29" s="39" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="H29" s="39"/>
       <c r="I29" s="39"/>
       <c r="J29" s="40" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="K29" s="40"/>
       <c r="L29" s="40"/>
@@ -3393,22 +3540,22 @@
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="41" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B30" s="41"/>
       <c r="C30" s="41"/>
       <c r="D30" s="41" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E30" s="41"/>
       <c r="F30" s="41"/>
       <c r="G30" s="41" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="H30" s="41"/>
       <c r="I30" s="41"/>
       <c r="J30" s="42" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="K30" s="42"/>
       <c r="L30" s="42"/>
@@ -3417,22 +3564,22 @@
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="39" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B31" s="39"/>
       <c r="C31" s="39"/>
       <c r="D31" s="39" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E31" s="39"/>
       <c r="F31" s="39"/>
       <c r="G31" s="39" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="H31" s="39"/>
       <c r="I31" s="39"/>
       <c r="J31" s="40" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="K31" s="40"/>
       <c r="L31" s="40"/>
@@ -3441,22 +3588,22 @@
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="41" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B32" s="41"/>
       <c r="C32" s="41"/>
       <c r="D32" s="41" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E32" s="41"/>
       <c r="F32" s="41"/>
       <c r="G32" s="41" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="H32" s="41"/>
       <c r="I32" s="41"/>
       <c r="J32" s="42" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="K32" s="42"/>
       <c r="L32" s="42"/>
@@ -3465,22 +3612,22 @@
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="39" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B33" s="39"/>
       <c r="C33" s="39"/>
       <c r="D33" s="39" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E33" s="39"/>
       <c r="F33" s="39"/>
       <c r="G33" s="39" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="H33" s="39"/>
       <c r="I33" s="39"/>
       <c r="J33" s="40" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="K33" s="40"/>
       <c r="L33" s="40"/>
@@ -3489,22 +3636,22 @@
     </row>
     <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="41" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B34" s="41"/>
       <c r="C34" s="41"/>
       <c r="D34" s="41" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E34" s="41"/>
       <c r="F34" s="41"/>
       <c r="G34" s="41" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="H34" s="41"/>
       <c r="I34" s="41"/>
       <c r="J34" s="42" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="K34" s="42"/>
       <c r="L34" s="42"/>
@@ -3513,22 +3660,22 @@
     </row>
     <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="39" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B35" s="39"/>
       <c r="C35" s="39"/>
       <c r="D35" s="39" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E35" s="39"/>
       <c r="F35" s="39"/>
       <c r="G35" s="39" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="H35" s="39"/>
       <c r="I35" s="39"/>
       <c r="J35" s="40" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="K35" s="40"/>
       <c r="L35" s="40"/>
@@ -3537,22 +3684,22 @@
     </row>
     <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="41" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B36" s="41"/>
       <c r="C36" s="41"/>
       <c r="D36" s="41" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E36" s="41"/>
       <c r="F36" s="41"/>
       <c r="G36" s="41" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="H36" s="41"/>
       <c r="I36" s="41"/>
       <c r="J36" s="42" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="K36" s="42"/>
       <c r="L36" s="42"/>
@@ -3561,22 +3708,22 @@
     </row>
     <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="39" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B37" s="39"/>
       <c r="C37" s="39"/>
       <c r="D37" s="39" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E37" s="39"/>
       <c r="F37" s="39"/>
       <c r="G37" s="39" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="H37" s="39"/>
       <c r="I37" s="39"/>
       <c r="J37" s="40" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="K37" s="40"/>
       <c r="L37" s="40"/>
@@ -3585,22 +3732,22 @@
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="41" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B38" s="41"/>
       <c r="C38" s="41"/>
       <c r="D38" s="41" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E38" s="41"/>
       <c r="F38" s="41"/>
       <c r="G38" s="41" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="H38" s="41"/>
       <c r="I38" s="41"/>
       <c r="J38" s="42" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="K38" s="42"/>
       <c r="L38" s="42"/>
@@ -3614,7 +3761,7 @@
       <c r="B39" s="43"/>
       <c r="C39" s="43"/>
       <c r="D39" s="43" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="E39" s="43"/>
       <c r="F39" s="43"/>
@@ -3725,7 +3872,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -3743,7 +3890,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3777,7 +3924,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -4101,7 +4248,7 @@
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="37" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B25" s="37"/>
       <c r="C25" s="37"/>
@@ -4114,7 +4261,7 @@
       <c r="H25" s="38"/>
       <c r="I25" s="38"/>
       <c r="J25" s="38" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="K25" s="38"/>
       <c r="L25" s="38"/>
@@ -4123,20 +4270,20 @@
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="39" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B26" s="39"/>
       <c r="C26" s="39"/>
       <c r="D26" s="39"/>
       <c r="E26" s="40" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="F26" s="40"/>
       <c r="G26" s="40"/>
       <c r="H26" s="40"/>
       <c r="I26" s="40"/>
       <c r="J26" s="39" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="K26" s="39"/>
       <c r="L26" s="39"/>
@@ -4145,20 +4292,20 @@
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="41" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B27" s="41"/>
       <c r="C27" s="41"/>
       <c r="D27" s="41"/>
       <c r="E27" s="42" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="F27" s="42"/>
       <c r="G27" s="42"/>
       <c r="H27" s="42"/>
       <c r="I27" s="42"/>
       <c r="J27" s="41" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="K27" s="41"/>
       <c r="L27" s="41"/>
@@ -4167,20 +4314,20 @@
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B28" s="39"/>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
       <c r="E28" s="40" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="F28" s="40"/>
       <c r="G28" s="40"/>
       <c r="H28" s="40"/>
       <c r="I28" s="40"/>
       <c r="J28" s="39" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="K28" s="39"/>
       <c r="L28" s="39"/>
@@ -4189,20 +4336,20 @@
     </row>
     <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="41" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B29" s="41"/>
       <c r="C29" s="41"/>
       <c r="D29" s="41"/>
       <c r="E29" s="42" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F29" s="42"/>
       <c r="G29" s="42"/>
       <c r="H29" s="42"/>
       <c r="I29" s="42"/>
       <c r="J29" s="41" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="K29" s="41"/>
       <c r="L29" s="41"/>
@@ -4211,20 +4358,20 @@
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="39" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B30" s="39"/>
       <c r="C30" s="39"/>
       <c r="D30" s="39"/>
       <c r="E30" s="40" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="F30" s="40"/>
       <c r="G30" s="40"/>
       <c r="H30" s="40"/>
       <c r="I30" s="40"/>
       <c r="J30" s="39" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="K30" s="39"/>
       <c r="L30" s="39"/>
@@ -4233,20 +4380,20 @@
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="41" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B31" s="41"/>
       <c r="C31" s="41"/>
       <c r="D31" s="41"/>
       <c r="E31" s="42" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="F31" s="42"/>
       <c r="G31" s="42"/>
       <c r="H31" s="42"/>
       <c r="I31" s="42"/>
       <c r="J31" s="41" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="K31" s="41"/>
       <c r="L31" s="41"/>
@@ -4255,20 +4402,20 @@
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="39" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B32" s="39"/>
       <c r="C32" s="39"/>
       <c r="D32" s="39"/>
       <c r="E32" s="40" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="F32" s="40"/>
       <c r="G32" s="40"/>
       <c r="H32" s="40"/>
       <c r="I32" s="40"/>
       <c r="J32" s="39" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="K32" s="39"/>
       <c r="L32" s="39"/>
@@ -4277,20 +4424,20 @@
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="41" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B33" s="41"/>
       <c r="C33" s="41"/>
       <c r="D33" s="41"/>
       <c r="E33" s="42" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="F33" s="42"/>
       <c r="G33" s="42"/>
       <c r="H33" s="42"/>
       <c r="I33" s="42"/>
       <c r="J33" s="41" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="K33" s="41"/>
       <c r="L33" s="41"/>
@@ -4299,20 +4446,20 @@
     </row>
     <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="39" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B34" s="39"/>
       <c r="C34" s="39"/>
       <c r="D34" s="39"/>
       <c r="E34" s="40" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F34" s="40"/>
       <c r="G34" s="40"/>
       <c r="H34" s="40"/>
       <c r="I34" s="40"/>
       <c r="J34" s="39" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="K34" s="39"/>
       <c r="L34" s="39"/>
@@ -4321,20 +4468,20 @@
     </row>
     <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="41" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B35" s="41"/>
       <c r="C35" s="41"/>
       <c r="D35" s="41"/>
       <c r="E35" s="42" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="F35" s="42"/>
       <c r="G35" s="42"/>
       <c r="H35" s="42"/>
       <c r="I35" s="42"/>
       <c r="J35" s="41" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="K35" s="41"/>
       <c r="L35" s="41"/>
@@ -4343,20 +4490,20 @@
     </row>
     <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="39" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B36" s="39"/>
       <c r="C36" s="39"/>
       <c r="D36" s="39"/>
       <c r="E36" s="40" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="F36" s="40"/>
       <c r="G36" s="40"/>
       <c r="H36" s="40"/>
       <c r="I36" s="40"/>
       <c r="J36" s="39" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="K36" s="39"/>
       <c r="L36" s="39"/>
@@ -4365,20 +4512,20 @@
     </row>
     <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="41" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B37" s="41"/>
       <c r="C37" s="41"/>
       <c r="D37" s="41"/>
       <c r="E37" s="42" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="F37" s="42"/>
       <c r="G37" s="42"/>
       <c r="H37" s="42"/>
       <c r="I37" s="42"/>
       <c r="J37" s="41" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="K37" s="41"/>
       <c r="L37" s="41"/>
@@ -4387,20 +4534,20 @@
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="39" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B38" s="39"/>
       <c r="C38" s="39"/>
       <c r="D38" s="39"/>
       <c r="E38" s="40" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="F38" s="40"/>
       <c r="G38" s="40"/>
       <c r="H38" s="40"/>
       <c r="I38" s="40"/>
       <c r="J38" s="39" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="K38" s="39"/>
       <c r="L38" s="39"/>
@@ -4409,20 +4556,20 @@
     </row>
     <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="41" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B39" s="41"/>
       <c r="C39" s="41"/>
       <c r="D39" s="41"/>
       <c r="E39" s="42" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F39" s="42"/>
       <c r="G39" s="42"/>
       <c r="H39" s="42"/>
       <c r="I39" s="42"/>
       <c r="J39" s="41" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="K39" s="41"/>
       <c r="L39" s="41"/>
@@ -4444,7 +4591,7 @@
       <c r="H40" s="44"/>
       <c r="I40" s="44"/>
       <c r="J40" s="43" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="K40" s="43"/>
       <c r="L40" s="43"/>

</xml_diff>

<commit_message>
feat(reporting): adopt REPORTING-UX-RATIONALIZATION-1 Rev 2.0
- unify dashboard and Excel period binding
- adopt Gregorian month/year reporting
- add Refund Analytics presentation
- rationalize reporting hierarchy
- standardize executive KPI terminology
- preserve financial laws and reporting SSOT

Production Certified
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -7,16 +7,16 @@
     <sheet sheetId="1" name="Cover" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Executive Summary" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Financial Summary" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Payment Method Analysis" state="visible" r:id="rId7"/>
+    <sheet sheetId="4" name="Payment Analytics" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Order Sales" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Check Revenue Trends" state="visible" r:id="rId9"/>
+    <sheet sheetId="6" name="Sales Trends" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="151">
   <si>
     <t>MINEUQR</t>
   </si>
@@ -60,10 +60,10 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>26 Jul 2026, 13:54</t>
-  </si>
-  <si>
-    <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Payment Method Analysis  ·  Order Sales  ·  Check Revenue Trends</t>
+    <t>27 Jul 2026, 14:30</t>
+  </si>
+  <si>
+    <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Payment Analytics  ·  Order Sales  ·  Sales Trends</t>
   </si>
   <si>
     <t>Confidential — Internal Use  ·  Prepared by MineuQR</t>
@@ -72,126 +72,138 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  26 Jul 2026, 13:54</t>
-  </si>
-  <si>
-    <t>AT A GLANCE</t>
-  </si>
-  <si>
-    <t>How is the restaurant performing operationally?</t>
-  </si>
-  <si>
-    <t>ORDERS SERVED</t>
-  </si>
-  <si>
-    <t>From completed kitchen orders — your Order Sales story for this period.</t>
+    <t>Monthly Report  ·  July 2026  ·  27 Jul 2026, 14:30</t>
+  </si>
+  <si>
+    <t>EXECUTIVE KPIS</t>
+  </si>
+  <si>
+    <t>How is the restaurant performing this period?</t>
+  </si>
+  <si>
+    <t>Gross Sales, Net Sales, refunds, tax, and order averages for the selected period.</t>
+  </si>
+  <si>
+    <t>Gross Sales</t>
+  </si>
+  <si>
+    <t>Net Sales</t>
+  </si>
+  <si>
+    <t>Refund Amount</t>
+  </si>
+  <si>
+    <t>14,612.50 ر.س</t>
+  </si>
+  <si>
+    <t>0.00 ر.س</t>
+  </si>
+  <si>
+    <t>Paid check totals for this period (gross)</t>
+  </si>
+  <si>
+    <t>Gross Sales after published refunds</t>
+  </si>
+  <si>
+    <t>Total refunded (published Settlement Records)</t>
+  </si>
+  <si>
+    <t>Refund Rate</t>
+  </si>
+  <si>
+    <t>Tax Collected</t>
+  </si>
+  <si>
+    <t>Orders</t>
+  </si>
+  <si>
+    <t>0.00%</t>
+  </si>
+  <si>
+    <t>2,191.91 ر.س</t>
+  </si>
+  <si>
+    <t>103</t>
+  </si>
+  <si>
+    <t>Refund Amount as a percent of Gross Sales</t>
+  </si>
+  <si>
+    <t>Tax on paid checks (frozen snapshot)</t>
+  </si>
+  <si>
+    <t>All orders placed in this period</t>
+  </si>
+  <si>
+    <t>Average Order</t>
+  </si>
+  <si>
+    <t>Average Check</t>
+  </si>
+  <si>
+    <t>215.98 ر.س</t>
+  </si>
+  <si>
+    <t>214.89 ر.س</t>
+  </si>
+  <si>
+    <t>Typical size of a completed order</t>
+  </si>
+  <si>
+    <t>Typical size of a paid check</t>
+  </si>
+  <si>
+    <t>Details: Financial Performance, Refund Analytics, Payment Analytics, Order Sales, and Trends follow. Operational rollups are on dedicated sheets.</t>
+  </si>
+  <si>
+    <t>Financial Summary</t>
+  </si>
+  <si>
+    <t>Monthly Report  ·  July 2026</t>
+  </si>
+  <si>
+    <t>MONEY COLLECTED</t>
+  </si>
+  <si>
+    <t>Paid guest checks for this reporting period — Gross Sales. Net Sales subtracts Refund Amount.</t>
+  </si>
+  <si>
+    <t>FINANCIAL PERFORMANCE</t>
+  </si>
+  <si>
+    <t>Paid Checks</t>
+  </si>
+  <si>
+    <t>68</t>
+  </si>
+  <si>
+    <t>Refund Count</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>TAX</t>
+  </si>
+  <si>
+    <t>Tax Collected covers the full reporting period — total tax from all paid checks in range (not a subset of sections).</t>
+  </si>
+  <si>
+    <t>ORDER SALES DETAIL</t>
   </si>
   <si>
     <t>Order Sales</t>
   </si>
   <si>
+    <t>19,222.00 ر.س</t>
+  </si>
+  <si>
     <t>Completed Orders</t>
   </si>
   <si>
-    <t>Average Order</t>
-  </si>
-  <si>
-    <t>19,222.00 ر.س</t>
-  </si>
-  <si>
     <t>89</t>
   </si>
   <si>
-    <t>215.98 ر.س</t>
-  </si>
-  <si>
-    <t>Value of orders that were completed (served)</t>
-  </si>
-  <si>
-    <t>How many orders were completed (served)</t>
-  </si>
-  <si>
-    <t>Typical size of a completed order</t>
-  </si>
-  <si>
-    <t>Check Revenue (Gross), Net Revenue, Refund Publications, Paid Checks, Average Check, and Tax Collected are in Financial Summary. Payment and refund mix are in Payment Method Analysis.</t>
-  </si>
-  <si>
-    <t>Financial Summary</t>
-  </si>
-  <si>
-    <t>Monthly Report  ·  July 2026</t>
-  </si>
-  <si>
-    <t>MONEY COLLECTED</t>
-  </si>
-  <si>
-    <t>Paid guest checks for this reporting period — Gross Check Revenue. Net Revenue subtracts Refund Publications.</t>
-  </si>
-  <si>
-    <t>CHECK REVENUE DETAIL</t>
-  </si>
-  <si>
-    <t>Check Revenue</t>
-  </si>
-  <si>
-    <t>14,612.50 ر.س</t>
-  </si>
-  <si>
-    <t>Refund Publications</t>
-  </si>
-  <si>
-    <t>0.00 ر.س</t>
-  </si>
-  <si>
-    <t>Net Revenue</t>
-  </si>
-  <si>
-    <t>Refund Rate</t>
-  </si>
-  <si>
-    <t>0.00%</t>
-  </si>
-  <si>
-    <t>Paid Checks</t>
-  </si>
-  <si>
-    <t>68</t>
-  </si>
-  <si>
-    <t>Refund Count</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>Average Check</t>
-  </si>
-  <si>
-    <t>214.89 ر.س</t>
-  </si>
-  <si>
-    <t>TAX</t>
-  </si>
-  <si>
-    <t>Tax Collected covers the full reporting period — total tax from all paid checks in range (not a subset of sections).</t>
-  </si>
-  <si>
-    <t>Tax Collected</t>
-  </si>
-  <si>
-    <t>2,191.91 ر.س</t>
-  </si>
-  <si>
-    <t>ORDER SALES DETAIL</t>
-  </si>
-  <si>
-    <t>Orders</t>
-  </si>
-  <si>
-    <t>103</t>
-  </si>
-  <si>
     <t>ADJUSTMENTS</t>
   </si>
   <si>
@@ -216,19 +228,19 @@
     <t>REPORTING BASIS</t>
   </si>
   <si>
-    <t>Check Revenue = sum of paid Check totals (not Order Sales).</t>
-  </si>
-  <si>
-    <t>Order Sales = completed (served) order totals from Order Read (not Check Revenue).</t>
+    <t>Gross Sales = sum of paid Check totals (not Order Sales).</t>
+  </si>
+  <si>
+    <t>Order Sales = completed (served) order totals from Order Read (not Gross Sales).</t>
   </si>
   <si>
     <t>SAR (ر.س)</t>
   </si>
   <si>
-    <t>Payment Method Analysis</t>
-  </si>
-  <si>
-    <t>Payment mix is from settlement tenders. Check Revenue remains Gross from paid checks; refund tenders are listed separately and do not replace Check Revenue.</t>
+    <t>Payment Analytics</t>
+  </si>
+  <si>
+    <t>Payment mix is from settlement tenders. Gross Sales remains from paid checks; refund tenders are listed separately and do not replace Gross Sales.</t>
   </si>
   <si>
     <t>PAYMENT MIX</t>
@@ -240,7 +252,7 @@
     <t>Complimentary</t>
   </si>
   <si>
-    <t>PAYMENT METHOD ANALYSIS</t>
+    <t>PAYMENT ANALYTICS</t>
   </si>
   <si>
     <t>Payment Method</t>
@@ -294,7 +306,7 @@
     <t>Other</t>
   </si>
   <si>
-    <t>REFUND MIX BY PAYMENT METHOD</t>
+    <t>REFUND BY PAYMENT METHOD</t>
   </si>
   <si>
     <t>Refund Tender Total</t>
@@ -408,13 +420,13 @@
     <t>1,646.00 ر.س</t>
   </si>
   <si>
-    <t>Check Revenue Trends</t>
-  </si>
-  <si>
-    <t>Monthly Report  ·  Daily Check Revenue — July 2026</t>
-  </si>
-  <si>
-    <t>CHECK REVENUE TRENDS</t>
+    <t>Sales Trends</t>
+  </si>
+  <si>
+    <t>Monthly Report  ·  Daily Gross Sales — July 2026</t>
+  </si>
+  <si>
+    <t>SALES TRENDS</t>
   </si>
   <si>
     <t>800.00 ر.س</t>
@@ -1698,7 +1710,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="10.2" customWidth="1"/>
@@ -1810,7 +1822,7 @@
     </row>
     <row r="8" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="19"/>
@@ -1828,7 +1840,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9" s="21"/>
       <c r="C9" s="21"/>
@@ -1846,19 +1858,19 @@
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
       <c r="D10" s="22"/>
       <c r="F10" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G10" s="22"/>
       <c r="H10" s="22"/>
       <c r="I10" s="22"/>
       <c r="K10" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L10" s="22"/>
       <c r="M10" s="22"/>
@@ -1866,19 +1878,19 @@
     </row>
     <row r="11" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B11" s="23"/>
       <c r="C11" s="23"/>
       <c r="D11" s="23"/>
       <c r="F11" s="23" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G11" s="23"/>
       <c r="H11" s="23"/>
       <c r="I11" s="23"/>
       <c r="K11" s="23" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="L11" s="23"/>
       <c r="M11" s="23"/>
@@ -1886,19 +1898,19 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B12" s="24"/>
       <c r="C12" s="24"/>
       <c r="D12" s="24"/>
       <c r="F12" s="24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G12" s="24"/>
       <c r="H12" s="24"/>
       <c r="I12" s="24"/>
       <c r="K12" s="24" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="L12" s="24"/>
       <c r="M12" s="24"/>
@@ -1918,26 +1930,152 @@
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
     </row>
+    <row r="15" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="F15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22"/>
+      <c r="K15" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="L15" s="22"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="22"/>
+    </row>
     <row r="16" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="25"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25"/>
-      <c r="L16" s="25"/>
-      <c r="M16" s="25"/>
-      <c r="N16" s="25"/>
+      <c r="A16" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="F16" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="K16" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="L16" s="23"/>
+      <c r="M16" s="23"/>
+      <c r="N16" s="23"/>
+    </row>
+    <row r="17" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="F17" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="24"/>
+      <c r="K17" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="L17" s="24"/>
+      <c r="M17" s="24"/>
+      <c r="N17" s="24"/>
+    </row>
+    <row r="18" ht="5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3"/>
+      <c r="N18" s="3"/>
+    </row>
+    <row r="20" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="F20" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+    </row>
+    <row r="21" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="F21" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+    </row>
+    <row r="22" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="F22" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="24"/>
+    </row>
+    <row r="23" ht="5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+    </row>
+    <row r="26" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" s="25"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
+      <c r="I26" s="25"/>
+      <c r="J26" s="25"/>
+      <c r="K26" s="25"/>
+      <c r="L26" s="25"/>
+      <c r="M26" s="25"/>
+      <c r="N26" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="39">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A5:N5"/>
@@ -1956,7 +2094,27 @@
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="F13:I13"/>
     <mergeCell ref="K13:N13"/>
-    <mergeCell ref="A16:N16"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="K15:N15"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="K16:N16"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="K17:N17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="K18:N18"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="F22:I22"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="A26:N26"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.55" bottom="0.55" header="0.25" footer="0.3"/>
@@ -1980,7 +2138,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -1998,7 +2156,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2048,7 +2206,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -2066,7 +2224,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="B6" s="21"/>
       <c r="C6" s="21"/>
@@ -2084,7 +2242,7 @@
     </row>
     <row r="7" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="19"/>
@@ -2102,7 +2260,7 @@
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="B8" s="26"/>
       <c r="C8" s="26"/>
@@ -2112,7 +2270,7 @@
       <c r="G8" s="26"/>
       <c r="H8" s="26"/>
       <c r="I8" s="27" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="J8" s="27"/>
       <c r="K8" s="27"/>
@@ -2122,7 +2280,7 @@
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="B9" s="28"/>
       <c r="C9" s="28"/>
@@ -2132,7 +2290,7 @@
       <c r="G9" s="28"/>
       <c r="H9" s="28"/>
       <c r="I9" s="29" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="J9" s="29"/>
       <c r="K9" s="29"/>
@@ -2142,7 +2300,7 @@
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="26" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="B10" s="26"/>
       <c r="C10" s="26"/>
@@ -2152,7 +2310,7 @@
       <c r="G10" s="26"/>
       <c r="H10" s="26"/>
       <c r="I10" s="27" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="J10" s="27"/>
       <c r="K10" s="27"/>
@@ -2162,7 +2320,7 @@
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="28" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B11" s="28"/>
       <c r="C11" s="28"/>
@@ -2172,7 +2330,7 @@
       <c r="G11" s="28"/>
       <c r="H11" s="28"/>
       <c r="I11" s="29" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="J11" s="29"/>
       <c r="K11" s="29"/>
@@ -2182,7 +2340,7 @@
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="26" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B12" s="26"/>
       <c r="C12" s="26"/>
@@ -2192,7 +2350,7 @@
       <c r="G12" s="26"/>
       <c r="H12" s="26"/>
       <c r="I12" s="27" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="J12" s="27"/>
       <c r="K12" s="27"/>
@@ -2202,7 +2360,7 @@
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="28" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B13" s="28"/>
       <c r="C13" s="28"/>
@@ -2212,7 +2370,7 @@
       <c r="G13" s="28"/>
       <c r="H13" s="28"/>
       <c r="I13" s="29" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="J13" s="29"/>
       <c r="K13" s="29"/>
@@ -2222,7 +2380,7 @@
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="B14" s="26"/>
       <c r="C14" s="26"/>
@@ -2232,7 +2390,7 @@
       <c r="G14" s="26"/>
       <c r="H14" s="26"/>
       <c r="I14" s="27" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="J14" s="27"/>
       <c r="K14" s="27"/>
@@ -2242,7 +2400,7 @@
     </row>
     <row r="16" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B16" s="19"/>
       <c r="C16" s="19"/>
@@ -2260,7 +2418,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B17" s="21"/>
       <c r="C17" s="21"/>
@@ -2278,7 +2436,7 @@
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="30" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="B18" s="30"/>
       <c r="C18" s="30"/>
@@ -2288,7 +2446,7 @@
       <c r="G18" s="30"/>
       <c r="H18" s="30"/>
       <c r="I18" s="31" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="J18" s="31"/>
       <c r="K18" s="31"/>
@@ -2298,7 +2456,7 @@
     </row>
     <row r="20" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B20" s="19"/>
       <c r="C20" s="19"/>
@@ -2316,7 +2474,7 @@
     </row>
     <row r="21" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="26" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="26"/>
@@ -2326,7 +2484,7 @@
       <c r="G21" s="26"/>
       <c r="H21" s="26"/>
       <c r="I21" s="27" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="J21" s="27"/>
       <c r="K21" s="27"/>
@@ -2336,7 +2494,7 @@
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="28" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="B22" s="28"/>
       <c r="C22" s="28"/>
@@ -2346,7 +2504,7 @@
       <c r="G22" s="28"/>
       <c r="H22" s="28"/>
       <c r="I22" s="29" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="J22" s="29"/>
       <c r="K22" s="29"/>
@@ -2356,7 +2514,7 @@
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="B23" s="26"/>
       <c r="C23" s="26"/>
@@ -2366,7 +2524,7 @@
       <c r="G23" s="26"/>
       <c r="H23" s="26"/>
       <c r="I23" s="27" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="J23" s="27"/>
       <c r="K23" s="27"/>
@@ -2376,7 +2534,7 @@
     </row>
     <row r="24" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="28" t="s">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="B24" s="28"/>
       <c r="C24" s="28"/>
@@ -2386,7 +2544,7 @@
       <c r="G24" s="28"/>
       <c r="H24" s="28"/>
       <c r="I24" s="29" t="s">
-        <v>27</v>
+        <v>61</v>
       </c>
       <c r="J24" s="29"/>
       <c r="K24" s="29"/>
@@ -2396,7 +2554,7 @@
     </row>
     <row r="26" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B26" s="19"/>
       <c r="C26" s="19"/>
@@ -2414,7 +2572,7 @@
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="26" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B27" s="26"/>
       <c r="C27" s="26"/>
@@ -2424,7 +2582,7 @@
       <c r="G27" s="26"/>
       <c r="H27" s="26"/>
       <c r="I27" s="27" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="J27" s="27"/>
       <c r="K27" s="27"/>
@@ -2434,7 +2592,7 @@
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="28" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B28" s="28"/>
       <c r="C28" s="28"/>
@@ -2444,7 +2602,7 @@
       <c r="G28" s="28"/>
       <c r="H28" s="28"/>
       <c r="I28" s="29" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J28" s="29"/>
       <c r="K28" s="29"/>
@@ -2454,7 +2612,7 @@
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="26" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B29" s="26"/>
       <c r="C29" s="26"/>
@@ -2464,7 +2622,7 @@
       <c r="G29" s="26"/>
       <c r="H29" s="26"/>
       <c r="I29" s="27" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J29" s="27"/>
       <c r="K29" s="27"/>
@@ -2474,7 +2632,7 @@
     </row>
     <row r="31" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
@@ -2492,7 +2650,7 @@
     </row>
     <row r="32" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="B32" s="26"/>
       <c r="C32" s="26"/>
@@ -2502,7 +2660,7 @@
       <c r="G32" s="26"/>
       <c r="H32" s="26"/>
       <c r="I32" s="27" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J32" s="27"/>
       <c r="K32" s="27"/>
@@ -2512,7 +2670,7 @@
     </row>
     <row r="33" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="28" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="B33" s="28"/>
       <c r="C33" s="28"/>
@@ -2522,7 +2680,7 @@
       <c r="G33" s="28"/>
       <c r="H33" s="28"/>
       <c r="I33" s="29" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="J33" s="29"/>
       <c r="K33" s="29"/>
@@ -2542,7 +2700,7 @@
       <c r="G34" s="26"/>
       <c r="H34" s="26"/>
       <c r="I34" s="27" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="J34" s="27"/>
       <c r="K34" s="27"/>
@@ -2665,7 +2823,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -2683,7 +2841,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2733,7 +2891,7 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B5" s="21"/>
       <c r="C5" s="21"/>
@@ -2751,7 +2909,7 @@
     </row>
     <row r="7" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="19"/>
@@ -2769,7 +2927,7 @@
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B8" s="26"/>
       <c r="C8" s="26"/>
@@ -2779,7 +2937,7 @@
       <c r="G8" s="26"/>
       <c r="H8" s="26"/>
       <c r="I8" s="27" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="J8" s="27"/>
       <c r="K8" s="27"/>
@@ -2789,7 +2947,7 @@
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B9" s="28"/>
       <c r="C9" s="28"/>
@@ -2799,7 +2957,7 @@
       <c r="G9" s="28"/>
       <c r="H9" s="28"/>
       <c r="I9" s="29" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J9" s="29"/>
       <c r="K9" s="29"/>
@@ -2809,7 +2967,7 @@
     </row>
     <row r="11" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B11" s="19"/>
       <c r="C11" s="19"/>
@@ -2827,119 +2985,119 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="32" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B12" s="32"/>
       <c r="C12" s="32"/>
       <c r="D12" s="32" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E12" s="32"/>
       <c r="F12" s="32"/>
       <c r="G12" s="32" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="H12" s="32"/>
       <c r="I12" s="32" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="J12" s="32"/>
       <c r="K12" s="32" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="L12" s="32"/>
       <c r="M12" s="32" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="N12" s="32"/>
     </row>
     <row r="13" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="33"/>
       <c r="D13" s="34" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E13" s="34"/>
       <c r="F13" s="34"/>
       <c r="G13" s="33" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="H13" s="33"/>
       <c r="I13" s="33" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="J13" s="33"/>
       <c r="K13" s="33" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="L13" s="33"/>
       <c r="M13" s="33" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="N13" s="33"/>
     </row>
     <row r="14" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="33" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="33"/>
       <c r="D14" s="34" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="E14" s="34"/>
       <c r="F14" s="34"/>
       <c r="G14" s="33" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H14" s="33"/>
       <c r="I14" s="33" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="J14" s="33"/>
       <c r="K14" s="33" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="L14" s="33"/>
       <c r="M14" s="33" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="N14" s="33"/>
     </row>
     <row r="15" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="35" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B15" s="35"/>
       <c r="C15" s="35"/>
       <c r="D15" s="36" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="E15" s="36"/>
       <c r="F15" s="36"/>
       <c r="G15" s="35" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H15" s="35"/>
       <c r="I15" s="35" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="J15" s="35"/>
       <c r="K15" s="35" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="L15" s="35"/>
       <c r="M15" s="35" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="N15" s="35"/>
     </row>
     <row r="17" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B17" s="19"/>
       <c r="C17" s="19"/>
@@ -2957,7 +3115,7 @@
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
@@ -2967,7 +3125,7 @@
       <c r="G18" s="26"/>
       <c r="H18" s="26"/>
       <c r="I18" s="27" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="J18" s="27"/>
       <c r="K18" s="27"/>
@@ -3036,7 +3194,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -3054,7 +3212,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3088,7 +3246,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -3378,7 +3536,7 @@
     </row>
     <row r="23" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B23" s="19"/>
       <c r="C23" s="19"/>
@@ -3396,22 +3554,22 @@
     </row>
     <row r="24" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="37" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B24" s="37"/>
       <c r="C24" s="37"/>
       <c r="D24" s="38" t="s">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="E24" s="38"/>
       <c r="F24" s="38"/>
       <c r="G24" s="38" t="s">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="H24" s="38"/>
       <c r="I24" s="38"/>
       <c r="J24" s="38" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="K24" s="38"/>
       <c r="L24" s="38"/>
@@ -3420,22 +3578,22 @@
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="39" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B25" s="39"/>
       <c r="C25" s="39"/>
       <c r="D25" s="39" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E25" s="39"/>
       <c r="F25" s="39"/>
       <c r="G25" s="39" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H25" s="39"/>
       <c r="I25" s="39"/>
       <c r="J25" s="40" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="K25" s="40"/>
       <c r="L25" s="40"/>
@@ -3444,22 +3602,22 @@
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="41" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B26" s="41"/>
       <c r="C26" s="41"/>
       <c r="D26" s="41" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E26" s="41"/>
       <c r="F26" s="41"/>
       <c r="G26" s="41" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H26" s="41"/>
       <c r="I26" s="41"/>
       <c r="J26" s="42" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="K26" s="42"/>
       <c r="L26" s="42"/>
@@ -3468,22 +3626,22 @@
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="39" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B27" s="39"/>
       <c r="C27" s="39"/>
       <c r="D27" s="39" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E27" s="39"/>
       <c r="F27" s="39"/>
       <c r="G27" s="39" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="H27" s="39"/>
       <c r="I27" s="39"/>
       <c r="J27" s="40" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="K27" s="40"/>
       <c r="L27" s="40"/>
@@ -3492,22 +3650,22 @@
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="41" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B28" s="41"/>
       <c r="C28" s="41"/>
       <c r="D28" s="41" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E28" s="41"/>
       <c r="F28" s="41"/>
       <c r="G28" s="41" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H28" s="41"/>
       <c r="I28" s="41"/>
       <c r="J28" s="42" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="K28" s="42"/>
       <c r="L28" s="42"/>
@@ -3516,22 +3674,22 @@
     </row>
     <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="39" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B29" s="39"/>
       <c r="C29" s="39"/>
       <c r="D29" s="39" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E29" s="39"/>
       <c r="F29" s="39"/>
       <c r="G29" s="39" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H29" s="39"/>
       <c r="I29" s="39"/>
       <c r="J29" s="40" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="K29" s="40"/>
       <c r="L29" s="40"/>
@@ -3540,22 +3698,22 @@
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="41" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B30" s="41"/>
       <c r="C30" s="41"/>
       <c r="D30" s="41" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E30" s="41"/>
       <c r="F30" s="41"/>
       <c r="G30" s="41" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H30" s="41"/>
       <c r="I30" s="41"/>
       <c r="J30" s="42" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="K30" s="42"/>
       <c r="L30" s="42"/>
@@ -3564,22 +3722,22 @@
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="39" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B31" s="39"/>
       <c r="C31" s="39"/>
       <c r="D31" s="39" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E31" s="39"/>
       <c r="F31" s="39"/>
       <c r="G31" s="39" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="H31" s="39"/>
       <c r="I31" s="39"/>
       <c r="J31" s="40" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="K31" s="40"/>
       <c r="L31" s="40"/>
@@ -3588,22 +3746,22 @@
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="41" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B32" s="41"/>
       <c r="C32" s="41"/>
       <c r="D32" s="41" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E32" s="41"/>
       <c r="F32" s="41"/>
       <c r="G32" s="41" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H32" s="41"/>
       <c r="I32" s="41"/>
       <c r="J32" s="42" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="K32" s="42"/>
       <c r="L32" s="42"/>
@@ -3612,22 +3770,22 @@
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="39" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B33" s="39"/>
       <c r="C33" s="39"/>
       <c r="D33" s="39" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E33" s="39"/>
       <c r="F33" s="39"/>
       <c r="G33" s="39" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H33" s="39"/>
       <c r="I33" s="39"/>
       <c r="J33" s="40" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="K33" s="40"/>
       <c r="L33" s="40"/>
@@ -3636,22 +3794,22 @@
     </row>
     <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="41" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B34" s="41"/>
       <c r="C34" s="41"/>
       <c r="D34" s="41" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E34" s="41"/>
       <c r="F34" s="41"/>
       <c r="G34" s="41" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H34" s="41"/>
       <c r="I34" s="41"/>
       <c r="J34" s="42" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="K34" s="42"/>
       <c r="L34" s="42"/>
@@ -3660,22 +3818,22 @@
     </row>
     <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="39" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B35" s="39"/>
       <c r="C35" s="39"/>
       <c r="D35" s="39" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E35" s="39"/>
       <c r="F35" s="39"/>
       <c r="G35" s="39" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="H35" s="39"/>
       <c r="I35" s="39"/>
       <c r="J35" s="40" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="K35" s="40"/>
       <c r="L35" s="40"/>
@@ -3684,22 +3842,22 @@
     </row>
     <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="41" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B36" s="41"/>
       <c r="C36" s="41"/>
       <c r="D36" s="41" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E36" s="41"/>
       <c r="F36" s="41"/>
       <c r="G36" s="41" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H36" s="41"/>
       <c r="I36" s="41"/>
       <c r="J36" s="42" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="K36" s="42"/>
       <c r="L36" s="42"/>
@@ -3708,22 +3866,22 @@
     </row>
     <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="39" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B37" s="39"/>
       <c r="C37" s="39"/>
       <c r="D37" s="39" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E37" s="39"/>
       <c r="F37" s="39"/>
       <c r="G37" s="39" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H37" s="39"/>
       <c r="I37" s="39"/>
       <c r="J37" s="40" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="K37" s="40"/>
       <c r="L37" s="40"/>
@@ -3732,22 +3890,22 @@
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="41" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B38" s="41"/>
       <c r="C38" s="41"/>
       <c r="D38" s="41" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E38" s="41"/>
       <c r="F38" s="41"/>
       <c r="G38" s="41" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H38" s="41"/>
       <c r="I38" s="41"/>
       <c r="J38" s="42" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="K38" s="42"/>
       <c r="L38" s="42"/>
@@ -3761,17 +3919,17 @@
       <c r="B39" s="43"/>
       <c r="C39" s="43"/>
       <c r="D39" s="43" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="E39" s="43"/>
       <c r="F39" s="43"/>
       <c r="G39" s="43" t="s">
-        <v>27</v>
+        <v>61</v>
       </c>
       <c r="H39" s="43"/>
       <c r="I39" s="43"/>
       <c r="J39" s="44" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="K39" s="44"/>
       <c r="L39" s="44"/>
@@ -3872,7 +4030,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -3890,7 +4048,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3924,7 +4082,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19"/>
@@ -4230,7 +4388,7 @@
     </row>
     <row r="24" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
@@ -4248,20 +4406,20 @@
     </row>
     <row r="25" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="37" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B25" s="37"/>
       <c r="C25" s="37"/>
       <c r="D25" s="37"/>
       <c r="E25" s="38" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="F25" s="38"/>
       <c r="G25" s="38"/>
       <c r="H25" s="38"/>
       <c r="I25" s="38"/>
       <c r="J25" s="38" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="K25" s="38"/>
       <c r="L25" s="38"/>
@@ -4270,20 +4428,20 @@
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="39" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B26" s="39"/>
       <c r="C26" s="39"/>
       <c r="D26" s="39"/>
       <c r="E26" s="40" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="F26" s="40"/>
       <c r="G26" s="40"/>
       <c r="H26" s="40"/>
       <c r="I26" s="40"/>
       <c r="J26" s="39" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="K26" s="39"/>
       <c r="L26" s="39"/>
@@ -4292,20 +4450,20 @@
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="41" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B27" s="41"/>
       <c r="C27" s="41"/>
       <c r="D27" s="41"/>
       <c r="E27" s="42" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="F27" s="42"/>
       <c r="G27" s="42"/>
       <c r="H27" s="42"/>
       <c r="I27" s="42"/>
       <c r="J27" s="41" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="K27" s="41"/>
       <c r="L27" s="41"/>
@@ -4314,20 +4472,20 @@
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B28" s="39"/>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
       <c r="E28" s="40" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="F28" s="40"/>
       <c r="G28" s="40"/>
       <c r="H28" s="40"/>
       <c r="I28" s="40"/>
       <c r="J28" s="39" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="K28" s="39"/>
       <c r="L28" s="39"/>
@@ -4336,20 +4494,20 @@
     </row>
     <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="41" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B29" s="41"/>
       <c r="C29" s="41"/>
       <c r="D29" s="41"/>
       <c r="E29" s="42" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F29" s="42"/>
       <c r="G29" s="42"/>
       <c r="H29" s="42"/>
       <c r="I29" s="42"/>
       <c r="J29" s="41" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="K29" s="41"/>
       <c r="L29" s="41"/>
@@ -4358,20 +4516,20 @@
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="39" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B30" s="39"/>
       <c r="C30" s="39"/>
       <c r="D30" s="39"/>
       <c r="E30" s="40" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="F30" s="40"/>
       <c r="G30" s="40"/>
       <c r="H30" s="40"/>
       <c r="I30" s="40"/>
       <c r="J30" s="39" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="K30" s="39"/>
       <c r="L30" s="39"/>
@@ -4380,20 +4538,20 @@
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="41" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B31" s="41"/>
       <c r="C31" s="41"/>
       <c r="D31" s="41"/>
       <c r="E31" s="42" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F31" s="42"/>
       <c r="G31" s="42"/>
       <c r="H31" s="42"/>
       <c r="I31" s="42"/>
       <c r="J31" s="41" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="K31" s="41"/>
       <c r="L31" s="41"/>
@@ -4402,20 +4560,20 @@
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="39" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B32" s="39"/>
       <c r="C32" s="39"/>
       <c r="D32" s="39"/>
       <c r="E32" s="40" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F32" s="40"/>
       <c r="G32" s="40"/>
       <c r="H32" s="40"/>
       <c r="I32" s="40"/>
       <c r="J32" s="39" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="K32" s="39"/>
       <c r="L32" s="39"/>
@@ -4424,20 +4582,20 @@
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="41" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B33" s="41"/>
       <c r="C33" s="41"/>
       <c r="D33" s="41"/>
       <c r="E33" s="42" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F33" s="42"/>
       <c r="G33" s="42"/>
       <c r="H33" s="42"/>
       <c r="I33" s="42"/>
       <c r="J33" s="41" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="K33" s="41"/>
       <c r="L33" s="41"/>
@@ -4446,20 +4604,20 @@
     </row>
     <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="39" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B34" s="39"/>
       <c r="C34" s="39"/>
       <c r="D34" s="39"/>
       <c r="E34" s="40" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F34" s="40"/>
       <c r="G34" s="40"/>
       <c r="H34" s="40"/>
       <c r="I34" s="40"/>
       <c r="J34" s="39" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="K34" s="39"/>
       <c r="L34" s="39"/>
@@ -4468,20 +4626,20 @@
     </row>
     <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="41" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B35" s="41"/>
       <c r="C35" s="41"/>
       <c r="D35" s="41"/>
       <c r="E35" s="42" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="F35" s="42"/>
       <c r="G35" s="42"/>
       <c r="H35" s="42"/>
       <c r="I35" s="42"/>
       <c r="J35" s="41" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="K35" s="41"/>
       <c r="L35" s="41"/>
@@ -4490,20 +4648,20 @@
     </row>
     <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="39" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B36" s="39"/>
       <c r="C36" s="39"/>
       <c r="D36" s="39"/>
       <c r="E36" s="40" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F36" s="40"/>
       <c r="G36" s="40"/>
       <c r="H36" s="40"/>
       <c r="I36" s="40"/>
       <c r="J36" s="39" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="K36" s="39"/>
       <c r="L36" s="39"/>
@@ -4512,20 +4670,20 @@
     </row>
     <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="41" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B37" s="41"/>
       <c r="C37" s="41"/>
       <c r="D37" s="41"/>
       <c r="E37" s="42" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="F37" s="42"/>
       <c r="G37" s="42"/>
       <c r="H37" s="42"/>
       <c r="I37" s="42"/>
       <c r="J37" s="41" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="K37" s="41"/>
       <c r="L37" s="41"/>
@@ -4534,20 +4692,20 @@
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="39" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B38" s="39"/>
       <c r="C38" s="39"/>
       <c r="D38" s="39"/>
       <c r="E38" s="40" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="F38" s="40"/>
       <c r="G38" s="40"/>
       <c r="H38" s="40"/>
       <c r="I38" s="40"/>
       <c r="J38" s="39" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="K38" s="39"/>
       <c r="L38" s="39"/>
@@ -4556,20 +4714,20 @@
     </row>
     <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="41" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B39" s="41"/>
       <c r="C39" s="41"/>
       <c r="D39" s="41"/>
       <c r="E39" s="42" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="F39" s="42"/>
       <c r="G39" s="42"/>
       <c r="H39" s="42"/>
       <c r="I39" s="42"/>
       <c r="J39" s="41" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="K39" s="41"/>
       <c r="L39" s="41"/>
@@ -4584,14 +4742,14 @@
       <c r="C40" s="43"/>
       <c r="D40" s="43"/>
       <c r="E40" s="44" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="F40" s="44"/>
       <c r="G40" s="44"/>
       <c r="H40" s="44"/>
       <c r="I40" s="44"/>
       <c r="J40" s="43" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="K40" s="43"/>
       <c r="L40" s="43"/>

</xml_diff>

<commit_message>
feat(reporting): adopt business terminology and financial governance
- adopt Business Language governance across reporting
- rename Order Sales to Sales Orders (مبيعات الطلبات)
- rename Check/Gross Revenue to Total Sales (إجمالي المبيعات)
- preserve Settlement Record as financial SSOT
- preserve Order Read as operational source
- update Dashboard, Excel and reporting presentation
- production certified
</commit_message>
<xml_diff>
--- a/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
+++ b/docs/engineering/programs/REPORTING-DESIGN-LANGUAGE-1/samples/reporting-design-language-en-2026-07.xlsx
@@ -8,7 +8,7 @@
     <sheet sheetId="2" name="Executive Summary" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Financial Summary" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Payment Analytics" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Order Sales" state="visible" r:id="rId8"/>
+    <sheet sheetId="5" name="Sales Orders" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="Sales Trends" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
@@ -60,10 +60,10 @@
     <t>Issued</t>
   </si>
   <si>
-    <t>27 Jul 2026, 14:30</t>
-  </si>
-  <si>
-    <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Payment Analytics  ·  Order Sales  ·  Sales Trends</t>
+    <t>27 Jul 2026, 15:32</t>
+  </si>
+  <si>
+    <t>Report Contents:  Executive Summary  ·  Financial Summary  ·  Payment Analytics  ·  Sales Orders  ·  Sales Trends</t>
   </si>
   <si>
     <t>Confidential — Internal Use  ·  Prepared by MineuQR</t>
@@ -72,7 +72,7 @@
     <t>Executive Summary</t>
   </si>
   <si>
-    <t>Monthly Report  ·  July 2026  ·  27 Jul 2026, 14:30</t>
+    <t>Monthly Report  ·  July 2026  ·  27 Jul 2026, 15:32</t>
   </si>
   <si>
     <t>EXECUTIVE KPIS</t>
@@ -81,10 +81,10 @@
     <t>How is the restaurant performing this period?</t>
   </si>
   <si>
-    <t>Gross Sales, Net Sales, refunds, tax, and order averages for the selected period.</t>
-  </si>
-  <si>
-    <t>Gross Sales</t>
+    <t>Total Sales, Net Sales, refunds, tax, and order averages for the selected period.</t>
+  </si>
+  <si>
+    <t>Total Sales</t>
   </si>
   <si>
     <t>Net Sales</t>
@@ -102,10 +102,10 @@
     <t>Paid check totals for this period (gross)</t>
   </si>
   <si>
-    <t>Gross Sales after published refunds</t>
-  </si>
-  <si>
-    <t>Total refunded (published Settlement Records)</t>
+    <t>Total Sales after published refunds</t>
+  </si>
+  <si>
+    <t>Total refunded (published)</t>
   </si>
   <si>
     <t>Refund Rate</t>
@@ -126,7 +126,7 @@
     <t>103</t>
   </si>
   <si>
-    <t>Refund Amount as a percent of Gross Sales</t>
+    <t>Refund Amount as a percent of Total Sales</t>
   </si>
   <si>
     <t>Tax on paid checks (frozen snapshot)</t>
@@ -153,7 +153,7 @@
     <t>Typical size of a paid check</t>
   </si>
   <si>
-    <t>Details: Financial Performance, Refund Analytics, Payment Analytics, Order Sales, and Trends follow. Operational rollups are on dedicated sheets.</t>
+    <t>Details: Financial Performance, Refund Analytics, Payment Analytics, Sales Orders, and Trends follow. Operational rollups are on dedicated sheets.</t>
   </si>
   <si>
     <t>Financial Summary</t>
@@ -165,7 +165,7 @@
     <t>MONEY COLLECTED</t>
   </si>
   <si>
-    <t>Paid guest checks for this reporting period — Gross Sales. Net Sales subtracts Refund Amount.</t>
+    <t>Paid guest checks for this reporting period — Total Sales. Net Sales subtracts Refund Amount.</t>
   </si>
   <si>
     <t>FINANCIAL PERFORMANCE</t>
@@ -189,10 +189,10 @@
     <t>Tax Collected covers the full reporting period — total tax from all paid checks in range (not a subset of sections).</t>
   </si>
   <si>
-    <t>ORDER SALES DETAIL</t>
-  </si>
-  <si>
-    <t>Order Sales</t>
+    <t>SALES ORDERS DETAIL</t>
+  </si>
+  <si>
+    <t>Sales Orders</t>
   </si>
   <si>
     <t>19,222.00 ر.س</t>
@@ -228,10 +228,10 @@
     <t>REPORTING BASIS</t>
   </si>
   <si>
-    <t>Gross Sales = sum of paid Check totals (not Order Sales).</t>
-  </si>
-  <si>
-    <t>Order Sales = completed (served) order totals from Order Read (not Gross Sales).</t>
+    <t>Total Sales = financial sales after payment across all sales channels (not Sales Orders).</t>
+  </si>
+  <si>
+    <t>Sales Orders = completed (served) order totals from operational order activity (not Total Sales).</t>
   </si>
   <si>
     <t>SAR (ر.س)</t>
@@ -240,7 +240,7 @@
     <t>Payment Analytics</t>
   </si>
   <si>
-    <t>Payment mix is from settlement tenders. Gross Sales remains from paid checks; refund tenders are listed separately and do not replace Gross Sales.</t>
+    <t>Payment mix is from payment tenders. Total Sales remains the financial sales total; refund tenders are listed separately and do not replace Total Sales.</t>
   </si>
   <si>
     <t>PAYMENT MIX</t>
@@ -312,10 +312,10 @@
     <t>Refund Tender Total</t>
   </si>
   <si>
-    <t>Monthly Report  ·  Daily Order Sales — July 2026</t>
-  </si>
-  <si>
-    <t>ORDER SALES TREND</t>
+    <t>Monthly Report  ·  Daily Sales Orders — July 2026</t>
+  </si>
+  <si>
+    <t>SALES ORDERS TREND</t>
   </si>
   <si>
     <t>Period</t>
@@ -423,7 +423,7 @@
     <t>Sales Trends</t>
   </si>
   <si>
-    <t>Monthly Report  ·  Daily Gross Sales — July 2026</t>
+    <t>Monthly Report  ·  Daily Total Sales — July 2026</t>
   </si>
   <si>
     <t>SALES TRENDS</t>

</xml_diff>